<commit_message>
Generate Excel teaching and growth candidate; retain exact baseline and sparse QA evidence
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/monGroup.xlsx
+++ b/space-battleship/config_excel/monGroup.xlsx
@@ -1013,7 +1013,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C320"/>
+  <dimension ref="A1:C390"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.888888888888889" defaultRowHeight="14.4"/>
   <cols>
     <col width="50.7777777777778" customWidth="1" style="3" min="2" max="2"/>
@@ -5826,6 +5826,1056 @@
         </is>
       </c>
     </row>
+    <row r="321">
+      <c r="A321" s="2" t="n">
+        <v>30011</v>
+      </c>
+      <c r="B321" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关1-层1-normal-laser-physical_attack</t>
+        </is>
+      </c>
+      <c r="C321" s="2" t="inlineStr">
+        <is>
+          <t>{null,41021,41022,41023,null,null,41026,41027,41028,null,null,41031,41032,41033,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" s="2" t="n">
+        <v>30012</v>
+      </c>
+      <c r="B322" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关1-层2-normal-laser-energy_attack</t>
+        </is>
+      </c>
+      <c r="C322" s="2" t="inlineStr">
+        <is>
+          <t>{null,41041,41042,41043,null,null,41046,41047,41048,null,null,41051,41052,41053,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" s="2" t="n">
+        <v>30013</v>
+      </c>
+      <c r="B323" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关1-层3-normal-laser-physical_attack</t>
+        </is>
+      </c>
+      <c r="C323" s="2" t="inlineStr">
+        <is>
+          <t>{null,41061,41062,41063,null,null,41066,41067,41068,null,null,41071,41072,41073,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" s="2" t="n">
+        <v>30014</v>
+      </c>
+      <c r="B324" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关1-层4-normal-laser-energy_attack</t>
+        </is>
+      </c>
+      <c r="C324" s="2" t="inlineStr">
+        <is>
+          <t>{null,41081,41082,41083,null,null,41086,41087,41088,null,null,41091,41092,41093,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" s="2" t="n">
+        <v>30015</v>
+      </c>
+      <c r="B325" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关1-层5-elite-laser-physical_attack</t>
+        </is>
+      </c>
+      <c r="C325" s="2" t="inlineStr">
+        <is>
+          <t>{41100,41101,41102,41103,41104,41105,41106,41107,41108,41109,41110,41111,41112,41113,41114}</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" s="2" t="n">
+        <v>30021</v>
+      </c>
+      <c r="B326" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关2-层1-normal-missile-energy_attack</t>
+        </is>
+      </c>
+      <c r="C326" s="2" t="inlineStr">
+        <is>
+          <t>{42020,42021,42022,42023,42024,42025,42026,42027,42028,42029,42030,42031,42032,42033,42034}</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" s="2" t="n">
+        <v>30022</v>
+      </c>
+      <c r="B327" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关2-层2-normal-missile-physical_attack</t>
+        </is>
+      </c>
+      <c r="C327" s="2" t="inlineStr">
+        <is>
+          <t>{42040,42041,42042,42043,42044,42045,42046,42047,42048,42049,42050,42051,42052,42053,42054}</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" s="2" t="n">
+        <v>30023</v>
+      </c>
+      <c r="B328" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关2-层3-normal-missile-energy_attack</t>
+        </is>
+      </c>
+      <c r="C328" s="2" t="inlineStr">
+        <is>
+          <t>{42060,42061,42062,42063,42064,42065,42066,42067,42068,42069,42070,42071,42072,42073,42074}</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" s="2" t="n">
+        <v>30024</v>
+      </c>
+      <c r="B329" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关2-层4-normal-missile-physical_attack</t>
+        </is>
+      </c>
+      <c r="C329" s="2" t="inlineStr">
+        <is>
+          <t>{42080,42081,42082,42083,42084,42085,42086,42087,42088,42089,42090,42091,42092,42093,42094}</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" s="2" t="n">
+        <v>30025</v>
+      </c>
+      <c r="B330" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关2-层5-elite-missile-energy_attack</t>
+        </is>
+      </c>
+      <c r="C330" s="2" t="inlineStr">
+        <is>
+          <t>{42100,42101,42102,42103,42104,42105,42106,42107,42108,42109,42110,42111,42112,42113,42114}</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" s="2" t="n">
+        <v>30031</v>
+      </c>
+      <c r="B331" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关3-层1-normal-cannon-physical_attack</t>
+        </is>
+      </c>
+      <c r="C331" s="2" t="inlineStr">
+        <is>
+          <t>{null,null,null,null,null,null,null,43027,null,null,null,null,null,null,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" s="2" t="n">
+        <v>30032</v>
+      </c>
+      <c r="B332" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关3-层2-normal-cannon-energy_attack</t>
+        </is>
+      </c>
+      <c r="C332" s="2" t="inlineStr">
+        <is>
+          <t>{null,null,null,null,null,null,null,43047,null,null,null,null,null,null,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" s="2" t="n">
+        <v>30033</v>
+      </c>
+      <c r="B333" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关3-层3-normal-cannon-physical_attack</t>
+        </is>
+      </c>
+      <c r="C333" s="2" t="inlineStr">
+        <is>
+          <t>{null,null,null,null,null,null,null,43067,null,null,null,null,null,null,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" s="2" t="n">
+        <v>30034</v>
+      </c>
+      <c r="B334" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关3-层4-normal-cannon-energy_attack</t>
+        </is>
+      </c>
+      <c r="C334" s="2" t="inlineStr">
+        <is>
+          <t>{null,null,null,null,null,null,null,43087,null,null,null,null,null,null,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" s="2" t="n">
+        <v>30035</v>
+      </c>
+      <c r="B335" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关3-层5-elite-cannon-physical_attack</t>
+        </is>
+      </c>
+      <c r="C335" s="2" t="inlineStr">
+        <is>
+          <t>{null,null,null,null,null,43105,null,43107,null,43109,null,null,null,null,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" s="2" t="n">
+        <v>30041</v>
+      </c>
+      <c r="B336" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关4-层1-normal-neutral1-energy_attack</t>
+        </is>
+      </c>
+      <c r="C336" s="2" t="inlineStr">
+        <is>
+          <t>{null,null,null,null,null,null,44026,44027,44028,null,null,null,null,null,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" s="2" t="n">
+        <v>30042</v>
+      </c>
+      <c r="B337" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关4-层2-normal-neutral1-physical_attack</t>
+        </is>
+      </c>
+      <c r="C337" s="2" t="inlineStr">
+        <is>
+          <t>{null,null,null,null,null,null,44046,44047,44048,null,null,null,null,null,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" s="2" t="n">
+        <v>30043</v>
+      </c>
+      <c r="B338" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关4-层3-normal-neutral1-energy_attack</t>
+        </is>
+      </c>
+      <c r="C338" s="2" t="inlineStr">
+        <is>
+          <t>{null,null,null,null,null,null,44066,44067,44068,null,null,null,null,null,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" s="2" t="n">
+        <v>30044</v>
+      </c>
+      <c r="B339" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关4-层4-normal-neutral1-physical_attack</t>
+        </is>
+      </c>
+      <c r="C339" s="2" t="inlineStr">
+        <is>
+          <t>{null,null,null,null,null,null,44086,44087,44088,null,null,null,null,null,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" s="2" t="n">
+        <v>30045</v>
+      </c>
+      <c r="B340" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关4-层5-elite-neutral1-energy_attack</t>
+        </is>
+      </c>
+      <c r="C340" s="2" t="inlineStr">
+        <is>
+          <t>{null,null,null,null,null,44105,null,44107,null,44109,null,44111,null,44113,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" s="2" t="n">
+        <v>30051</v>
+      </c>
+      <c r="B341" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关5-层1-normal-neutral2-physical_attack</t>
+        </is>
+      </c>
+      <c r="C341" s="2" t="inlineStr">
+        <is>
+          <t>{null,null,null,null,null,null,45026,45027,45028,null,null,null,null,null,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" s="2" t="n">
+        <v>30052</v>
+      </c>
+      <c r="B342" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关5-层2-normal-neutral2-energy_attack</t>
+        </is>
+      </c>
+      <c r="C342" s="2" t="inlineStr">
+        <is>
+          <t>{null,null,null,null,null,null,45046,45047,45048,null,null,null,null,null,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" s="2" t="n">
+        <v>30053</v>
+      </c>
+      <c r="B343" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关5-层3-normal-neutral2-physical_attack</t>
+        </is>
+      </c>
+      <c r="C343" s="2" t="inlineStr">
+        <is>
+          <t>{null,null,null,null,null,null,45066,45067,45068,null,null,null,null,null,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" s="2" t="n">
+        <v>30054</v>
+      </c>
+      <c r="B344" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关5-层4-normal-neutral2-energy_attack</t>
+        </is>
+      </c>
+      <c r="C344" s="2" t="inlineStr">
+        <is>
+          <t>{null,null,null,null,null,null,45086,45087,45088,null,null,null,null,null,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" s="2" t="n">
+        <v>30055</v>
+      </c>
+      <c r="B345" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关5-层5-elite-neutral2-physical_attack</t>
+        </is>
+      </c>
+      <c r="C345" s="2" t="inlineStr">
+        <is>
+          <t>{null,null,null,null,null,45105,null,45107,null,45109,null,45111,null,45113,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" s="2" t="n">
+        <v>30061</v>
+      </c>
+      <c r="B346" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关6-层1-normal-longLaser-energy_attack</t>
+        </is>
+      </c>
+      <c r="C346" s="2" t="inlineStr">
+        <is>
+          <t>{null,null,null,null,null,null,46026,46027,46028,null,null,null,null,null,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" s="2" t="n">
+        <v>30062</v>
+      </c>
+      <c r="B347" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关6-层2-normal-longLaser-physical_attack</t>
+        </is>
+      </c>
+      <c r="C347" s="2" t="inlineStr">
+        <is>
+          <t>{null,null,null,null,null,null,46046,46047,46048,null,null,null,null,null,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" s="2" t="n">
+        <v>30063</v>
+      </c>
+      <c r="B348" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关6-层3-normal-longLaser-energy_attack</t>
+        </is>
+      </c>
+      <c r="C348" s="2" t="inlineStr">
+        <is>
+          <t>{null,null,null,null,null,null,46066,46067,46068,null,null,null,null,null,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" s="2" t="n">
+        <v>30064</v>
+      </c>
+      <c r="B349" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关6-层4-normal-longLaser-physical_attack</t>
+        </is>
+      </c>
+      <c r="C349" s="2" t="inlineStr">
+        <is>
+          <t>{null,null,null,null,null,null,46086,46087,46088,null,null,null,null,null,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" s="2" t="n">
+        <v>30065</v>
+      </c>
+      <c r="B350" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关6-层5-normal-longLaser-energy_attack</t>
+        </is>
+      </c>
+      <c r="C350" s="2" t="inlineStr">
+        <is>
+          <t>{null,null,null,null,null,null,46106,46107,46108,null,null,null,null,null,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" s="2" t="n">
+        <v>30066</v>
+      </c>
+      <c r="B351" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关6-层6-elite-longLaser-physical_attack</t>
+        </is>
+      </c>
+      <c r="C351" s="2" t="inlineStr">
+        <is>
+          <t>{null,null,null,null,null,46125,null,46127,null,46129,null,null,null,null,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" s="2" t="n">
+        <v>30067</v>
+      </c>
+      <c r="B352" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关6-层7-elite-longLaser-energy_attack</t>
+        </is>
+      </c>
+      <c r="C352" s="2" t="inlineStr">
+        <is>
+          <t>{null,null,null,null,null,46145,null,46147,null,46149,null,null,null,null,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" s="2" t="n">
+        <v>30068</v>
+      </c>
+      <c r="B353" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关6-层8-elite-longLaser-physical_attack</t>
+        </is>
+      </c>
+      <c r="C353" s="2" t="inlineStr">
+        <is>
+          <t>{null,null,null,null,null,46165,null,46167,null,46169,null,null,null,null,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" s="2" t="n">
+        <v>30069</v>
+      </c>
+      <c r="B354" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关6-层9-boss-longLaser-energy_attack</t>
+        </is>
+      </c>
+      <c r="C354" s="2" t="inlineStr">
+        <is>
+          <t>{null,null,null,null,null,null,null,46187,null,null,null,null,null,null,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" s="2" t="n">
+        <v>30071</v>
+      </c>
+      <c r="B355" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关7-层1-normal-laser-physical_attack</t>
+        </is>
+      </c>
+      <c r="C355" s="2" t="inlineStr">
+        <is>
+          <t>{null,47021,47022,47023,null,null,47026,47027,47028,null,null,47031,47032,47033,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" s="2" t="n">
+        <v>30072</v>
+      </c>
+      <c r="B356" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关7-层2-normal-laser-energy_attack</t>
+        </is>
+      </c>
+      <c r="C356" s="2" t="inlineStr">
+        <is>
+          <t>{null,47041,47042,47043,null,null,47046,47047,47048,null,null,47051,47052,47053,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" s="2" t="n">
+        <v>30073</v>
+      </c>
+      <c r="B357" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关7-层3-normal-laser-physical_attack</t>
+        </is>
+      </c>
+      <c r="C357" s="2" t="inlineStr">
+        <is>
+          <t>{null,47061,47062,47063,null,null,47066,47067,47068,null,null,47071,47072,47073,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" s="2" t="n">
+        <v>30074</v>
+      </c>
+      <c r="B358" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关7-层4-normal-laser-energy_attack</t>
+        </is>
+      </c>
+      <c r="C358" s="2" t="inlineStr">
+        <is>
+          <t>{null,47081,47082,47083,null,null,47086,47087,47088,null,null,47091,47092,47093,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" s="2" t="n">
+        <v>30075</v>
+      </c>
+      <c r="B359" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关7-层5-normal-laser-physical_attack</t>
+        </is>
+      </c>
+      <c r="C359" s="2" t="inlineStr">
+        <is>
+          <t>{null,47101,47102,47103,null,null,47106,47107,47108,null,null,47111,47112,47113,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" s="2" t="n">
+        <v>30076</v>
+      </c>
+      <c r="B360" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关7-层6-elite-laser-energy_attack</t>
+        </is>
+      </c>
+      <c r="C360" s="2" t="inlineStr">
+        <is>
+          <t>{47120,47121,47122,47123,47124,47125,47126,47127,47128,47129,47130,47131,47132,47133,47134}</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" s="2" t="n">
+        <v>30077</v>
+      </c>
+      <c r="B361" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关7-层7-elite-laser-physical_attack</t>
+        </is>
+      </c>
+      <c r="C361" s="2" t="inlineStr">
+        <is>
+          <t>{47140,47141,47142,47143,47144,47145,47146,47147,47148,47149,47150,47151,47152,47153,47154}</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" s="2" t="n">
+        <v>30078</v>
+      </c>
+      <c r="B362" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关7-层8-elite-laser-energy_attack</t>
+        </is>
+      </c>
+      <c r="C362" s="2" t="inlineStr">
+        <is>
+          <t>{47160,47161,47162,47163,47164,47165,47166,47167,47168,47169,47170,47171,47172,47173,47174}</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" s="2" t="n">
+        <v>30079</v>
+      </c>
+      <c r="B363" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关7-层9-boss-laser-physical_attack</t>
+        </is>
+      </c>
+      <c r="C363" s="2" t="inlineStr">
+        <is>
+          <t>{null,null,null,null,null,null,null,47187,null,null,null,null,null,null,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" s="2" t="n">
+        <v>30081</v>
+      </c>
+      <c r="B364" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关8-层1-normal-missile-energy_attack</t>
+        </is>
+      </c>
+      <c r="C364" s="2" t="inlineStr">
+        <is>
+          <t>{48020,48021,48022,48023,48024,48025,48026,48027,48028,48029,48030,48031,48032,48033,48034}</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" s="2" t="n">
+        <v>30082</v>
+      </c>
+      <c r="B365" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关8-层2-normal-missile-physical_attack</t>
+        </is>
+      </c>
+      <c r="C365" s="2" t="inlineStr">
+        <is>
+          <t>{48040,48041,48042,48043,48044,48045,48046,48047,48048,48049,48050,48051,48052,48053,48054}</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" s="2" t="n">
+        <v>30083</v>
+      </c>
+      <c r="B366" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关8-层3-normal-missile-energy_attack</t>
+        </is>
+      </c>
+      <c r="C366" s="2" t="inlineStr">
+        <is>
+          <t>{48060,48061,48062,48063,48064,48065,48066,48067,48068,48069,48070,48071,48072,48073,48074}</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" s="2" t="n">
+        <v>30084</v>
+      </c>
+      <c r="B367" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关8-层4-normal-missile-physical_attack</t>
+        </is>
+      </c>
+      <c r="C367" s="2" t="inlineStr">
+        <is>
+          <t>{48080,48081,48082,48083,48084,48085,48086,48087,48088,48089,48090,48091,48092,48093,48094}</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" s="2" t="n">
+        <v>30085</v>
+      </c>
+      <c r="B368" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关8-层5-normal-missile-energy_attack</t>
+        </is>
+      </c>
+      <c r="C368" s="2" t="inlineStr">
+        <is>
+          <t>{48100,48101,48102,48103,48104,48105,48106,48107,48108,48109,48110,48111,48112,48113,48114}</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" s="2" t="n">
+        <v>30086</v>
+      </c>
+      <c r="B369" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关8-层6-elite-missile-physical_attack</t>
+        </is>
+      </c>
+      <c r="C369" s="2" t="inlineStr">
+        <is>
+          <t>{48120,48121,48122,48123,48124,48125,48126,48127,48128,48129,48130,48131,48132,48133,48134}</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" s="2" t="n">
+        <v>30087</v>
+      </c>
+      <c r="B370" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关8-层7-elite-missile-energy_attack</t>
+        </is>
+      </c>
+      <c r="C370" s="2" t="inlineStr">
+        <is>
+          <t>{48140,48141,48142,48143,48144,48145,48146,48147,48148,48149,48150,48151,48152,48153,48154}</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" s="2" t="n">
+        <v>30088</v>
+      </c>
+      <c r="B371" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关8-层8-elite-missile-physical_attack</t>
+        </is>
+      </c>
+      <c r="C371" s="2" t="inlineStr">
+        <is>
+          <t>{48160,48161,48162,48163,48164,48165,48166,48167,48168,48169,48170,48171,48172,48173,48174}</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" s="2" t="n">
+        <v>30089</v>
+      </c>
+      <c r="B372" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关8-层9-boss-missile-energy_attack</t>
+        </is>
+      </c>
+      <c r="C372" s="2" t="inlineStr">
+        <is>
+          <t>{null,null,null,null,null,null,null,48187,null,null,null,null,null,null,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" s="2" t="n">
+        <v>30091</v>
+      </c>
+      <c r="B373" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关9-层1-normal-cannon-physical_attack</t>
+        </is>
+      </c>
+      <c r="C373" s="2" t="inlineStr">
+        <is>
+          <t>{null,null,null,null,null,null,null,49027,null,null,null,null,null,null,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" s="2" t="n">
+        <v>30092</v>
+      </c>
+      <c r="B374" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关9-层2-normal-cannon-energy_attack</t>
+        </is>
+      </c>
+      <c r="C374" s="2" t="inlineStr">
+        <is>
+          <t>{null,null,null,null,null,null,null,49047,null,null,null,null,null,null,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" s="2" t="n">
+        <v>30093</v>
+      </c>
+      <c r="B375" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关9-层3-normal-cannon-physical_attack</t>
+        </is>
+      </c>
+      <c r="C375" s="2" t="inlineStr">
+        <is>
+          <t>{null,null,null,null,null,null,null,49067,null,null,null,null,null,null,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" s="2" t="n">
+        <v>30094</v>
+      </c>
+      <c r="B376" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关9-层4-normal-cannon-energy_attack</t>
+        </is>
+      </c>
+      <c r="C376" s="2" t="inlineStr">
+        <is>
+          <t>{null,null,null,null,null,null,null,49087,null,null,null,null,null,null,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" s="2" t="n">
+        <v>30095</v>
+      </c>
+      <c r="B377" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关9-层5-normal-cannon-physical_attack</t>
+        </is>
+      </c>
+      <c r="C377" s="2" t="inlineStr">
+        <is>
+          <t>{null,null,null,null,null,null,null,49107,null,null,null,null,null,null,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" s="2" t="n">
+        <v>30096</v>
+      </c>
+      <c r="B378" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关9-层6-elite-cannon-energy_attack</t>
+        </is>
+      </c>
+      <c r="C378" s="2" t="inlineStr">
+        <is>
+          <t>{null,null,null,null,null,49125,null,49127,null,49129,null,null,null,null,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" s="2" t="n">
+        <v>30097</v>
+      </c>
+      <c r="B379" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关9-层7-elite-cannon-physical_attack</t>
+        </is>
+      </c>
+      <c r="C379" s="2" t="inlineStr">
+        <is>
+          <t>{null,null,null,null,null,49145,null,49147,null,49149,null,null,null,null,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" s="2" t="n">
+        <v>30098</v>
+      </c>
+      <c r="B380" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关9-层8-elite-cannon-energy_attack</t>
+        </is>
+      </c>
+      <c r="C380" s="2" t="inlineStr">
+        <is>
+          <t>{null,null,null,null,null,49165,null,49167,null,49169,null,null,null,null,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" s="2" t="n">
+        <v>30099</v>
+      </c>
+      <c r="B381" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关9-层9-boss-cannon-physical_attack</t>
+        </is>
+      </c>
+      <c r="C381" s="2" t="inlineStr">
+        <is>
+          <t>{null,null,null,null,null,null,null,49187,null,null,null,null,null,null,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" s="2" t="n">
+        <v>30101</v>
+      </c>
+      <c r="B382" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关10-层1-normal-neutral3-energy_attack</t>
+        </is>
+      </c>
+      <c r="C382" s="2" t="inlineStr">
+        <is>
+          <t>{null,null,null,null,null,null,50026,50027,50028,null,null,null,null,null,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" s="2" t="n">
+        <v>30102</v>
+      </c>
+      <c r="B383" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关10-层2-normal-neutral3-physical_attack</t>
+        </is>
+      </c>
+      <c r="C383" s="2" t="inlineStr">
+        <is>
+          <t>{null,null,null,null,null,null,50046,50047,50048,null,null,null,null,null,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" s="2" t="n">
+        <v>30103</v>
+      </c>
+      <c r="B384" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关10-层3-normal-neutral3-energy_attack</t>
+        </is>
+      </c>
+      <c r="C384" s="2" t="inlineStr">
+        <is>
+          <t>{null,null,null,null,null,null,50066,50067,50068,null,null,null,null,null,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" s="2" t="n">
+        <v>30104</v>
+      </c>
+      <c r="B385" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关10-层4-normal-neutral3-physical_attack</t>
+        </is>
+      </c>
+      <c r="C385" s="2" t="inlineStr">
+        <is>
+          <t>{null,null,null,null,null,null,50086,50087,50088,null,null,null,null,null,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" s="2" t="n">
+        <v>30105</v>
+      </c>
+      <c r="B386" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关10-层5-normal-neutral3-energy_attack</t>
+        </is>
+      </c>
+      <c r="C386" s="2" t="inlineStr">
+        <is>
+          <t>{null,null,null,null,null,null,50106,50107,50108,null,null,null,null,null,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" s="2" t="n">
+        <v>30106</v>
+      </c>
+      <c r="B387" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关10-层6-elite-neutral3-physical_attack</t>
+        </is>
+      </c>
+      <c r="C387" s="2" t="inlineStr">
+        <is>
+          <t>{null,null,null,null,null,50125,null,50127,null,50129,null,50131,null,50133,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" s="2" t="n">
+        <v>30107</v>
+      </c>
+      <c r="B388" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关10-层7-elite-neutral3-energy_attack</t>
+        </is>
+      </c>
+      <c r="C388" s="2" t="inlineStr">
+        <is>
+          <t>{null,null,null,null,null,50145,null,50147,null,50149,null,50151,null,50153,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" s="2" t="n">
+        <v>30108</v>
+      </c>
+      <c r="B389" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关10-层8-elite-neutral3-physical_attack</t>
+        </is>
+      </c>
+      <c r="C389" s="2" t="inlineStr">
+        <is>
+          <t>{null,null,null,null,null,50165,null,50167,null,50169,null,50171,null,50173,null}</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" s="2" t="n">
+        <v>30109</v>
+      </c>
+      <c r="B390" s="2" t="inlineStr">
+        <is>
+          <t>校准early-v3-关10-层9-boss-neutral3-energy_attack</t>
+        </is>
+      </c>
+      <c r="C390" s="2" t="inlineStr">
+        <is>
+          <t>{null,null,null,null,null,null,null,50187,null,null,null,null,null,null,null}</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add draft configurable late-wave progression gates
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/monGroup.xlsx
+++ b/space-battleship/config_excel/monGroup.xlsx
@@ -1013,7 +1013,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2280"/>
+  <dimension ref="A1:F2280"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.888888888888889" defaultRowHeight="14.4"/>
   <cols>
     <col width="50.7777777777778" customWidth="1" style="3" min="2" max="2"/>
@@ -1041,6 +1041,16 @@
           <t>combatTier</t>
         </is>
       </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>atkMultiplier</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>lifeMultiplier</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1063,6 +1073,16 @@
           <t>Runtime wave tier, separate from final-wave completion</t>
         </is>
       </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>本波攻击倍率；空白为1，仅影响本波，不改变奖励或下关</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>本波生命及护盾倍率；空白为1，仅影响本波，不改变奖励或下关</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1083,6 +1103,16 @@
       <c r="D3" s="2" t="inlineStr">
         <is>
           <t>string</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>number</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>number</t>
         </is>
       </c>
     </row>
@@ -7780,6 +7810,12 @@
           <t>elite</t>
         </is>
       </c>
+      <c r="E407" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F407" s="2" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="408">
       <c r="A408" s="2" t="n">
@@ -7800,6 +7836,12 @@
           <t>boss</t>
         </is>
       </c>
+      <c r="E408" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="F408" s="2" t="n">
+        <v>1024</v>
+      </c>
     </row>
     <row r="409">
       <c r="A409" s="2" t="n">
@@ -8320,6 +8362,12 @@
           <t>elite</t>
         </is>
       </c>
+      <c r="E434" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="F434" s="2" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="435">
       <c r="A435" s="2" t="n">
@@ -8340,6 +8388,12 @@
           <t>boss</t>
         </is>
       </c>
+      <c r="E435" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="F435" s="2" t="n">
+        <v>1024</v>
+      </c>
     </row>
     <row r="436">
       <c r="A436" s="2" t="n">
@@ -8860,6 +8914,12 @@
           <t>elite</t>
         </is>
       </c>
+      <c r="E461" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="F461" s="2" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="462">
       <c r="A462" s="2" t="n">
@@ -8880,6 +8940,12 @@
           <t>boss</t>
         </is>
       </c>
+      <c r="E462" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="F462" s="2" t="n">
+        <v>256</v>
+      </c>
     </row>
     <row r="463">
       <c r="A463" s="2" t="n">
@@ -9220,6 +9286,12 @@
           <t>boss</t>
         </is>
       </c>
+      <c r="E479" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F479" s="2" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="480">
       <c r="A480" s="2" t="n">
@@ -9239,6 +9311,12 @@
         <is>
           <t>ultimate</t>
         </is>
+      </c>
+      <c r="E480" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F480" s="2" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="481">

</xml_diff>

<commit_message>
Distribute midgame combat pressure across continuous wave bands
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/monGroup.xlsx
+++ b/space-battleship/config_excel/monGroup.xlsx
@@ -1013,7 +1013,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2280"/>
+  <dimension ref="A1:F2280"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.888888888888889" defaultRowHeight="14.4"/>
   <cols>
     <col width="50.7777777777778" customWidth="1" style="3" min="2" max="2"/>
@@ -1041,6 +1041,16 @@
           <t>combatTier</t>
         </is>
       </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>atkMultiplier</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>lifeMultiplier</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1063,6 +1073,16 @@
           <t>Runtime wave tier, separate from final-wave completion</t>
         </is>
       </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>本波攻击倍率；空白为1，不改变跨关插值锚点</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>本波生命及护盾倍率；空白为1，不改变资源和跨关插值锚点</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1083,6 +1103,16 @@
       <c r="D3" s="2" t="inlineStr">
         <is>
           <t>string</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>float</t>
         </is>
       </c>
     </row>
@@ -7460,6 +7490,12 @@
           <t>normal</t>
         </is>
       </c>
+      <c r="E391" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F391" s="2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="392">
       <c r="A392" s="2" t="n">
@@ -7480,6 +7516,12 @@
           <t>normal</t>
         </is>
       </c>
+      <c r="E392" s="2" t="n">
+        <v>1.125</v>
+      </c>
+      <c r="F392" s="2" t="n">
+        <v>1.375</v>
+      </c>
     </row>
     <row r="393">
       <c r="A393" s="2" t="n">
@@ -7500,6 +7542,12 @@
           <t>normal</t>
         </is>
       </c>
+      <c r="E393" s="2" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="F393" s="2" t="n">
+        <v>1.75</v>
+      </c>
     </row>
     <row r="394">
       <c r="A394" s="2" t="n">
@@ -7520,6 +7568,12 @@
           <t>normal</t>
         </is>
       </c>
+      <c r="E394" s="2" t="n">
+        <v>1.375</v>
+      </c>
+      <c r="F394" s="2" t="n">
+        <v>2.125</v>
+      </c>
     </row>
     <row r="395">
       <c r="A395" s="2" t="n">
@@ -7540,6 +7594,12 @@
           <t>normal</t>
         </is>
       </c>
+      <c r="E395" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F395" s="2" t="n">
+        <v>2.5</v>
+      </c>
     </row>
     <row r="396">
       <c r="A396" s="2" t="n">
@@ -7560,6 +7620,12 @@
           <t>elite</t>
         </is>
       </c>
+      <c r="E396" s="2" t="n">
+        <v>1.625</v>
+      </c>
+      <c r="F396" s="2" t="n">
+        <v>2.875</v>
+      </c>
     </row>
     <row r="397">
       <c r="A397" s="2" t="n">
@@ -7580,6 +7646,12 @@
           <t>elite</t>
         </is>
       </c>
+      <c r="E397" s="2" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="F397" s="2" t="n">
+        <v>3.25</v>
+      </c>
     </row>
     <row r="398">
       <c r="A398" s="2" t="n">
@@ -7600,6 +7672,12 @@
           <t>elite</t>
         </is>
       </c>
+      <c r="E398" s="2" t="n">
+        <v>1.875</v>
+      </c>
+      <c r="F398" s="2" t="n">
+        <v>3.625</v>
+      </c>
     </row>
     <row r="399">
       <c r="A399" s="2" t="n">
@@ -7620,6 +7698,12 @@
           <t>boss</t>
         </is>
       </c>
+      <c r="E399" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F399" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="400">
       <c r="A400" s="2" t="n">
@@ -7640,6 +7724,12 @@
           <t>normal</t>
         </is>
       </c>
+      <c r="E400" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F400" s="2" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="401">
       <c r="A401" s="2" t="n">
@@ -7660,6 +7750,12 @@
           <t>normal</t>
         </is>
       </c>
+      <c r="E401" s="2" t="n">
+        <v>2.25</v>
+      </c>
+      <c r="F401" s="2" t="n">
+        <v>4.5</v>
+      </c>
     </row>
     <row r="402">
       <c r="A402" s="2" t="n">
@@ -7680,6 +7776,12 @@
           <t>normal</t>
         </is>
       </c>
+      <c r="E402" s="2" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F402" s="2" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="403">
       <c r="A403" s="2" t="n">
@@ -7700,6 +7802,12 @@
           <t>normal</t>
         </is>
       </c>
+      <c r="E403" s="2" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="F403" s="2" t="n">
+        <v>5.5</v>
+      </c>
     </row>
     <row r="404">
       <c r="A404" s="2" t="n">
@@ -7720,6 +7828,12 @@
           <t>normal</t>
         </is>
       </c>
+      <c r="E404" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F404" s="2" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="405">
       <c r="A405" s="2" t="n">
@@ -7740,6 +7854,12 @@
           <t>elite</t>
         </is>
       </c>
+      <c r="E405" s="2" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="F405" s="2" t="n">
+        <v>6.5</v>
+      </c>
     </row>
     <row r="406">
       <c r="A406" s="2" t="n">
@@ -7760,6 +7880,12 @@
           <t>elite</t>
         </is>
       </c>
+      <c r="E406" s="2" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F406" s="2" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="407">
       <c r="A407" s="2" t="n">
@@ -7780,6 +7906,12 @@
           <t>elite</t>
         </is>
       </c>
+      <c r="E407" s="2" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="F407" s="2" t="n">
+        <v>7.5</v>
+      </c>
     </row>
     <row r="408">
       <c r="A408" s="2" t="n">
@@ -7800,6 +7932,12 @@
           <t>boss</t>
         </is>
       </c>
+      <c r="E408" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="F408" s="2" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="409">
       <c r="A409" s="2" t="n">
@@ -7820,6 +7958,12 @@
           <t>normal</t>
         </is>
       </c>
+      <c r="E409" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="F409" s="2" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="410">
       <c r="A410" s="2" t="n">
@@ -7840,6 +7984,12 @@
           <t>normal</t>
         </is>
       </c>
+      <c r="E410" s="2" t="n">
+        <v>3.875</v>
+      </c>
+      <c r="F410" s="2" t="n">
+        <v>7.75</v>
+      </c>
     </row>
     <row r="411">
       <c r="A411" s="2" t="n">
@@ -7860,6 +8010,12 @@
           <t>normal</t>
         </is>
       </c>
+      <c r="E411" s="2" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="F411" s="2" t="n">
+        <v>7.5</v>
+      </c>
     </row>
     <row r="412">
       <c r="A412" s="2" t="n">
@@ -7880,6 +8036,12 @@
           <t>normal</t>
         </is>
       </c>
+      <c r="E412" s="2" t="n">
+        <v>3.625</v>
+      </c>
+      <c r="F412" s="2" t="n">
+        <v>7.25</v>
+      </c>
     </row>
     <row r="413">
       <c r="A413" s="2" t="n">
@@ -7900,6 +8062,12 @@
           <t>normal</t>
         </is>
       </c>
+      <c r="E413" s="2" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F413" s="2" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="414">
       <c r="A414" s="2" t="n">
@@ -7920,6 +8088,12 @@
           <t>elite</t>
         </is>
       </c>
+      <c r="E414" s="2" t="n">
+        <v>3.375</v>
+      </c>
+      <c r="F414" s="2" t="n">
+        <v>6.75</v>
+      </c>
     </row>
     <row r="415">
       <c r="A415" s="2" t="n">
@@ -7940,6 +8114,12 @@
           <t>elite</t>
         </is>
       </c>
+      <c r="E415" s="2" t="n">
+        <v>3.25</v>
+      </c>
+      <c r="F415" s="2" t="n">
+        <v>6.5</v>
+      </c>
     </row>
     <row r="416">
       <c r="A416" s="2" t="n">
@@ -7960,6 +8140,12 @@
           <t>elite</t>
         </is>
       </c>
+      <c r="E416" s="2" t="n">
+        <v>3.125</v>
+      </c>
+      <c r="F416" s="2" t="n">
+        <v>6.25</v>
+      </c>
     </row>
     <row r="417">
       <c r="A417" s="2" t="n">
@@ -7980,6 +8166,12 @@
           <t>boss</t>
         </is>
       </c>
+      <c r="E417" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F417" s="2" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="418">
       <c r="A418" s="2" t="n">
@@ -8000,6 +8192,12 @@
           <t>normal</t>
         </is>
       </c>
+      <c r="E418" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F418" s="2" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="419">
       <c r="A419" s="2" t="n">
@@ -8020,6 +8218,12 @@
           <t>normal</t>
         </is>
       </c>
+      <c r="E419" s="2" t="n">
+        <v>3.375</v>
+      </c>
+      <c r="F419" s="2" t="n">
+        <v>6.75</v>
+      </c>
     </row>
     <row r="420">
       <c r="A420" s="2" t="n">
@@ -8040,6 +8244,12 @@
           <t>normal</t>
         </is>
       </c>
+      <c r="E420" s="2" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="F420" s="2" t="n">
+        <v>7.5</v>
+      </c>
     </row>
     <row r="421">
       <c r="A421" s="2" t="n">
@@ -8060,6 +8270,12 @@
           <t>normal</t>
         </is>
       </c>
+      <c r="E421" s="2" t="n">
+        <v>4.125</v>
+      </c>
+      <c r="F421" s="2" t="n">
+        <v>8.25</v>
+      </c>
     </row>
     <row r="422">
       <c r="A422" s="2" t="n">
@@ -8080,6 +8296,12 @@
           <t>normal</t>
         </is>
       </c>
+      <c r="E422" s="2" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="F422" s="2" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="423">
       <c r="A423" s="2" t="n">
@@ -8100,6 +8322,12 @@
           <t>elite</t>
         </is>
       </c>
+      <c r="E423" s="2" t="n">
+        <v>4.875</v>
+      </c>
+      <c r="F423" s="2" t="n">
+        <v>9.75</v>
+      </c>
     </row>
     <row r="424">
       <c r="A424" s="2" t="n">
@@ -8120,6 +8348,12 @@
           <t>elite</t>
         </is>
       </c>
+      <c r="E424" s="2" t="n">
+        <v>5.25</v>
+      </c>
+      <c r="F424" s="2" t="n">
+        <v>10.5</v>
+      </c>
     </row>
     <row r="425">
       <c r="A425" s="2" t="n">
@@ -8140,6 +8374,12 @@
           <t>elite</t>
         </is>
       </c>
+      <c r="E425" s="2" t="n">
+        <v>5.625</v>
+      </c>
+      <c r="F425" s="2" t="n">
+        <v>11.25</v>
+      </c>
     </row>
     <row r="426">
       <c r="A426" s="2" t="n">
@@ -8160,6 +8400,12 @@
           <t>boss</t>
         </is>
       </c>
+      <c r="E426" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F426" s="2" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="427">
       <c r="A427" s="2" t="n">
@@ -8180,6 +8426,12 @@
           <t>normal</t>
         </is>
       </c>
+      <c r="E427" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F427" s="2" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="428">
       <c r="A428" s="2" t="n">
@@ -8200,6 +8452,12 @@
           <t>normal</t>
         </is>
       </c>
+      <c r="E428" s="2" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="F428" s="2" t="n">
+        <v>12.5</v>
+      </c>
     </row>
     <row r="429">
       <c r="A429" s="2" t="n">
@@ -8220,6 +8478,12 @@
           <t>normal</t>
         </is>
       </c>
+      <c r="E429" s="2" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="F429" s="2" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="430">
       <c r="A430" s="2" t="n">
@@ -8240,6 +8504,12 @@
           <t>normal</t>
         </is>
       </c>
+      <c r="E430" s="2" t="n">
+        <v>6.75</v>
+      </c>
+      <c r="F430" s="2" t="n">
+        <v>13.5</v>
+      </c>
     </row>
     <row r="431">
       <c r="A431" s="2" t="n">
@@ -8260,6 +8530,12 @@
           <t>normal</t>
         </is>
       </c>
+      <c r="E431" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="F431" s="2" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="432">
       <c r="A432" s="2" t="n">
@@ -8280,6 +8556,12 @@
           <t>elite</t>
         </is>
       </c>
+      <c r="E432" s="2" t="n">
+        <v>7.25</v>
+      </c>
+      <c r="F432" s="2" t="n">
+        <v>14.5</v>
+      </c>
     </row>
     <row r="433">
       <c r="A433" s="2" t="n">
@@ -8300,6 +8582,12 @@
           <t>elite</t>
         </is>
       </c>
+      <c r="E433" s="2" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="F433" s="2" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="434">
       <c r="A434" s="2" t="n">
@@ -8320,6 +8608,12 @@
           <t>elite</t>
         </is>
       </c>
+      <c r="E434" s="2" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="F434" s="2" t="n">
+        <v>15.5</v>
+      </c>
     </row>
     <row r="435">
       <c r="A435" s="2" t="n">
@@ -8340,6 +8634,12 @@
           <t>boss</t>
         </is>
       </c>
+      <c r="E435" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="F435" s="2" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="436">
       <c r="A436" s="2" t="n">
@@ -8360,6 +8660,12 @@
           <t>normal</t>
         </is>
       </c>
+      <c r="E436" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="F436" s="2" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="437">
       <c r="A437" s="2" t="n">
@@ -8380,6 +8686,12 @@
           <t>normal</t>
         </is>
       </c>
+      <c r="E437" s="2" t="n">
+        <v>7.75</v>
+      </c>
+      <c r="F437" s="2" t="n">
+        <v>15.5</v>
+      </c>
     </row>
     <row r="438">
       <c r="A438" s="2" t="n">
@@ -8400,6 +8712,12 @@
           <t>normal</t>
         </is>
       </c>
+      <c r="E438" s="2" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="F438" s="2" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="439">
       <c r="A439" s="2" t="n">
@@ -8420,6 +8738,12 @@
           <t>normal</t>
         </is>
       </c>
+      <c r="E439" s="2" t="n">
+        <v>7.25</v>
+      </c>
+      <c r="F439" s="2" t="n">
+        <v>14.5</v>
+      </c>
     </row>
     <row r="440">
       <c r="A440" s="2" t="n">
@@ -8440,6 +8764,12 @@
           <t>normal</t>
         </is>
       </c>
+      <c r="E440" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="F440" s="2" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="441">
       <c r="A441" s="2" t="n">
@@ -8460,6 +8790,12 @@
           <t>elite</t>
         </is>
       </c>
+      <c r="E441" s="2" t="n">
+        <v>6.75</v>
+      </c>
+      <c r="F441" s="2" t="n">
+        <v>13.5</v>
+      </c>
     </row>
     <row r="442">
       <c r="A442" s="2" t="n">
@@ -8480,6 +8816,12 @@
           <t>elite</t>
         </is>
       </c>
+      <c r="E442" s="2" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="F442" s="2" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="443">
       <c r="A443" s="2" t="n">
@@ -8500,6 +8842,12 @@
           <t>elite</t>
         </is>
       </c>
+      <c r="E443" s="2" t="n">
+        <v>6.25</v>
+      </c>
+      <c r="F443" s="2" t="n">
+        <v>12.5</v>
+      </c>
     </row>
     <row r="444">
       <c r="A444" s="2" t="n">
@@ -8520,6 +8868,12 @@
           <t>boss</t>
         </is>
       </c>
+      <c r="E444" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F444" s="2" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="445">
       <c r="A445" s="2" t="n">
@@ -8540,6 +8894,12 @@
           <t>normal</t>
         </is>
       </c>
+      <c r="E445" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="F445" s="2" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="446">
       <c r="A446" s="2" t="n">
@@ -8560,6 +8920,12 @@
           <t>normal</t>
         </is>
       </c>
+      <c r="E446" s="2" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="F446" s="2" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="447">
       <c r="A447" s="2" t="n">
@@ -8580,6 +8946,12 @@
           <t>normal</t>
         </is>
       </c>
+      <c r="E447" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="F447" s="2" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="448">
       <c r="A448" s="2" t="n">
@@ -8600,6 +8972,12 @@
           <t>normal</t>
         </is>
       </c>
+      <c r="E448" s="2" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="F448" s="2" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="449">
       <c r="A449" s="2" t="n">
@@ -8620,6 +8998,12 @@
           <t>normal</t>
         </is>
       </c>
+      <c r="E449" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="F449" s="2" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="450">
       <c r="A450" s="2" t="n">
@@ -8640,6 +9024,12 @@
           <t>elite</t>
         </is>
       </c>
+      <c r="E450" s="2" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="F450" s="2" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="451">
       <c r="A451" s="2" t="n">
@@ -8660,6 +9050,12 @@
           <t>elite</t>
         </is>
       </c>
+      <c r="E451" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F451" s="2" t="n">
+        <v>18</v>
+      </c>
     </row>
     <row r="452">
       <c r="A452" s="2" t="n">
@@ -8680,6 +9076,12 @@
           <t>elite</t>
         </is>
       </c>
+      <c r="E452" s="2" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="F452" s="2" t="n">
+        <v>19</v>
+      </c>
     </row>
     <row r="453">
       <c r="A453" s="2" t="n">
@@ -8700,6 +9102,12 @@
           <t>boss</t>
         </is>
       </c>
+      <c r="E453" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="F453" s="2" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="454">
       <c r="A454" s="2" t="n">
@@ -8720,6 +9128,12 @@
           <t>normal</t>
         </is>
       </c>
+      <c r="E454" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="F454" s="2" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="455">
       <c r="A455" s="2" t="n">
@@ -8740,6 +9154,12 @@
           <t>normal</t>
         </is>
       </c>
+      <c r="E455" s="2" t="n">
+        <v>10.25</v>
+      </c>
+      <c r="F455" s="2" t="n">
+        <v>20.5</v>
+      </c>
     </row>
     <row r="456">
       <c r="A456" s="2" t="n">
@@ -8760,6 +9180,12 @@
           <t>normal</t>
         </is>
       </c>
+      <c r="E456" s="2" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="F456" s="2" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="457">
       <c r="A457" s="2" t="n">
@@ -8780,6 +9206,12 @@
           <t>normal</t>
         </is>
       </c>
+      <c r="E457" s="2" t="n">
+        <v>10.75</v>
+      </c>
+      <c r="F457" s="2" t="n">
+        <v>21.5</v>
+      </c>
     </row>
     <row r="458">
       <c r="A458" s="2" t="n">
@@ -8800,6 +9232,12 @@
           <t>normal</t>
         </is>
       </c>
+      <c r="E458" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="F458" s="2" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="459">
       <c r="A459" s="2" t="n">
@@ -8820,6 +9258,12 @@
           <t>elite</t>
         </is>
       </c>
+      <c r="E459" s="2" t="n">
+        <v>11.25</v>
+      </c>
+      <c r="F459" s="2" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="460">
       <c r="A460" s="2" t="n">
@@ -8840,6 +9284,12 @@
           <t>elite</t>
         </is>
       </c>
+      <c r="E460" s="2" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="F460" s="2" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="461">
       <c r="A461" s="2" t="n">
@@ -8860,6 +9310,12 @@
           <t>elite</t>
         </is>
       </c>
+      <c r="E461" s="2" t="n">
+        <v>11.75</v>
+      </c>
+      <c r="F461" s="2" t="n">
+        <v>23.5</v>
+      </c>
     </row>
     <row r="462">
       <c r="A462" s="2" t="n">
@@ -8880,6 +9336,12 @@
           <t>boss</t>
         </is>
       </c>
+      <c r="E462" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="F462" s="2" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="463">
       <c r="A463" s="2" t="n">
@@ -8900,6 +9362,12 @@
           <t>normal</t>
         </is>
       </c>
+      <c r="E463" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="F463" s="2" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="464">
       <c r="A464" s="2" t="n">
@@ -8920,6 +9388,12 @@
           <t>normal</t>
         </is>
       </c>
+      <c r="E464" s="2" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="F464" s="2" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="465">
       <c r="A465" s="2" t="n">
@@ -8940,6 +9414,12 @@
           <t>normal</t>
         </is>
       </c>
+      <c r="E465" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="F465" s="2" t="n">
+        <v>26</v>
+      </c>
     </row>
     <row r="466">
       <c r="A466" s="2" t="n">
@@ -8960,6 +9440,12 @@
           <t>normal</t>
         </is>
       </c>
+      <c r="E466" s="2" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="F466" s="2" t="n">
+        <v>27</v>
+      </c>
     </row>
     <row r="467">
       <c r="A467" s="2" t="n">
@@ -8980,6 +9466,12 @@
           <t>normal</t>
         </is>
       </c>
+      <c r="E467" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="F467" s="2" t="n">
+        <v>28</v>
+      </c>
     </row>
     <row r="468">
       <c r="A468" s="2" t="n">
@@ -9000,6 +9492,12 @@
           <t>elite</t>
         </is>
       </c>
+      <c r="E468" s="2" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="F468" s="2" t="n">
+        <v>29</v>
+      </c>
     </row>
     <row r="469">
       <c r="A469" s="2" t="n">
@@ -9020,6 +9518,12 @@
           <t>elite</t>
         </is>
       </c>
+      <c r="E469" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="F469" s="2" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="470">
       <c r="A470" s="2" t="n">
@@ -9040,6 +9544,12 @@
           <t>elite</t>
         </is>
       </c>
+      <c r="E470" s="2" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="F470" s="2" t="n">
+        <v>31</v>
+      </c>
     </row>
     <row r="471">
       <c r="A471" s="2" t="n">
@@ -9060,6 +9570,12 @@
           <t>boss</t>
         </is>
       </c>
+      <c r="E471" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="F471" s="2" t="n">
+        <v>32</v>
+      </c>
     </row>
     <row r="472">
       <c r="A472" s="2" t="n">
@@ -9080,6 +9596,12 @@
           <t>elite</t>
         </is>
       </c>
+      <c r="E472" t="n">
+        <v>16</v>
+      </c>
+      <c r="F472" t="n">
+        <v>32</v>
+      </c>
     </row>
     <row r="473">
       <c r="A473" s="2" t="n">
@@ -9100,6 +9622,12 @@
           <t>elite</t>
         </is>
       </c>
+      <c r="E473" t="n">
+        <v>3.391110215352182</v>
+      </c>
+      <c r="F473" t="n">
+        <v>5.605023522991008</v>
+      </c>
     </row>
     <row r="474">
       <c r="A474" s="2" t="n">
@@ -9120,6 +9648,12 @@
           <t>elite</t>
         </is>
       </c>
+      <c r="E474" t="n">
+        <v>2.127461929935275</v>
+      </c>
+      <c r="F474" t="n">
+        <v>3.156649161856778</v>
+      </c>
     </row>
     <row r="475">
       <c r="A475" s="2" t="n">
@@ -9140,6 +9674,12 @@
           <t>elite</t>
         </is>
       </c>
+      <c r="E475" t="n">
+        <v>1.648015526593405</v>
+      </c>
+      <c r="F475" t="n">
+        <v>2.236366506256873</v>
+      </c>
     </row>
     <row r="476">
       <c r="A476" s="2" t="n">
@@ -9160,6 +9700,12 @@
           <t>elite</t>
         </is>
       </c>
+      <c r="E476" t="n">
+        <v>1.395646246917129</v>
+      </c>
+      <c r="F476" t="n">
+        <v>1.753846098162387</v>
+      </c>
     </row>
     <row r="477">
       <c r="A477" s="2" t="n">
@@ -9180,6 +9726,12 @@
           <t>boss</t>
         </is>
       </c>
+      <c r="E477" t="n">
+        <v>1.239919029849584</v>
+      </c>
+      <c r="F477" t="n">
+        <v>1.456750492140449</v>
+      </c>
     </row>
     <row r="478">
       <c r="A478" s="2" t="n">
@@ -9200,6 +9752,12 @@
           <t>boss</t>
         </is>
       </c>
+      <c r="E478" t="n">
+        <v>1.134242642197337</v>
+      </c>
+      <c r="F478" t="n">
+        <v>1.255422883125648</v>
+      </c>
     </row>
     <row r="479">
       <c r="A479" s="2" t="n">
@@ -9220,6 +9778,12 @@
           <t>boss</t>
         </is>
       </c>
+      <c r="E479" t="n">
+        <v>1.057828295156404</v>
+      </c>
+      <c r="F479" t="n">
+        <v>1.109984786431736</v>
+      </c>
     </row>
     <row r="480">
       <c r="A480" s="2" t="n">
@@ -9239,6 +9803,12 @@
         <is>
           <t>ultimate</t>
         </is>
+      </c>
+      <c r="E480" t="n">
+        <v>1</v>
+      </c>
+      <c r="F480" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="481">

</xml_diff>

<commit_message>
Shape midgame accumulation and release with smooth absolute wave growth
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/monGroup.xlsx
+++ b/space-battleship/config_excel/monGroup.xlsx
@@ -7517,10 +7517,10 @@
         </is>
       </c>
       <c r="E392" s="2" t="n">
-        <v>1.125</v>
+        <v>0.5324901793116744</v>
       </c>
       <c r="F392" s="2" t="n">
-        <v>1.375</v>
+        <v>0.4866262989023714</v>
       </c>
     </row>
     <row r="393">
@@ -7543,10 +7543,10 @@
         </is>
       </c>
       <c r="E393" s="2" t="n">
-        <v>1.25</v>
+        <v>0.5685766072036965</v>
       </c>
       <c r="F393" s="2" t="n">
-        <v>1.75</v>
+        <v>0.5893697628939644</v>
       </c>
     </row>
     <row r="394">
@@ -7569,10 +7569,10 @@
         </is>
       </c>
       <c r="E394" s="2" t="n">
-        <v>1.375</v>
+        <v>0.7330769879429946</v>
       </c>
       <c r="F394" s="2" t="n">
-        <v>2.125</v>
+        <v>0.8814634834042079</v>
       </c>
     </row>
     <row r="395">
@@ -7595,10 +7595,10 @@
         </is>
       </c>
       <c r="E395" s="2" t="n">
-        <v>1.5</v>
+        <v>1.033966733686373</v>
       </c>
       <c r="F395" s="2" t="n">
-        <v>2.5</v>
+        <v>1.452249478385389</v>
       </c>
     </row>
     <row r="396">
@@ -7621,10 +7621,10 @@
         </is>
       </c>
       <c r="E396" s="2" t="n">
-        <v>1.625</v>
+        <v>1.53731829326964</v>
       </c>
       <c r="F396" s="2" t="n">
-        <v>2.875</v>
+        <v>2.529921892018751</v>
       </c>
     </row>
     <row r="397">
@@ -7647,10 +7647,10 @@
         </is>
       </c>
       <c r="E397" s="2" t="n">
-        <v>1.75</v>
+        <v>2.366494402833543</v>
       </c>
       <c r="F397" s="2" t="n">
-        <v>3.25</v>
+        <v>4.570446168006661</v>
       </c>
     </row>
     <row r="398">
@@ -7673,10 +7673,10 @@
         </is>
       </c>
       <c r="E398" s="2" t="n">
-        <v>1.875</v>
+        <v>3.733702808621944</v>
       </c>
       <c r="F398" s="2" t="n">
-        <v>3.625</v>
+        <v>8.470668656818301</v>
       </c>
     </row>
     <row r="399">
@@ -7699,10 +7699,10 @@
         </is>
       </c>
       <c r="E399" s="2" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F399" s="2" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
     </row>
     <row r="400">
@@ -7725,10 +7725,10 @@
         </is>
       </c>
       <c r="E400" s="2" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="F400" s="2" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
     </row>
     <row r="401">
@@ -7751,10 +7751,10 @@
         </is>
       </c>
       <c r="E401" s="2" t="n">
-        <v>2.25</v>
+        <v>3.478938441688168</v>
       </c>
       <c r="F401" s="2" t="n">
-        <v>4.5</v>
+        <v>8.826387079624727</v>
       </c>
     </row>
     <row r="402">
@@ -7777,10 +7777,10 @@
         </is>
       </c>
       <c r="E402" s="2" t="n">
-        <v>2.5</v>
+        <v>3.259663030130004</v>
       </c>
       <c r="F402" s="2" t="n">
-        <v>5</v>
+        <v>9.427003419616131</v>
       </c>
     </row>
     <row r="403">
@@ -7803,10 +7803,10 @@
         </is>
       </c>
       <c r="E403" s="2" t="n">
-        <v>2.75</v>
+        <v>3.575145032011695</v>
       </c>
       <c r="F403" s="2" t="n">
-        <v>5.5</v>
+        <v>12.1047694889808</v>
       </c>
     </row>
     <row r="404">
@@ -7829,10 +7829,10 @@
         </is>
       </c>
       <c r="E404" s="2" t="n">
-        <v>3</v>
+        <v>4.245160408187956</v>
       </c>
       <c r="F404" s="2" t="n">
-        <v>6</v>
+        <v>16.97957173522325</v>
       </c>
     </row>
     <row r="405">
@@ -7855,10 +7855,10 @@
         </is>
       </c>
       <c r="E405" s="2" t="n">
-        <v>3.25</v>
+        <v>5.28854526470762</v>
       </c>
       <c r="F405" s="2" t="n">
-        <v>6.5</v>
+        <v>25.09140256607924</v>
       </c>
     </row>
     <row r="406">
@@ -7881,10 +7881,10 @@
         </is>
       </c>
       <c r="E406" s="2" t="n">
-        <v>3.5</v>
+        <v>6.803814155506166</v>
       </c>
       <c r="F406" s="2" t="n">
-        <v>7</v>
+        <v>38.37624408240584</v>
       </c>
     </row>
     <row r="407">
@@ -7907,10 +7907,10 @@
         </is>
       </c>
       <c r="E407" s="2" t="n">
-        <v>3.75</v>
+        <v>8.957652652226891</v>
       </c>
       <c r="F407" s="2" t="n">
-        <v>7.5</v>
+        <v>60.14590712943249</v>
       </c>
     </row>
     <row r="408">
@@ -7933,10 +7933,10 @@
         </is>
       </c>
       <c r="E408" s="2" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="F408" s="2" t="n">
-        <v>8</v>
+        <v>96</v>
       </c>
     </row>
     <row r="409">
@@ -7959,10 +7959,10 @@
         </is>
       </c>
       <c r="E409" s="2" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="F409" s="2" t="n">
-        <v>8</v>
+        <v>96</v>
       </c>
     </row>
     <row r="410">
@@ -7985,10 +7985,10 @@
         </is>
       </c>
       <c r="E410" s="2" t="n">
-        <v>3.875</v>
+        <v>6.065080688320603</v>
       </c>
       <c r="F410" s="2" t="n">
-        <v>7.75</v>
+        <v>35.59654231167815</v>
       </c>
     </row>
     <row r="411">
@@ -8011,10 +8011,10 @@
         </is>
       </c>
       <c r="E411" s="2" t="n">
-        <v>3.75</v>
+        <v>4.953616586983959</v>
       </c>
       <c r="F411" s="2" t="n">
-        <v>7.5</v>
+        <v>25.55477753400599</v>
       </c>
     </row>
     <row r="412">
@@ -8037,10 +8037,10 @@
         </is>
       </c>
       <c r="E412" s="2" t="n">
-        <v>3.625</v>
+        <v>4.735907262666692</v>
       </c>
       <c r="F412" s="2" t="n">
-        <v>7.25</v>
+        <v>22.05609168050223</v>
       </c>
     </row>
     <row r="413">
@@ -8063,10 +8063,10 @@
         </is>
       </c>
       <c r="E413" s="2" t="n">
-        <v>3.5</v>
+        <v>4.901889008840915</v>
       </c>
       <c r="F413" s="2" t="n">
-        <v>7</v>
+        <v>20.79564340114026</v>
       </c>
     </row>
     <row r="414">
@@ -8089,10 +8089,10 @@
         </is>
       </c>
       <c r="E414" s="2" t="n">
-        <v>3.375</v>
+        <v>5.323109957194588</v>
       </c>
       <c r="F414" s="2" t="n">
-        <v>6.75</v>
+        <v>20.65590191253872</v>
       </c>
     </row>
     <row r="415">
@@ -8115,10 +8115,10 @@
         </is>
       </c>
       <c r="E415" s="2" t="n">
-        <v>3.25</v>
+        <v>5.969548666013317</v>
       </c>
       <c r="F415" s="2" t="n">
-        <v>6.5</v>
+        <v>21.2351477360025</v>
       </c>
     </row>
     <row r="416">
@@ -8141,10 +8141,10 @@
         </is>
       </c>
       <c r="E416" s="2" t="n">
-        <v>3.125</v>
+        <v>6.850828815107059</v>
       </c>
       <c r="F416" s="2" t="n">
-        <v>6.25</v>
+        <v>22.3703352813583</v>
       </c>
     </row>
     <row r="417">
@@ -8167,10 +8167,10 @@
         </is>
       </c>
       <c r="E417" s="2" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F417" s="2" t="n">
-        <v>6</v>
+        <v>24</v>
       </c>
     </row>
     <row r="418">
@@ -8193,10 +8193,10 @@
         </is>
       </c>
       <c r="E418" s="2" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F418" s="2" t="n">
-        <v>6</v>
+        <v>24</v>
       </c>
     </row>
     <row r="419">
@@ -8219,10 +8219,10 @@
         </is>
       </c>
       <c r="E419" s="2" t="n">
-        <v>3.375</v>
+        <v>5.058412362836491</v>
       </c>
       <c r="F419" s="2" t="n">
-        <v>6.75</v>
+        <v>14.2268552436008</v>
       </c>
     </row>
     <row r="420">
@@ -8245,10 +8245,10 @@
         </is>
       </c>
       <c r="E420" s="2" t="n">
-        <v>3.75</v>
+        <v>5.168552623922572</v>
       </c>
       <c r="F420" s="2" t="n">
-        <v>7.5</v>
+        <v>16.32804888590069</v>
       </c>
     </row>
     <row r="421">
@@ -8271,10 +8271,10 @@
         </is>
       </c>
       <c r="E421" s="2" t="n">
-        <v>4.125</v>
+        <v>6.181852654835754</v>
       </c>
       <c r="F421" s="2" t="n">
-        <v>8.25</v>
+        <v>22.52951460951273</v>
       </c>
     </row>
     <row r="422">
@@ -8297,10 +8297,10 @@
         </is>
       </c>
       <c r="E422" s="2" t="n">
-        <v>4.5</v>
+        <v>8.004751231611612</v>
       </c>
       <c r="F422" s="2" t="n">
-        <v>9</v>
+        <v>33.9591434704465</v>
       </c>
     </row>
     <row r="423">
@@ -8323,10 +8323,10 @@
         </is>
       </c>
       <c r="E423" s="2" t="n">
-        <v>4.875</v>
+        <v>10.87473567718933</v>
       </c>
       <c r="F423" s="2" t="n">
-        <v>9.75</v>
+        <v>53.92493348957762</v>
       </c>
     </row>
     <row r="424">
@@ -8349,10 +8349,10 @@
         </is>
       </c>
       <c r="E424" s="2" t="n">
-        <v>5.25</v>
+        <v>15.25680782244697</v>
       </c>
       <c r="F424" s="2" t="n">
-        <v>10.5</v>
+        <v>88.62613940585517</v>
       </c>
     </row>
     <row r="425">
@@ -8375,10 +8375,10 @@
         </is>
       </c>
       <c r="E425" s="2" t="n">
-        <v>5.625</v>
+        <v>21.90454319924028</v>
       </c>
       <c r="F425" s="2" t="n">
-        <v>11.25</v>
+        <v>149.2588624793426</v>
       </c>
     </row>
     <row r="426">
@@ -8401,10 +8401,10 @@
         </is>
       </c>
       <c r="E426" s="2" t="n">
-        <v>6</v>
+        <v>32</v>
       </c>
       <c r="F426" s="2" t="n">
-        <v>12</v>
+        <v>256</v>
       </c>
     </row>
     <row r="427">
@@ -8427,10 +8427,10 @@
         </is>
       </c>
       <c r="E427" s="2" t="n">
-        <v>6</v>
+        <v>32</v>
       </c>
       <c r="F427" s="2" t="n">
-        <v>12</v>
+        <v>256</v>
       </c>
     </row>
     <row r="428">
@@ -8453,10 +8453,10 @@
         </is>
       </c>
       <c r="E428" s="2" t="n">
-        <v>6.25</v>
+        <v>19.79125080161339</v>
       </c>
       <c r="F428" s="2" t="n">
-        <v>12.5</v>
+        <v>159.4681191773176</v>
       </c>
     </row>
     <row r="429">
@@ -8479,10 +8479,10 @@
         </is>
       </c>
       <c r="E429" s="2" t="n">
-        <v>6.5</v>
+        <v>18.62815390545874</v>
       </c>
       <c r="F429" s="2" t="n">
-        <v>13</v>
+        <v>157.3939522338765</v>
       </c>
     </row>
     <row r="430">
@@ -8505,10 +8505,10 @@
         </is>
       </c>
       <c r="E430" s="2" t="n">
-        <v>6.75</v>
+        <v>20.30258310625938</v>
       </c>
       <c r="F430" s="2" t="n">
-        <v>13.5</v>
+        <v>181.2205985098322</v>
       </c>
     </row>
     <row r="431">
@@ -8531,10 +8531,10 @@
         </is>
       </c>
       <c r="E431" s="2" t="n">
-        <v>7</v>
+        <v>23.86341635273138</v>
       </c>
       <c r="F431" s="2" t="n">
-        <v>14</v>
+        <v>225.6220294016744</v>
       </c>
     </row>
     <row r="432">
@@ -8557,10 +8557,10 @@
         </is>
       </c>
       <c r="E432" s="2" t="n">
-        <v>7.25</v>
+        <v>29.37418126443648</v>
       </c>
       <c r="F432" s="2" t="n">
-        <v>14.5</v>
+        <v>294.5450257663789</v>
       </c>
     </row>
     <row r="433">
@@ -8583,10 +8583,10 @@
         </is>
       </c>
       <c r="E433" s="2" t="n">
-        <v>7.5</v>
+        <v>37.30257282907881</v>
       </c>
       <c r="F433" s="2" t="n">
-        <v>15</v>
+        <v>396.9735342831585</v>
       </c>
     </row>
     <row r="434">
@@ -8609,10 +8609,10 @@
         </is>
       </c>
       <c r="E434" s="2" t="n">
-        <v>7.75</v>
+        <v>48.44769535919042</v>
       </c>
       <c r="F434" s="2" t="n">
-        <v>15.5</v>
+        <v>547.4133448621855</v>
       </c>
     </row>
     <row r="435">
@@ -8635,10 +8635,10 @@
         </is>
       </c>
       <c r="E435" s="2" t="n">
-        <v>8</v>
+        <v>64</v>
       </c>
       <c r="F435" s="2" t="n">
-        <v>16</v>
+        <v>768</v>
       </c>
     </row>
     <row r="436">
@@ -8661,10 +8661,10 @@
         </is>
       </c>
       <c r="E436" s="2" t="n">
-        <v>8</v>
+        <v>64</v>
       </c>
       <c r="F436" s="2" t="n">
-        <v>16</v>
+        <v>768</v>
       </c>
     </row>
     <row r="437">
@@ -8687,10 +8687,10 @@
         </is>
       </c>
       <c r="E437" s="2" t="n">
-        <v>7.75</v>
+        <v>32.10911954299499</v>
       </c>
       <c r="F437" s="2" t="n">
-        <v>15.5</v>
+        <v>333.3389504130951</v>
       </c>
     </row>
     <row r="438">
@@ -8713,10 +8713,10 @@
         </is>
       </c>
       <c r="E438" s="2" t="n">
-        <v>7.5</v>
+        <v>24.51602926425373</v>
       </c>
       <c r="F438" s="2" t="n">
-        <v>15</v>
+        <v>229.2404061781276</v>
       </c>
     </row>
     <row r="439">
@@ -8739,10 +8739,10 @@
         </is>
       </c>
       <c r="E439" s="2" t="n">
-        <v>7.25</v>
+        <v>21.67488338600252</v>
       </c>
       <c r="F439" s="2" t="n">
-        <v>14.5</v>
+        <v>183.9084252597998</v>
       </c>
     </row>
     <row r="440">
@@ -8765,10 +8765,10 @@
         </is>
       </c>
       <c r="E440" s="2" t="n">
-        <v>7</v>
+        <v>20.66632478255037</v>
       </c>
       <c r="F440" s="2" t="n">
-        <v>14</v>
+        <v>159.5388669749946</v>
       </c>
     </row>
     <row r="441">
@@ -8791,10 +8791,10 @@
         </is>
       </c>
       <c r="E441" s="2" t="n">
-        <v>6.75</v>
+        <v>20.63581193306492</v>
       </c>
       <c r="F441" s="2" t="n">
-        <v>13.5</v>
+        <v>145.1201210115109</v>
       </c>
     </row>
     <row r="442">
@@ -8817,10 +8817,10 @@
         </is>
       </c>
       <c r="E442" s="2" t="n">
-        <v>6.5</v>
+        <v>21.25786950161368</v>
       </c>
       <c r="F442" s="2" t="n">
-        <v>13</v>
+        <v>136.2788404861893</v>
       </c>
     </row>
     <row r="443">
@@ -8843,10 +8843,10 @@
         </is>
       </c>
       <c r="E443" s="2" t="n">
-        <v>6.25</v>
+        <v>22.3964523925201</v>
       </c>
       <c r="F443" s="2" t="n">
-        <v>12.5</v>
+        <v>130.9402582709814</v>
       </c>
     </row>
     <row r="444">
@@ -8869,10 +8869,10 @@
         </is>
       </c>
       <c r="E444" s="2" t="n">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="F444" s="2" t="n">
-        <v>12</v>
+        <v>128</v>
       </c>
     </row>
     <row r="445">
@@ -8895,10 +8895,10 @@
         </is>
       </c>
       <c r="E445" s="2" t="n">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="F445" s="2" t="n">
-        <v>12</v>
+        <v>128</v>
       </c>
     </row>
     <row r="446">
@@ -8921,10 +8921,10 @@
         </is>
       </c>
       <c r="E446" s="2" t="n">
-        <v>6.5</v>
+        <v>16.77956111598912</v>
       </c>
       <c r="F446" s="2" t="n">
-        <v>13</v>
+        <v>94.82031097088398</v>
       </c>
     </row>
     <row r="447">
@@ -8947,10 +8947,10 @@
         </is>
       </c>
       <c r="E447" s="2" t="n">
-        <v>7</v>
+        <v>17.8534957240967</v>
       </c>
       <c r="F447" s="2" t="n">
-        <v>14</v>
+        <v>111.2943309423256</v>
       </c>
     </row>
     <row r="448">
@@ -8973,10 +8973,10 @@
         </is>
       </c>
       <c r="E448" s="2" t="n">
-        <v>7.5</v>
+        <v>21.9963608110104</v>
       </c>
       <c r="F448" s="2" t="n">
-        <v>15</v>
+        <v>152.3877516570505</v>
       </c>
     </row>
     <row r="449">
@@ -8999,10 +8999,10 @@
         </is>
       </c>
       <c r="E449" s="2" t="n">
-        <v>8</v>
+        <v>29.22659679188993</v>
       </c>
       <c r="F449" s="2" t="n">
-        <v>16</v>
+        <v>225.6220294016744</v>
       </c>
     </row>
     <row r="450">
@@ -9025,10 +9025,10 @@
         </is>
       </c>
       <c r="E450" s="2" t="n">
-        <v>8.5</v>
+        <v>40.66843793549465</v>
       </c>
       <c r="F450" s="2" t="n">
-        <v>17</v>
+        <v>350.2750403300375</v>
       </c>
     </row>
     <row r="451">
@@ -9051,10 +9051,10 @@
         </is>
       </c>
       <c r="E451" s="2" t="n">
-        <v>9</v>
+        <v>58.38168153185204</v>
       </c>
       <c r="F451" s="2" t="n">
-        <v>18</v>
+        <v>561.4053560864236</v>
       </c>
     </row>
     <row r="452">
@@ -9077,10 +9077,10 @@
         </is>
       </c>
       <c r="E452" s="2" t="n">
-        <v>9.5</v>
+        <v>85.7150389380769</v>
       </c>
       <c r="F452" s="2" t="n">
-        <v>19</v>
+        <v>920.6358387133145</v>
       </c>
     </row>
     <row r="453">
@@ -9103,10 +9103,10 @@
         </is>
       </c>
       <c r="E453" s="2" t="n">
-        <v>10</v>
+        <v>128</v>
       </c>
       <c r="F453" s="2" t="n">
-        <v>20</v>
+        <v>1536</v>
       </c>
     </row>
     <row r="454">
@@ -9129,10 +9129,10 @@
         </is>
       </c>
       <c r="E454" s="2" t="n">
-        <v>10</v>
+        <v>128</v>
       </c>
       <c r="F454" s="2" t="n">
-        <v>20</v>
+        <v>1536</v>
       </c>
     </row>
     <row r="455">
@@ -9155,10 +9155,10 @@
         </is>
       </c>
       <c r="E455" s="2" t="n">
-        <v>10.25</v>
+        <v>72.59462802062869</v>
       </c>
       <c r="F455" s="2" t="n">
-        <v>20.5</v>
+        <v>701.3381552236845</v>
       </c>
     </row>
     <row r="456">
@@ -9181,10 +9181,10 @@
         </is>
       </c>
       <c r="E456" s="2" t="n">
-        <v>10.5</v>
+        <v>62.65739136757894</v>
       </c>
       <c r="F456" s="2" t="n">
-        <v>21</v>
+        <v>507.3924255641834</v>
       </c>
     </row>
     <row r="457">
@@ -9207,10 +9207,10 @@
         </is>
       </c>
       <c r="E457" s="2" t="n">
-        <v>10.75</v>
+        <v>62.62172690043518</v>
       </c>
       <c r="F457" s="2" t="n">
-        <v>21.5</v>
+        <v>428.2189118107935</v>
       </c>
     </row>
     <row r="458">
@@ -9233,10 +9233,10 @@
         </is>
       </c>
       <c r="E458" s="2" t="n">
-        <v>11</v>
+        <v>67.49593410117721</v>
       </c>
       <c r="F458" s="2" t="n">
-        <v>22</v>
+        <v>390.7888182304993</v>
       </c>
     </row>
     <row r="459">
@@ -9259,10 +9259,10 @@
         </is>
       </c>
       <c r="E459" s="2" t="n">
-        <v>11.25</v>
+        <v>76.18720029841968</v>
       </c>
       <c r="F459" s="2" t="n">
-        <v>22.5</v>
+        <v>373.9509702999416</v>
       </c>
     </row>
     <row r="460">
@@ -9285,10 +9285,10 @@
         </is>
       </c>
       <c r="E460" s="2" t="n">
-        <v>11.5</v>
+        <v>88.7209700324954</v>
       </c>
       <c r="F460" s="2" t="n">
-        <v>23</v>
+        <v>369.4254999388413</v>
       </c>
     </row>
     <row r="461">
@@ -9311,10 +9311,10 @@
         </is>
       </c>
       <c r="E461" s="2" t="n">
-        <v>11.75</v>
+        <v>105.6651728380158</v>
       </c>
       <c r="F461" s="2" t="n">
-        <v>23.5</v>
+        <v>373.4075033600386</v>
       </c>
     </row>
     <row r="462">
@@ -9337,10 +9337,10 @@
         </is>
       </c>
       <c r="E462" s="2" t="n">
-        <v>12</v>
+        <v>128</v>
       </c>
       <c r="F462" s="2" t="n">
-        <v>24</v>
+        <v>384</v>
       </c>
     </row>
     <row r="463">
@@ -9363,10 +9363,10 @@
         </is>
       </c>
       <c r="E463" s="2" t="n">
-        <v>12</v>
+        <v>128</v>
       </c>
       <c r="F463" s="2" t="n">
-        <v>24</v>
+        <v>384</v>
       </c>
     </row>
     <row r="464">
@@ -9389,10 +9389,10 @@
         </is>
       </c>
       <c r="E464" s="2" t="n">
-        <v>12.5</v>
+        <v>55.9781105999381</v>
       </c>
       <c r="F464" s="2" t="n">
-        <v>25</v>
+        <v>152.8365826432048</v>
       </c>
     </row>
     <row r="465">
@@ -9415,10 +9415,10 @@
         </is>
       </c>
       <c r="E465" s="2" t="n">
-        <v>13</v>
+        <v>37.25630781091748</v>
       </c>
       <c r="F465" s="2" t="n">
-        <v>26</v>
+        <v>96.3837178932465</v>
       </c>
     </row>
     <row r="466">
@@ -9441,10 +9441,10 @@
         </is>
       </c>
       <c r="E466" s="2" t="n">
-        <v>13.5</v>
+        <v>28.71218838007889</v>
       </c>
       <c r="F466" s="2" t="n">
-        <v>27</v>
+        <v>70.90639107984764</v>
       </c>
     </row>
     <row r="467">
@@ -9467,10 +9467,10 @@
         </is>
       </c>
       <c r="E467" s="2" t="n">
-        <v>14</v>
+        <v>23.86341635273137</v>
       </c>
       <c r="F467" s="2" t="n">
-        <v>28</v>
+        <v>56.40550735041862</v>
       </c>
     </row>
     <row r="468">
@@ -9493,10 +9493,10 @@
         </is>
       </c>
       <c r="E468" s="2" t="n">
-        <v>14.5</v>
+        <v>20.77068276388587</v>
       </c>
       <c r="F468" s="2" t="n">
-        <v>29</v>
+        <v>47.04937827586711</v>
       </c>
     </row>
     <row r="469">
@@ -9519,10 +9519,10 @@
         </is>
       </c>
       <c r="E469" s="2" t="n">
-        <v>15</v>
+        <v>18.65128641453941</v>
       </c>
       <c r="F469" s="2" t="n">
-        <v>30</v>
+        <v>40.51594168262429</v>
       </c>
     </row>
     <row r="470">
@@ -9545,10 +9545,10 @@
         </is>
       </c>
       <c r="E470" s="2" t="n">
-        <v>15.5</v>
+        <v>17.12884696067179</v>
       </c>
       <c r="F470" s="2" t="n">
-        <v>31</v>
+        <v>35.69784104042281</v>
       </c>
     </row>
     <row r="471">
@@ -9596,10 +9596,10 @@
           <t>elite</t>
         </is>
       </c>
-      <c r="E472" t="n">
+      <c r="E472" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="F472" t="n">
+      <c r="F472" s="2" t="n">
         <v>32</v>
       </c>
     </row>
@@ -9622,11 +9622,11 @@
           <t>elite</t>
         </is>
       </c>
-      <c r="E473" t="n">
-        <v>3.391110215352182</v>
-      </c>
-      <c r="F473" t="n">
-        <v>5.605023522991008</v>
+      <c r="E473" s="2" t="n">
+        <v>3.235952807469516</v>
+      </c>
+      <c r="F473" s="2" t="n">
+        <v>5.588455157324755</v>
       </c>
     </row>
     <row r="474">
@@ -9648,11 +9648,11 @@
           <t>elite</t>
         </is>
       </c>
-      <c r="E474" t="n">
-        <v>2.127461929935275</v>
-      </c>
-      <c r="F474" t="n">
-        <v>3.156649161856778</v>
+      <c r="E474" s="2" t="n">
+        <v>1.97621037190018</v>
+      </c>
+      <c r="F474" s="2" t="n">
+        <v>3.140985228833101</v>
       </c>
     </row>
     <row r="475">
@@ -9674,11 +9674,11 @@
           <t>elite</t>
         </is>
       </c>
-      <c r="E475" t="n">
-        <v>1.648015526593405</v>
-      </c>
-      <c r="F475" t="n">
-        <v>2.236366506256873</v>
+      <c r="E475" s="2" t="n">
+        <v>1.513142604888616</v>
+      </c>
+      <c r="F475" s="2" t="n">
+        <v>2.222770152728302</v>
       </c>
     </row>
     <row r="476">
@@ -9700,11 +9700,11 @@
           <t>elite</t>
         </is>
       </c>
-      <c r="E476" t="n">
-        <v>1.395646246917129</v>
-      </c>
-      <c r="F476" t="n">
-        <v>1.753846098162387</v>
+      <c r="E476" s="2" t="n">
+        <v>1.282015940389144</v>
+      </c>
+      <c r="F476" s="2" t="n">
+        <v>1.742688300058309</v>
       </c>
     </row>
     <row r="477">
@@ -9726,11 +9726,11 @@
           <t>boss</t>
         </is>
       </c>
-      <c r="E477" t="n">
-        <v>1.239919029849584</v>
-      </c>
-      <c r="F477" t="n">
-        <v>1.456750492140449</v>
+      <c r="E477" s="2" t="n">
+        <v>1.150725459593069</v>
+      </c>
+      <c r="F477" s="2" t="n">
+        <v>1.44821976633041</v>
       </c>
     </row>
     <row r="478">
@@ -9752,11 +9752,11 @@
           <t>boss</t>
         </is>
       </c>
-      <c r="E478" t="n">
-        <v>1.134242642197337</v>
-      </c>
-      <c r="F478" t="n">
-        <v>1.255422883125648</v>
+      <c r="E478" s="2" t="n">
+        <v>1.072187376389279</v>
+      </c>
+      <c r="F478" s="2" t="n">
+        <v>1.249643672739781</v>
       </c>
     </row>
     <row r="479">
@@ -9778,11 +9778,11 @@
           <t>boss</t>
         </is>
       </c>
-      <c r="E479" t="n">
-        <v>1.057828295156404</v>
-      </c>
-      <c r="F479" t="n">
-        <v>1.109984786431736</v>
+      <c r="E479" s="2" t="n">
+        <v>1.025492519529902</v>
+      </c>
+      <c r="F479" s="2" t="n">
+        <v>1.107053703990455</v>
       </c>
     </row>
     <row r="480">
@@ -9804,10 +9804,10 @@
           <t>ultimate</t>
         </is>
       </c>
-      <c r="E480" t="n">
+      <c r="E480" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="F480" t="n">
+      <c r="F480" s="2" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Calibrate stronger accumulation bands with paid checkpoint probes
Stage checkpoint only; normal 1x total pacing remains unverified. Ratio/import checks pass. Fixed 14-stage QA over 900 game seconds: passive reaches wave 6; reactor 42-to-46 purchase at 300 seconds costs 7317394 uranium and reaches wave 9. Full 11-20 candidate calibration is still running.
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/monGroup.xlsx
+++ b/space-battleship/config_excel/monGroup.xlsx
@@ -7517,10 +7517,10 @@
         </is>
       </c>
       <c r="E392" s="2" t="n">
-        <v>0.5324901793116744</v>
+        <v>0.5676004044101436</v>
       </c>
       <c r="F392" s="2" t="n">
-        <v>0.4866262989023714</v>
+        <v>0.5306697418713109</v>
       </c>
     </row>
     <row r="393">
@@ -7543,10 +7543,10 @@
         </is>
       </c>
       <c r="E393" s="2" t="n">
-        <v>0.5685766072036965</v>
+        <v>0.6460277524252244</v>
       </c>
       <c r="F393" s="2" t="n">
-        <v>0.5893697628939644</v>
+        <v>0.700882715400969</v>
       </c>
     </row>
     <row r="394">
@@ -7569,10 +7569,10 @@
         </is>
       </c>
       <c r="E394" s="2" t="n">
-        <v>0.7330769879429946</v>
+        <v>0.8878566826756916</v>
       </c>
       <c r="F394" s="2" t="n">
-        <v>0.8814634834042079</v>
+        <v>1.143116711259041</v>
       </c>
     </row>
     <row r="395">
@@ -7595,10 +7595,10 @@
         </is>
       </c>
       <c r="E395" s="2" t="n">
-        <v>1.033966733686373</v>
+        <v>1.3348453133666</v>
       </c>
       <c r="F395" s="2" t="n">
-        <v>1.452249478385389</v>
+        <v>2.05379090828187</v>
       </c>
     </row>
     <row r="396">
@@ -7621,10 +7621,10 @@
         </is>
       </c>
       <c r="E396" s="2" t="n">
-        <v>1.53731829326964</v>
+        <v>2.115530366424058</v>
       </c>
       <c r="F396" s="2" t="n">
-        <v>2.529921892018751</v>
+        <v>3.901672929307857</v>
       </c>
     </row>
     <row r="397">
@@ -7647,10 +7647,10 @@
         </is>
       </c>
       <c r="E397" s="2" t="n">
-        <v>2.366494402833543</v>
+        <v>3.471299164982791</v>
       </c>
       <c r="F397" s="2" t="n">
-        <v>4.570446168006661</v>
+        <v>7.686543597573756</v>
       </c>
     </row>
     <row r="398">
@@ -7673,10 +7673,10 @@
         </is>
       </c>
       <c r="E398" s="2" t="n">
-        <v>3.733702808621944</v>
+        <v>5.837910093709082</v>
       </c>
       <c r="F398" s="2" t="n">
-        <v>8.470668656818301</v>
+        <v>15.53527481389893</v>
       </c>
     </row>
     <row r="399">
@@ -7699,10 +7699,10 @@
         </is>
       </c>
       <c r="E399" s="2" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F399" s="2" t="n">
-        <v>16</v>
+        <v>32</v>
       </c>
     </row>
     <row r="400">
@@ -7725,10 +7725,10 @@
         </is>
       </c>
       <c r="E400" s="2" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F400" s="2" t="n">
-        <v>16</v>
+        <v>32</v>
       </c>
     </row>
     <row r="401">
@@ -7751,10 +7751,10 @@
         </is>
       </c>
       <c r="E401" s="2" t="n">
-        <v>3.478938441688168</v>
+        <v>6.70562466700849</v>
       </c>
       <c r="F401" s="2" t="n">
-        <v>8.826387079624727</v>
+        <v>20.99280462971563</v>
       </c>
     </row>
     <row r="402">
@@ -7777,10 +7777,10 @@
         </is>
       </c>
       <c r="E402" s="2" t="n">
-        <v>3.259663030130004</v>
+        <v>7.266226829631691</v>
       </c>
       <c r="F402" s="2" t="n">
-        <v>9.427003419616131</v>
+        <v>26.66359217711736</v>
       </c>
     </row>
     <row r="403">
@@ -7803,10 +7803,10 @@
         </is>
       </c>
       <c r="E403" s="2" t="n">
-        <v>3.575145032011695</v>
+        <v>9.216661891152189</v>
       </c>
       <c r="F403" s="2" t="n">
-        <v>12.1047694889808</v>
+        <v>40.71542908302596</v>
       </c>
     </row>
     <row r="404">
@@ -7829,10 +7829,10 @@
         </is>
       </c>
       <c r="E404" s="2" t="n">
-        <v>4.245160408187956</v>
+        <v>12.65662299746536</v>
       </c>
       <c r="F404" s="2" t="n">
-        <v>16.97957173522325</v>
+        <v>67.91828694089298</v>
       </c>
     </row>
     <row r="405">
@@ -7855,10 +7855,10 @@
         </is>
       </c>
       <c r="E405" s="2" t="n">
-        <v>5.28854526470762</v>
+        <v>18.23491368420642</v>
       </c>
       <c r="F405" s="2" t="n">
-        <v>25.09140256607924</v>
+        <v>119.3554978279158</v>
       </c>
     </row>
     <row r="406">
@@ -7881,10 +7881,10 @@
         </is>
       </c>
       <c r="E406" s="2" t="n">
-        <v>6.803814155506166</v>
+        <v>27.13086721357822</v>
       </c>
       <c r="F406" s="2" t="n">
-        <v>38.37624408240584</v>
+        <v>217.0888194171143</v>
       </c>
     </row>
     <row r="407">
@@ -7907,10 +7907,10 @@
         </is>
       </c>
       <c r="E407" s="2" t="n">
-        <v>8.957652652226891</v>
+        <v>41.30942962945242</v>
       </c>
       <c r="F407" s="2" t="n">
-        <v>60.14590712943249</v>
+        <v>404.6118215785808</v>
       </c>
     </row>
     <row r="408">
@@ -7933,10 +7933,10 @@
         </is>
       </c>
       <c r="E408" s="2" t="n">
-        <v>12</v>
+        <v>64</v>
       </c>
       <c r="F408" s="2" t="n">
-        <v>96</v>
+        <v>768</v>
       </c>
     </row>
     <row r="409">
@@ -7959,10 +7959,10 @@
         </is>
       </c>
       <c r="E409" s="2" t="n">
-        <v>12</v>
+        <v>64</v>
       </c>
       <c r="F409" s="2" t="n">
-        <v>96</v>
+        <v>768</v>
       </c>
     </row>
     <row r="410">
@@ -7985,10 +7985,10 @@
         </is>
       </c>
       <c r="E410" s="2" t="n">
-        <v>6.065080688320603</v>
+        <v>28.6147014703964</v>
       </c>
       <c r="F410" s="2" t="n">
-        <v>35.59654231167815</v>
+        <v>239.4640386025386</v>
       </c>
     </row>
     <row r="411">
@@ -8011,10 +8011,10 @@
         </is>
       </c>
       <c r="E411" s="2" t="n">
-        <v>4.953616586983959</v>
+        <v>20.67421049569029</v>
       </c>
       <c r="F411" s="2" t="n">
-        <v>25.55477753400599</v>
+        <v>144.5596518880741</v>
       </c>
     </row>
     <row r="412">
@@ -8037,10 +8037,10 @@
         </is>
       </c>
       <c r="E412" s="2" t="n">
-        <v>4.735907262666692</v>
+        <v>17.4849197301217</v>
       </c>
       <c r="F412" s="2" t="n">
-        <v>22.05609168050223</v>
+        <v>104.9170446224223</v>
       </c>
     </row>
     <row r="413">
@@ -8063,10 +8063,10 @@
         </is>
       </c>
       <c r="E413" s="2" t="n">
-        <v>4.901889008840915</v>
+        <v>16.00950246322323</v>
       </c>
       <c r="F413" s="2" t="n">
-        <v>20.79564340114026</v>
+        <v>83.18257360456101</v>
       </c>
     </row>
     <row r="414">
@@ -8089,10 +8089,10 @@
         </is>
       </c>
       <c r="E414" s="2" t="n">
-        <v>5.323109957194588</v>
+        <v>15.37919868190371</v>
       </c>
       <c r="F414" s="2" t="n">
-        <v>20.65590191253872</v>
+        <v>69.47789548834463</v>
       </c>
     </row>
     <row r="415">
@@ -8115,10 +8115,10 @@
         </is>
       </c>
       <c r="E415" s="2" t="n">
-        <v>5.969548666013317</v>
+        <v>15.25680782244698</v>
       </c>
       <c r="F415" s="2" t="n">
-        <v>21.2351477360025</v>
+        <v>60.06206785450212</v>
       </c>
     </row>
     <row r="416">
@@ -8141,10 +8141,10 @@
         </is>
       </c>
       <c r="E416" s="2" t="n">
-        <v>6.850828815107059</v>
+        <v>15.48885103497648</v>
       </c>
       <c r="F416" s="2" t="n">
-        <v>22.3703352813583</v>
+        <v>53.20592376317538</v>
       </c>
     </row>
     <row r="417">
@@ -8167,10 +8167,10 @@
         </is>
       </c>
       <c r="E417" s="2" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="F417" s="2" t="n">
-        <v>24</v>
+        <v>48</v>
       </c>
     </row>
     <row r="418">
@@ -8193,10 +8193,10 @@
         </is>
       </c>
       <c r="E418" s="2" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="F418" s="2" t="n">
-        <v>24</v>
+        <v>48</v>
       </c>
     </row>
     <row r="419">
@@ -8219,10 +8219,10 @@
         </is>
       </c>
       <c r="E419" s="2" t="n">
-        <v>5.058412362836491</v>
+        <v>11.60604854400072</v>
       </c>
       <c r="F419" s="2" t="n">
-        <v>14.2268552436008</v>
+        <v>32.64217322391502</v>
       </c>
     </row>
     <row r="420">
@@ -8245,10 +8245,10 @@
         </is>
       </c>
       <c r="E420" s="2" t="n">
-        <v>5.168552623922572</v>
+        <v>13.60439558584383</v>
       </c>
       <c r="F420" s="2" t="n">
-        <v>16.32804888590069</v>
+        <v>42.97784164190359</v>
       </c>
     </row>
     <row r="421">
@@ -8271,10 +8271,10 @@
         </is>
       </c>
       <c r="E421" s="2" t="n">
-        <v>6.181852654835754</v>
+        <v>18.6667673852378</v>
       </c>
       <c r="F421" s="2" t="n">
-        <v>22.52951460951273</v>
+        <v>68.03028671172113</v>
       </c>
     </row>
     <row r="422">
@@ -8297,10 +8297,10 @@
         </is>
       </c>
       <c r="E422" s="2" t="n">
-        <v>8.004751231611612</v>
+        <v>27.72927167020172</v>
       </c>
       <c r="F422" s="2" t="n">
-        <v>33.9591434704465</v>
+        <v>117.6379237446685</v>
       </c>
     </row>
     <row r="423">
@@ -8323,10 +8323,10 @@
         </is>
       </c>
       <c r="E423" s="2" t="n">
-        <v>10.87473567718933</v>
+        <v>43.21648985876418</v>
       </c>
       <c r="F423" s="2" t="n">
-        <v>53.92493348957762</v>
+        <v>214.2991250973733</v>
       </c>
     </row>
     <row r="424">
@@ -8349,10 +8349,10 @@
         </is>
       </c>
       <c r="E424" s="2" t="n">
-        <v>15.25680782244697</v>
+        <v>69.55600219574146</v>
       </c>
       <c r="F424" s="2" t="n">
-        <v>88.62613940585517</v>
+        <v>404.0478204126096</v>
       </c>
     </row>
     <row r="425">
@@ -8375,10 +8375,10 @@
         </is>
       </c>
       <c r="E425" s="2" t="n">
-        <v>21.90454319924028</v>
+        <v>114.5632417799229</v>
       </c>
       <c r="F425" s="2" t="n">
-        <v>149.2588624793426</v>
+        <v>780.6407554123412</v>
       </c>
     </row>
     <row r="426">
@@ -8401,10 +8401,10 @@
         </is>
       </c>
       <c r="E426" s="2" t="n">
-        <v>32</v>
+        <v>192</v>
       </c>
       <c r="F426" s="2" t="n">
-        <v>256</v>
+        <v>1536</v>
       </c>
     </row>
     <row r="427">
@@ -8427,10 +8427,10 @@
         </is>
       </c>
       <c r="E427" s="2" t="n">
-        <v>32</v>
+        <v>192</v>
       </c>
       <c r="F427" s="2" t="n">
-        <v>256</v>
+        <v>1536</v>
       </c>
     </row>
     <row r="428">
@@ -8453,10 +8453,10 @@
         </is>
       </c>
       <c r="E428" s="2" t="n">
-        <v>19.79125080161339</v>
+        <v>123.0954030924953</v>
       </c>
       <c r="F428" s="2" t="n">
-        <v>159.4681191773176</v>
+        <v>956.8087150639058</v>
       </c>
     </row>
     <row r="429">
@@ -8479,10 +8479,10 @@
         </is>
       </c>
       <c r="E429" s="2" t="n">
-        <v>18.62815390545874</v>
+        <v>120.1035244331235</v>
       </c>
       <c r="F429" s="2" t="n">
-        <v>157.3939522338765</v>
+        <v>944.3637134032589</v>
       </c>
     </row>
     <row r="430">
@@ -8505,10 +8505,10 @@
         </is>
       </c>
       <c r="E430" s="2" t="n">
-        <v>20.30258310625938</v>
+        <v>135.692103049277</v>
       </c>
       <c r="F430" s="2" t="n">
-        <v>181.2205985098322</v>
+        <v>1087.323591058993</v>
       </c>
     </row>
     <row r="431">
@@ -8531,10 +8531,10 @@
         </is>
       </c>
       <c r="E431" s="2" t="n">
-        <v>23.86341635273138</v>
+        <v>165.330598260403</v>
       </c>
       <c r="F431" s="2" t="n">
-        <v>225.6220294016744</v>
+        <v>1353.732176410047</v>
       </c>
     </row>
     <row r="432">
@@ -8557,10 +8557,10 @@
         </is>
       </c>
       <c r="E432" s="2" t="n">
-        <v>29.37418126443648</v>
+        <v>210.9617557624764</v>
       </c>
       <c r="F432" s="2" t="n">
-        <v>294.5450257663789</v>
+        <v>1767.270154598273</v>
       </c>
     </row>
     <row r="433">
@@ -8583,10 +8583,10 @@
         </is>
       </c>
       <c r="E433" s="2" t="n">
-        <v>37.30257282907881</v>
+        <v>277.7116442540056</v>
       </c>
       <c r="F433" s="2" t="n">
-        <v>396.9735342831585</v>
+        <v>2381.841205698951</v>
       </c>
     </row>
     <row r="434">
@@ -8609,10 +8609,10 @@
         </is>
       </c>
       <c r="E434" s="2" t="n">
-        <v>48.44769535919042</v>
+        <v>373.8916510707061</v>
       </c>
       <c r="F434" s="2" t="n">
-        <v>547.4133448621855</v>
+        <v>3284.480069173113</v>
       </c>
     </row>
     <row r="435">
@@ -8635,10 +8635,10 @@
         </is>
       </c>
       <c r="E435" s="2" t="n">
-        <v>64</v>
+        <v>512</v>
       </c>
       <c r="F435" s="2" t="n">
-        <v>768</v>
+        <v>4608</v>
       </c>
     </row>
     <row r="436">
@@ -8661,10 +8661,10 @@
         </is>
       </c>
       <c r="E436" s="2" t="n">
-        <v>64</v>
+        <v>512</v>
       </c>
       <c r="F436" s="2" t="n">
-        <v>768</v>
+        <v>4608</v>
       </c>
     </row>
     <row r="437">
@@ -8687,10 +8687,10 @@
         </is>
       </c>
       <c r="E437" s="2" t="n">
-        <v>32.10911954299499</v>
+        <v>223.9124423997523</v>
       </c>
       <c r="F437" s="2" t="n">
-        <v>333.3389504130951</v>
+        <v>1834.038991718458</v>
       </c>
     </row>
     <row r="438">
@@ -8713,10 +8713,10 @@
         </is>
       </c>
       <c r="E438" s="2" t="n">
-        <v>24.51602926425373</v>
+        <v>149.0252312436699</v>
       </c>
       <c r="F438" s="2" t="n">
-        <v>229.2404061781276</v>
+        <v>1156.604614718958</v>
       </c>
     </row>
     <row r="439">
@@ -8739,10 +8739,10 @@
         </is>
       </c>
       <c r="E439" s="2" t="n">
-        <v>21.67488338600252</v>
+        <v>114.8487535203156</v>
       </c>
       <c r="F439" s="2" t="n">
-        <v>183.9084252597998</v>
+        <v>850.8766929581715</v>
       </c>
     </row>
     <row r="440">
@@ -8765,10 +8765,10 @@
         </is>
       </c>
       <c r="E440" s="2" t="n">
-        <v>20.66632478255037</v>
+        <v>95.4536654109255</v>
       </c>
       <c r="F440" s="2" t="n">
-        <v>159.5388669749946</v>
+        <v>676.8660882050235</v>
       </c>
     </row>
     <row r="441">
@@ -8791,10 +8791,10 @@
         </is>
       </c>
       <c r="E441" s="2" t="n">
-        <v>20.63581193306492</v>
+        <v>83.08273105554346</v>
       </c>
       <c r="F441" s="2" t="n">
-        <v>145.1201210115109</v>
+        <v>564.5925393104054</v>
       </c>
     </row>
     <row r="442">
@@ -8817,10 +8817,10 @@
         </is>
       </c>
       <c r="E442" s="2" t="n">
-        <v>21.25786950161368</v>
+        <v>74.60514565815761</v>
       </c>
       <c r="F442" s="2" t="n">
-        <v>136.2788404861893</v>
+        <v>486.1913001914915</v>
       </c>
     </row>
     <row r="443">
@@ -8843,10 +8843,10 @@
         </is>
       </c>
       <c r="E443" s="2" t="n">
-        <v>22.3964523925201</v>
+        <v>68.51538784268716</v>
       </c>
       <c r="F443" s="2" t="n">
-        <v>130.9402582709814</v>
+        <v>428.3740924850737</v>
       </c>
     </row>
     <row r="444">
@@ -8869,10 +8869,10 @@
         </is>
       </c>
       <c r="E444" s="2" t="n">
-        <v>24</v>
+        <v>64</v>
       </c>
       <c r="F444" s="2" t="n">
-        <v>128</v>
+        <v>384.0000000000001</v>
       </c>
     </row>
     <row r="445">
@@ -8895,10 +8895,10 @@
         </is>
       </c>
       <c r="E445" s="2" t="n">
-        <v>24</v>
+        <v>64</v>
       </c>
       <c r="F445" s="2" t="n">
-        <v>128</v>
+        <v>384.0000000000001</v>
       </c>
     </row>
     <row r="446">
@@ -8921,10 +8921,10 @@
         </is>
       </c>
       <c r="E446" s="2" t="n">
-        <v>16.77956111598912</v>
+        <v>51.3321537511015</v>
       </c>
       <c r="F446" s="2" t="n">
-        <v>94.82031097088398</v>
+        <v>294.8763703041248</v>
       </c>
     </row>
     <row r="447">
@@ -8947,10 +8947,10 @@
         </is>
       </c>
       <c r="E447" s="2" t="n">
-        <v>17.8534957240967</v>
+        <v>62.65739136757894</v>
       </c>
       <c r="F447" s="2" t="n">
-        <v>111.2943309423256</v>
+        <v>358.7806248391246</v>
       </c>
     </row>
     <row r="448">
@@ -8973,10 +8973,10 @@
         </is>
       </c>
       <c r="E448" s="2" t="n">
-        <v>21.9963608110104</v>
+        <v>88.56049548181952</v>
       </c>
       <c r="F448" s="2" t="n">
-        <v>152.3877516570505</v>
+        <v>509.2409767041184</v>
       </c>
     </row>
     <row r="449">
@@ -8999,10 +8999,10 @@
         </is>
       </c>
       <c r="E449" s="2" t="n">
-        <v>29.22659679188993</v>
+        <v>134.9918682023545</v>
       </c>
       <c r="F449" s="2" t="n">
-        <v>225.6220294016744</v>
+        <v>781.5776364609985</v>
       </c>
     </row>
     <row r="450">
@@ -9025,10 +9025,10 @@
         </is>
       </c>
       <c r="E450" s="2" t="n">
-        <v>40.66843793549465</v>
+        <v>215.4899438825213</v>
       </c>
       <c r="F450" s="2" t="n">
-        <v>350.2750403300375</v>
+        <v>1257.816121623477</v>
       </c>
     </row>
     <row r="451">
@@ -9051,10 +9051,10 @@
         </is>
       </c>
       <c r="E451" s="2" t="n">
-        <v>58.38168153185204</v>
+        <v>354.8838801299817</v>
       </c>
       <c r="F451" s="2" t="n">
-        <v>561.4053560864236</v>
+        <v>2089.786209199881</v>
       </c>
     </row>
     <row r="452">
@@ -9077,10 +9077,10 @@
         </is>
       </c>
       <c r="E452" s="2" t="n">
-        <v>85.7150389380769</v>
+        <v>597.7324819920763</v>
       </c>
       <c r="F452" s="2" t="n">
-        <v>920.6358387133145</v>
+        <v>3552.470878329283</v>
       </c>
     </row>
     <row r="453">
@@ -9103,10 +9103,10 @@
         </is>
       </c>
       <c r="E453" s="2" t="n">
-        <v>128</v>
+        <v>1024</v>
       </c>
       <c r="F453" s="2" t="n">
-        <v>1536</v>
+        <v>6144</v>
       </c>
     </row>
     <row r="454">
@@ -9129,10 +9129,10 @@
         </is>
       </c>
       <c r="E454" s="2" t="n">
-        <v>128</v>
+        <v>1024</v>
       </c>
       <c r="F454" s="2" t="n">
-        <v>1536</v>
+        <v>6144</v>
       </c>
     </row>
     <row r="455">
@@ -9155,10 +9155,10 @@
         </is>
       </c>
       <c r="E455" s="2" t="n">
-        <v>72.59462802062869</v>
+        <v>488.3564997537882</v>
       </c>
       <c r="F455" s="2" t="n">
-        <v>701.3381552236845</v>
+        <v>2445.385322291276</v>
       </c>
     </row>
     <row r="456">
@@ -9181,10 +9181,10 @@
         </is>
       </c>
       <c r="E456" s="2" t="n">
-        <v>62.65739136757894</v>
+        <v>354.4437306197962</v>
       </c>
       <c r="F456" s="2" t="n">
-        <v>507.3924255641834</v>
+        <v>1542.139486291944</v>
       </c>
     </row>
     <row r="457">
@@ -9207,10 +9207,10 @@
         </is>
       </c>
       <c r="E457" s="2" t="n">
-        <v>62.62172690043518</v>
+        <v>297.8808127350192</v>
       </c>
       <c r="F457" s="2" t="n">
-        <v>428.2189118107935</v>
+        <v>1134.502257277562</v>
       </c>
     </row>
     <row r="458">
@@ -9233,10 +9233,10 @@
         </is>
       </c>
       <c r="E458" s="2" t="n">
-        <v>67.49593410117721</v>
+        <v>269.9837364047089</v>
       </c>
       <c r="F458" s="2" t="n">
-        <v>390.7888182304993</v>
+        <v>902.4881176066978</v>
       </c>
     </row>
     <row r="459">
@@ -9259,10 +9259,10 @@
         </is>
       </c>
       <c r="E459" s="2" t="n">
-        <v>76.18720029841968</v>
+        <v>256.2621744766313</v>
       </c>
       <c r="F459" s="2" t="n">
-        <v>373.9509702999416</v>
+        <v>752.7900524138739</v>
       </c>
     </row>
     <row r="460">
@@ -9285,10 +9285,10 @@
         </is>
       </c>
       <c r="E460" s="2" t="n">
-        <v>88.7209700324954</v>
+        <v>250.9407981737039</v>
       </c>
       <c r="F460" s="2" t="n">
-        <v>369.4254999388413</v>
+        <v>648.2550669219886</v>
       </c>
     </row>
     <row r="461">
@@ -9311,10 +9311,10 @@
         </is>
       </c>
       <c r="E461" s="2" t="n">
-        <v>105.6651728380158</v>
+        <v>251.3155506939212</v>
       </c>
       <c r="F461" s="2" t="n">
-        <v>373.4075033600386</v>
+        <v>571.1654566467648</v>
       </c>
     </row>
     <row r="462">
@@ -9337,10 +9337,10 @@
         </is>
       </c>
       <c r="E462" s="2" t="n">
-        <v>128</v>
+        <v>256</v>
       </c>
       <c r="F462" s="2" t="n">
-        <v>384</v>
+        <v>512</v>
       </c>
     </row>
     <row r="463">
@@ -9363,10 +9363,10 @@
         </is>
       </c>
       <c r="E463" s="2" t="n">
-        <v>128</v>
+        <v>256</v>
       </c>
       <c r="F463" s="2" t="n">
-        <v>384</v>
+        <v>512</v>
       </c>
     </row>
     <row r="464">
@@ -9389,10 +9389,10 @@
         </is>
       </c>
       <c r="E464" s="2" t="n">
-        <v>55.9781105999381</v>
+        <v>108.0017740826299</v>
       </c>
       <c r="F464" s="2" t="n">
-        <v>152.8365826432048</v>
+        <v>202.144749121721</v>
       </c>
     </row>
     <row r="465">
@@ -9415,10 +9415,10 @@
         </is>
       </c>
       <c r="E465" s="2" t="n">
-        <v>37.25630781091748</v>
+        <v>69.34180216208662</v>
       </c>
       <c r="F465" s="2" t="n">
-        <v>96.3837178932465</v>
+        <v>126.4547741947134</v>
       </c>
     </row>
     <row r="466">
@@ -9441,10 +9441,10 @@
         </is>
       </c>
       <c r="E466" s="2" t="n">
-        <v>28.71218838007889</v>
+        <v>51.55185107897695</v>
       </c>
       <c r="F466" s="2" t="n">
-        <v>70.90639107984764</v>
+        <v>92.28122413600921</v>
       </c>
     </row>
     <row r="467">
@@ -9467,10 +9467,10 @@
         </is>
       </c>
       <c r="E467" s="2" t="n">
-        <v>23.86341635273137</v>
+        <v>41.33264956510073</v>
       </c>
       <c r="F467" s="2" t="n">
-        <v>56.40550735041862</v>
+        <v>72.81919686751712</v>
       </c>
     </row>
     <row r="468">
@@ -9493,10 +9493,10 @@
         </is>
       </c>
       <c r="E468" s="2" t="n">
-        <v>20.77068276388587</v>
+        <v>34.70516056072824</v>
       </c>
       <c r="F468" s="2" t="n">
-        <v>47.04937827586711</v>
+        <v>60.25244476556771</v>
       </c>
     </row>
     <row r="469">
@@ -9519,10 +9519,10 @@
         </is>
       </c>
       <c r="E469" s="2" t="n">
-        <v>18.65128641453941</v>
+        <v>30.06316735633945</v>
       </c>
       <c r="F469" s="2" t="n">
-        <v>40.51594168262429</v>
+        <v>51.46869197815998</v>
       </c>
     </row>
     <row r="470">
@@ -9545,10 +9545,10 @@
         </is>
       </c>
       <c r="E470" s="2" t="n">
-        <v>17.12884696067179</v>
+        <v>26.63402053600463</v>
       </c>
       <c r="F470" s="2" t="n">
-        <v>35.69784104042281</v>
+        <v>44.98373942487196</v>
       </c>
     </row>
     <row r="471">
@@ -9571,10 +9571,10 @@
         </is>
       </c>
       <c r="E471" s="2" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="F471" s="2" t="n">
-        <v>32</v>
+        <v>40</v>
       </c>
     </row>
     <row r="472">
@@ -9597,10 +9597,10 @@
         </is>
       </c>
       <c r="E472" s="2" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="F472" s="2" t="n">
-        <v>32</v>
+        <v>40</v>
       </c>
     </row>
     <row r="473">
@@ -9623,10 +9623,10 @@
         </is>
       </c>
       <c r="E473" s="2" t="n">
-        <v>3.235952807469516</v>
+        <v>4.61404717992635</v>
       </c>
       <c r="F473" s="2" t="n">
-        <v>5.588455157324755</v>
+        <v>6.793413216515661</v>
       </c>
     </row>
     <row r="474">
@@ -9649,10 +9649,10 @@
         </is>
       </c>
       <c r="E474" s="2" t="n">
-        <v>1.97621037190018</v>
+        <v>2.678561477405338</v>
       </c>
       <c r="F474" s="2" t="n">
-        <v>3.140985228833101</v>
+        <v>3.713200530214782</v>
       </c>
     </row>
     <row r="475">
@@ -9675,10 +9675,10 @@
         </is>
       </c>
       <c r="E475" s="2" t="n">
-        <v>1.513142604888616</v>
+        <v>1.949561306027979</v>
       </c>
       <c r="F475" s="2" t="n">
-        <v>2.222770152728302</v>
+        <v>2.555426031861377</v>
       </c>
     </row>
     <row r="476">
@@ -9701,10 +9701,10 @@
         </is>
       </c>
       <c r="E476" s="2" t="n">
-        <v>1.282015940389144</v>
+        <v>1.570142448033869</v>
       </c>
       <c r="F476" s="2" t="n">
-        <v>1.742688300058309</v>
+        <v>1.948384751261965</v>
       </c>
     </row>
     <row r="477">
@@ -9727,10 +9727,10 @@
         </is>
       </c>
       <c r="E477" s="2" t="n">
-        <v>1.150725459593069</v>
+        <v>1.339695023226408</v>
       </c>
       <c r="F477" s="2" t="n">
-        <v>1.44821976633041</v>
+        <v>1.574619863309849</v>
       </c>
     </row>
     <row r="478">
@@ -9753,10 +9753,10 @@
         </is>
       </c>
       <c r="E478" s="2" t="n">
-        <v>1.072187376389279</v>
+        <v>1.186570383980938</v>
       </c>
       <c r="F478" s="2" t="n">
-        <v>1.249643672739781</v>
+        <v>1.321337309095369</v>
       </c>
     </row>
     <row r="479">
@@ -9779,10 +9779,10 @@
         </is>
       </c>
       <c r="E479" s="2" t="n">
-        <v>1.025492519529902</v>
+        <v>1.078807368523075</v>
       </c>
       <c r="F479" s="2" t="n">
-        <v>1.107053703990455</v>
+        <v>1.138367375927505</v>
       </c>
     </row>
     <row r="480">

</xml_diff>

<commit_message>
Lift middle-stage combat bands beyond the original stage20 endpoint
User approved raising the complete 11-20 curve and deferring stage21+ transition handling. Preserve first10 stages, all income, reward, unlock and crew behavior. Apply cumulative thresholds from measured V4 local combat growth while keeping release bands after unlocks. Excel and runtime projection stay synchronized.

Experimental V5 calibration has started from the same stage10 QA source with original-rule transactions and fixed1/60 logical steps. A 230 minute middle-stage planning budget is a heuristic, not a measured result or total-duration acceptance. Wave source/boundary and isolation checks pass; stage21+ transition is deliberately unresolved.
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/monGroup.xlsx
+++ b/space-battleship/config_excel/monGroup.xlsx
@@ -7517,10 +7517,10 @@
         </is>
       </c>
       <c r="E392" s="2" t="n">
-        <v>0.5676004044101436</v>
+        <v>0.6027754510829806</v>
       </c>
       <c r="F392" s="2" t="n">
-        <v>0.5306697418713109</v>
+        <v>0.5600005631590167</v>
       </c>
     </row>
     <row r="393">
@@ -7543,10 +7543,10 @@
         </is>
       </c>
       <c r="E393" s="2" t="n">
-        <v>0.6460277524252244</v>
+        <v>0.7285794139621287</v>
       </c>
       <c r="F393" s="2" t="n">
-        <v>0.700882715400969</v>
+        <v>0.7805012925108775</v>
       </c>
     </row>
     <row r="394">
@@ -7569,10 +7569,10 @@
         </is>
       </c>
       <c r="E394" s="2" t="n">
-        <v>0.8878566826756916</v>
+        <v>1.06336276624705</v>
       </c>
       <c r="F394" s="2" t="n">
-        <v>1.143116711259041</v>
+        <v>1.343330850717981</v>
       </c>
     </row>
     <row r="395">
@@ -7595,10 +7595,10 @@
         </is>
       </c>
       <c r="E395" s="2" t="n">
-        <v>1.3348453133666</v>
+        <v>1.69778379120333</v>
       </c>
       <c r="F395" s="2" t="n">
-        <v>2.05379090828187</v>
+        <v>2.546905201566314</v>
       </c>
     </row>
     <row r="396">
@@ -7621,10 +7621,10 @@
         </is>
       </c>
       <c r="E396" s="2" t="n">
-        <v>2.115530366424058</v>
+        <v>2.857482413024759</v>
       </c>
       <c r="F396" s="2" t="n">
-        <v>3.901672929307857</v>
+        <v>5.105891150979167</v>
       </c>
     </row>
     <row r="397">
@@ -7647,10 +7647,10 @@
         </is>
       </c>
       <c r="E397" s="2" t="n">
-        <v>3.471299164982791</v>
+        <v>4.979310477016353</v>
       </c>
       <c r="F397" s="2" t="n">
-        <v>7.686543597573756</v>
+        <v>10.61490043353493</v>
       </c>
     </row>
     <row r="398">
@@ -7673,10 +7673,10 @@
         </is>
       </c>
       <c r="E398" s="2" t="n">
-        <v>5.837910093709082</v>
+        <v>8.892982258863762</v>
       </c>
       <c r="F398" s="2" t="n">
-        <v>15.53527481389893</v>
+        <v>22.63955616989358</v>
       </c>
     </row>
     <row r="399">
@@ -7699,10 +7699,10 @@
         </is>
       </c>
       <c r="E399" s="2" t="n">
-        <v>10</v>
+        <v>16.17718246648805</v>
       </c>
       <c r="F399" s="2" t="n">
-        <v>32</v>
+        <v>49.21110139391978</v>
       </c>
     </row>
     <row r="400">
@@ -7725,10 +7725,10 @@
         </is>
       </c>
       <c r="E400" s="2" t="n">
-        <v>10</v>
+        <v>16.17718246648805</v>
       </c>
       <c r="F400" s="2" t="n">
-        <v>32</v>
+        <v>49.21110139391978</v>
       </c>
     </row>
     <row r="401">
@@ -7751,10 +7751,10 @@
         </is>
       </c>
       <c r="E401" s="2" t="n">
-        <v>6.70562466700849</v>
+        <v>15.42909495998082</v>
       </c>
       <c r="F401" s="2" t="n">
-        <v>20.99280462971563</v>
+        <v>44.24628481726457</v>
       </c>
     </row>
     <row r="402">
@@ -7777,10 +7777,10 @@
         </is>
       </c>
       <c r="E402" s="2" t="n">
-        <v>7.266226829631691</v>
+        <v>23.77981594354123</v>
       </c>
       <c r="F402" s="2" t="n">
-        <v>26.66359217711736</v>
+        <v>77.02261237902138</v>
       </c>
     </row>
     <row r="403">
@@ -7803,10 +7803,10 @@
         </is>
       </c>
       <c r="E403" s="2" t="n">
-        <v>9.216661891152189</v>
+        <v>42.90140550832775</v>
       </c>
       <c r="F403" s="2" t="n">
-        <v>40.71542908302596</v>
+        <v>161.1951023061239</v>
       </c>
     </row>
     <row r="404">
@@ -7829,10 +7829,10 @@
         </is>
       </c>
       <c r="E404" s="2" t="n">
-        <v>12.65662299746536</v>
+        <v>83.79421474191265</v>
       </c>
       <c r="F404" s="2" t="n">
-        <v>67.91828694089298</v>
+        <v>368.5299510566441</v>
       </c>
     </row>
     <row r="405">
@@ -7855,10 +7855,10 @@
         </is>
       </c>
       <c r="E405" s="2" t="n">
-        <v>18.23491368420642</v>
+        <v>171.7110445842339</v>
       </c>
       <c r="F405" s="2" t="n">
-        <v>119.3554978279158</v>
+        <v>887.6090761267244</v>
       </c>
     </row>
     <row r="406">
@@ -7881,10 +7881,10 @@
         </is>
       </c>
       <c r="E406" s="2" t="n">
-        <v>27.13086721357822</v>
+        <v>363.3762351373805</v>
       </c>
       <c r="F406" s="2" t="n">
-        <v>217.0888194171143</v>
+        <v>2212.636144447598</v>
       </c>
     </row>
     <row r="407">
@@ -7907,10 +7907,10 @@
         </is>
       </c>
       <c r="E407" s="2" t="n">
-        <v>41.30942962945242</v>
+        <v>786.9377343543295</v>
       </c>
       <c r="F407" s="2" t="n">
-        <v>404.6118215785808</v>
+        <v>5652.028628082166</v>
       </c>
     </row>
     <row r="408">
@@ -7933,10 +7933,10 @@
         </is>
       </c>
       <c r="E408" s="2" t="n">
-        <v>64</v>
+        <v>1734.081371631208</v>
       </c>
       <c r="F408" s="2" t="n">
-        <v>768</v>
+        <v>14703.48373037106</v>
       </c>
     </row>
     <row r="409">
@@ -7959,10 +7959,10 @@
         </is>
       </c>
       <c r="E409" s="2" t="n">
-        <v>64</v>
+        <v>1734.081371631208</v>
       </c>
       <c r="F409" s="2" t="n">
-        <v>768</v>
+        <v>14703.48373037106</v>
       </c>
     </row>
     <row r="410">
@@ -7985,10 +7985,10 @@
         </is>
       </c>
       <c r="E410" s="2" t="n">
-        <v>28.6147014703964</v>
+        <v>815.9283346805465</v>
       </c>
       <c r="F410" s="2" t="n">
-        <v>239.4640386025386</v>
+        <v>4798.865672930985</v>
       </c>
     </row>
     <row r="411">
@@ -8011,10 +8011,10 @@
         </is>
       </c>
       <c r="E411" s="2" t="n">
-        <v>20.67421049569029</v>
+        <v>620.390339214493</v>
       </c>
       <c r="F411" s="2" t="n">
-        <v>144.5596518880741</v>
+        <v>3032.387168325816</v>
       </c>
     </row>
     <row r="412">
@@ -8037,10 +8037,10 @@
         </is>
       </c>
       <c r="E412" s="2" t="n">
-        <v>17.4849197301217</v>
+        <v>552.1702861222619</v>
       </c>
       <c r="F412" s="2" t="n">
-        <v>104.9170446224223</v>
+        <v>2303.683812768523</v>
       </c>
     </row>
     <row r="413">
@@ -8063,10 +8063,10 @@
         </is>
       </c>
       <c r="E413" s="2" t="n">
-        <v>16.00950246322323</v>
+        <v>532.0598915008038</v>
       </c>
       <c r="F413" s="2" t="n">
-        <v>83.18257360456101</v>
+        <v>1911.826339590628</v>
       </c>
     </row>
     <row r="414">
@@ -8089,10 +8089,10 @@
         </is>
       </c>
       <c r="E414" s="2" t="n">
-        <v>15.37919868190371</v>
+        <v>537.885318771933</v>
       </c>
       <c r="F414" s="2" t="n">
-        <v>69.47789548834463</v>
+        <v>1671.483170935145</v>
       </c>
     </row>
     <row r="415">
@@ -8115,10 +8115,10 @@
         </is>
       </c>
       <c r="E415" s="2" t="n">
-        <v>15.25680782244698</v>
+        <v>561.555849858323</v>
       </c>
       <c r="F415" s="2" t="n">
-        <v>60.06206785450212</v>
+        <v>1512.49831387441</v>
       </c>
     </row>
     <row r="416">
@@ -8141,10 +8141,10 @@
         </is>
       </c>
       <c r="E416" s="2" t="n">
-        <v>15.48885103497648</v>
+        <v>599.9592861488059</v>
       </c>
       <c r="F416" s="2" t="n">
-        <v>53.20592376317538</v>
+        <v>1402.470943645809</v>
       </c>
     </row>
     <row r="417">
@@ -8167,10 +8167,10 @@
         </is>
       </c>
       <c r="E417" s="2" t="n">
-        <v>16</v>
+        <v>652.2226194122828</v>
       </c>
       <c r="F417" s="2" t="n">
-        <v>48</v>
+        <v>1324.385409186241</v>
       </c>
     </row>
     <row r="418">
@@ -8193,10 +8193,10 @@
         </is>
       </c>
       <c r="E418" s="2" t="n">
-        <v>16</v>
+        <v>652.2226194122828</v>
       </c>
       <c r="F418" s="2" t="n">
-        <v>48</v>
+        <v>1324.385409186241</v>
       </c>
     </row>
     <row r="419">
@@ -8219,10 +8219,10 @@
         </is>
       </c>
       <c r="E419" s="2" t="n">
-        <v>11.60604854400072</v>
+        <v>694.9702902148998</v>
       </c>
       <c r="F419" s="2" t="n">
-        <v>32.64217322391502</v>
+        <v>1270.511559572846</v>
       </c>
     </row>
     <row r="420">
@@ -8245,10 +8245,10 @@
         </is>
       </c>
       <c r="E420" s="2" t="n">
-        <v>13.60439558584383</v>
+        <v>1196.649850021172</v>
       </c>
       <c r="F420" s="2" t="n">
-        <v>42.97784164190359</v>
+        <v>2359.774818971994</v>
       </c>
     </row>
     <row r="421">
@@ -8271,10 +8271,10 @@
         </is>
       </c>
       <c r="E421" s="2" t="n">
-        <v>18.6667673852378</v>
+        <v>2411.920213316881</v>
       </c>
       <c r="F421" s="2" t="n">
-        <v>68.03028671172113</v>
+        <v>5269.321145173129</v>
       </c>
     </row>
     <row r="422">
@@ -8297,10 +8297,10 @@
         </is>
       </c>
       <c r="E422" s="2" t="n">
-        <v>27.72927167020172</v>
+        <v>5263.059343519646</v>
       </c>
       <c r="F422" s="2" t="n">
-        <v>117.6379237446685</v>
+        <v>12853.63972927639</v>
       </c>
     </row>
     <row r="423">
@@ -8323,10 +8323,10 @@
         </is>
       </c>
       <c r="E423" s="2" t="n">
-        <v>43.21648985876418</v>
+        <v>12049.11852611687</v>
       </c>
       <c r="F423" s="2" t="n">
-        <v>214.2991250973733</v>
+        <v>33031.29310677554</v>
       </c>
     </row>
     <row r="424">
@@ -8349,10 +8349,10 @@
         </is>
       </c>
       <c r="E424" s="2" t="n">
-        <v>69.55600219574146</v>
+        <v>28486.97812562146</v>
       </c>
       <c r="F424" s="2" t="n">
-        <v>404.0478204126096</v>
+        <v>87854.5688286629</v>
       </c>
     </row>
     <row r="425">
@@ -8375,10 +8375,10 @@
         </is>
       </c>
       <c r="E425" s="2" t="n">
-        <v>114.5632417799229</v>
+        <v>68922.82128562266</v>
       </c>
       <c r="F425" s="2" t="n">
-        <v>780.6407554123412</v>
+        <v>239446.895065223</v>
       </c>
     </row>
     <row r="426">
@@ -8401,10 +8401,10 @@
         </is>
       </c>
       <c r="E426" s="2" t="n">
-        <v>192</v>
+        <v>169677.7761697887</v>
       </c>
       <c r="F426" s="2" t="n">
-        <v>1536</v>
+        <v>664623.3728540518</v>
       </c>
     </row>
     <row r="427">
@@ -8427,10 +8427,10 @@
         </is>
       </c>
       <c r="E427" s="2" t="n">
-        <v>192</v>
+        <v>169677.7761697887</v>
       </c>
       <c r="F427" s="2" t="n">
-        <v>1536</v>
+        <v>664623.3728540518</v>
       </c>
     </row>
     <row r="428">
@@ -8453,10 +8453,10 @@
         </is>
       </c>
       <c r="E428" s="2" t="n">
-        <v>123.0954030924953</v>
+        <v>163384.1315216832</v>
       </c>
       <c r="F428" s="2" t="n">
-        <v>956.8087150639058</v>
+        <v>595744.0091406531</v>
       </c>
     </row>
     <row r="429">
@@ -8479,10 +8479,10 @@
         </is>
       </c>
       <c r="E429" s="2" t="n">
-        <v>120.1035244331235</v>
+        <v>239424.2277375267</v>
       </c>
       <c r="F429" s="2" t="n">
-        <v>944.3637134032589</v>
+        <v>846104.5284947836</v>
       </c>
     </row>
     <row r="430">
@@ -8505,10 +8505,10 @@
         </is>
       </c>
       <c r="E430" s="2" t="n">
-        <v>135.692103049277</v>
+        <v>406266.6949501505</v>
       </c>
       <c r="F430" s="2" t="n">
-        <v>1087.323591058993</v>
+        <v>1401824.693623829</v>
       </c>
     </row>
     <row r="431">
@@ -8531,10 +8531,10 @@
         </is>
       </c>
       <c r="E431" s="2" t="n">
-        <v>165.330598260403</v>
+        <v>743454.1482799333</v>
       </c>
       <c r="F431" s="2" t="n">
-        <v>1353.732176410047</v>
+        <v>2511411.125006217</v>
       </c>
     </row>
     <row r="432">
@@ -8557,10 +8557,10 @@
         </is>
       </c>
       <c r="E432" s="2" t="n">
-        <v>210.9617557624764</v>
+        <v>1424783.861636898</v>
       </c>
       <c r="F432" s="2" t="n">
-        <v>1767.270154598273</v>
+        <v>4717785.29365459</v>
       </c>
     </row>
     <row r="433">
@@ -8583,10 +8583,10 @@
         </is>
       </c>
       <c r="E433" s="2" t="n">
-        <v>277.7116442540056</v>
+        <v>2816979.26326412</v>
       </c>
       <c r="F433" s="2" t="n">
-        <v>2381.841205698951</v>
+        <v>9149517.670550179</v>
       </c>
     </row>
     <row r="434">
@@ -8609,10 +8609,10 @@
         </is>
       </c>
       <c r="E434" s="2" t="n">
-        <v>373.8916510707061</v>
+        <v>5696126.58400094</v>
       </c>
       <c r="F434" s="2" t="n">
-        <v>3284.480069173113</v>
+        <v>18155248.33498522</v>
       </c>
     </row>
     <row r="435">
@@ -8635,10 +8635,10 @@
         </is>
       </c>
       <c r="E435" s="2" t="n">
-        <v>512</v>
+        <v>11715157.44473026</v>
       </c>
       <c r="F435" s="2" t="n">
-        <v>4608</v>
+        <v>36652044.08523786</v>
       </c>
     </row>
     <row r="436">
@@ -8661,10 +8661,10 @@
         </is>
       </c>
       <c r="E436" s="2" t="n">
-        <v>512</v>
+        <v>11715157.44473026</v>
       </c>
       <c r="F436" s="2" t="n">
-        <v>4608</v>
+        <v>36652044.08523786</v>
       </c>
     </row>
     <row r="437">
@@ -8687,10 +8687,10 @@
         </is>
       </c>
       <c r="E437" s="2" t="n">
-        <v>223.9124423997523</v>
+        <v>5466390.319638171</v>
       </c>
       <c r="F437" s="2" t="n">
-        <v>1834.038991718458</v>
+        <v>15458807.36192416</v>
       </c>
     </row>
     <row r="438">
@@ -8713,10 +8713,10 @@
         </is>
       </c>
       <c r="E438" s="2" t="n">
-        <v>149.0252312436699</v>
+        <v>3881740.140855308</v>
       </c>
       <c r="F438" s="2" t="n">
-        <v>1156.604614718958</v>
+        <v>10330801.86883282</v>
       </c>
     </row>
     <row r="439">
@@ -8739,10 +8739,10 @@
         </is>
       </c>
       <c r="E439" s="2" t="n">
-        <v>114.8487535203156</v>
+        <v>3191811.117251148</v>
       </c>
       <c r="F439" s="2" t="n">
-        <v>850.8766929581715</v>
+        <v>8053736.7582355</v>
       </c>
     </row>
     <row r="440">
@@ -8765,10 +8765,10 @@
         </is>
       </c>
       <c r="E440" s="2" t="n">
-        <v>95.4536654109255</v>
+        <v>2830399.570762326</v>
       </c>
       <c r="F440" s="2" t="n">
-        <v>676.8660882050235</v>
+        <v>6789147.582477466</v>
       </c>
     </row>
     <row r="441">
@@ -8791,10 +8791,10 @@
         </is>
       </c>
       <c r="E441" s="2" t="n">
-        <v>83.08273105554346</v>
+        <v>2628513.104791808</v>
       </c>
       <c r="F441" s="2" t="n">
-        <v>564.5925393104054</v>
+        <v>6001078.659770884</v>
       </c>
     </row>
     <row r="442">
@@ -8817,10 +8817,10 @@
         </is>
       </c>
       <c r="E442" s="2" t="n">
-        <v>74.60514565815761</v>
+        <v>2518328.659726613</v>
       </c>
       <c r="F442" s="2" t="n">
-        <v>486.1913001914915</v>
+        <v>5476247.383946548</v>
       </c>
     </row>
     <row r="443">
@@ -8843,10 +8843,10 @@
         </is>
       </c>
       <c r="E443" s="2" t="n">
-        <v>68.51538784268716</v>
+        <v>2467606.971852489</v>
       </c>
       <c r="F443" s="2" t="n">
-        <v>428.3740924850737</v>
+        <v>5113058.523174551</v>
       </c>
     </row>
     <row r="444">
@@ -8869,10 +8869,10 @@
         </is>
       </c>
       <c r="E444" s="2" t="n">
-        <v>64</v>
+        <v>2459303.256776251</v>
       </c>
       <c r="F444" s="2" t="n">
-        <v>384.0000000000001</v>
+        <v>4857026.59523688</v>
       </c>
     </row>
     <row r="445">
@@ -8895,10 +8895,10 @@
         </is>
       </c>
       <c r="E445" s="2" t="n">
-        <v>64</v>
+        <v>2459303.256776251</v>
       </c>
       <c r="F445" s="2" t="n">
-        <v>384.0000000000001</v>
+        <v>4857026.59523688</v>
       </c>
     </row>
     <row r="446">
@@ -8921,10 +8921,10 @@
         </is>
       </c>
       <c r="E446" s="2" t="n">
-        <v>51.3321537511015</v>
+        <v>3162397.326773776</v>
       </c>
       <c r="F446" s="2" t="n">
-        <v>294.8763703041248</v>
+        <v>5689782.461285776</v>
       </c>
     </row>
     <row r="447">
@@ -8947,10 +8947,10 @@
         </is>
       </c>
       <c r="E447" s="2" t="n">
-        <v>62.65739136757894</v>
+        <v>6188623.961584205</v>
       </c>
       <c r="F447" s="2" t="n">
-        <v>358.7806248391246</v>
+        <v>10560904.24790799</v>
       </c>
     </row>
     <row r="448">
@@ -8973,10 +8973,10 @@
         </is>
       </c>
       <c r="E448" s="2" t="n">
-        <v>88.56049548181952</v>
+        <v>14023507.76399199</v>
       </c>
       <c r="F448" s="2" t="n">
-        <v>509.2409767041184</v>
+        <v>22867142.52365892</v>
       </c>
     </row>
     <row r="449">
@@ -8999,10 +8999,10 @@
         </is>
       </c>
       <c r="E449" s="2" t="n">
-        <v>134.9918682023545</v>
+        <v>34270391.53577247</v>
       </c>
       <c r="F449" s="2" t="n">
-        <v>781.5776364609985</v>
+        <v>53539845.48003841</v>
       </c>
     </row>
     <row r="450">
@@ -9025,10 +9025,10 @@
         </is>
       </c>
       <c r="E450" s="2" t="n">
-        <v>215.4899438825213</v>
+        <v>87706807.56329431</v>
       </c>
       <c r="F450" s="2" t="n">
-        <v>1257.816121623477</v>
+        <v>131443337.8668317</v>
       </c>
     </row>
     <row r="451">
@@ -9051,10 +9051,10 @@
         </is>
       </c>
       <c r="E451" s="2" t="n">
-        <v>354.8838801299817</v>
+        <v>231572724.437511</v>
       </c>
       <c r="F451" s="2" t="n">
-        <v>2089.786209199881</v>
+        <v>333149920.5720967</v>
       </c>
     </row>
     <row r="452">
@@ -9077,10 +9077,10 @@
         </is>
       </c>
       <c r="E452" s="2" t="n">
-        <v>597.7324819920763</v>
+        <v>625320729.7944261</v>
       </c>
       <c r="F452" s="2" t="n">
-        <v>3552.470878329283</v>
+        <v>863942451.9009268</v>
       </c>
     </row>
     <row r="453">
@@ -9103,10 +9103,10 @@
         </is>
       </c>
       <c r="E453" s="2" t="n">
-        <v>1024</v>
+        <v>1717476339.055149</v>
       </c>
       <c r="F453" s="2" t="n">
-        <v>6144</v>
+        <v>2279407265.423798</v>
       </c>
     </row>
     <row r="454">
@@ -9129,10 +9129,10 @@
         </is>
       </c>
       <c r="E454" s="2" t="n">
-        <v>1024</v>
+        <v>1717476339.055149</v>
       </c>
       <c r="F454" s="2" t="n">
-        <v>6144</v>
+        <v>2279407265.423798</v>
       </c>
     </row>
     <row r="455">
@@ -9155,10 +9155,10 @@
         </is>
       </c>
       <c r="E455" s="2" t="n">
-        <v>488.3564997537882</v>
+        <v>996630316.2979915</v>
       </c>
       <c r="F455" s="2" t="n">
-        <v>2445.385322291276</v>
+        <v>1081322530.116531</v>
       </c>
     </row>
     <row r="456">
@@ -9181,10 +9181,10 @@
         </is>
       </c>
       <c r="E456" s="2" t="n">
-        <v>354.4437306197962</v>
+        <v>880137926.5145465</v>
       </c>
       <c r="F456" s="2" t="n">
-        <v>1542.139486291944</v>
+        <v>812772194.5311005</v>
       </c>
     </row>
     <row r="457">
@@ -9207,10 +9207,10 @@
         </is>
       </c>
       <c r="E457" s="2" t="n">
-        <v>297.8808127350192</v>
+        <v>900020252.8655517</v>
       </c>
       <c r="F457" s="2" t="n">
-        <v>1134.502257277562</v>
+        <v>712668845.9968609</v>
       </c>
     </row>
     <row r="458">
@@ -9233,10 +9233,10 @@
         </is>
       </c>
       <c r="E458" s="2" t="n">
-        <v>269.9837364047089</v>
+        <v>992552919.2990483</v>
       </c>
       <c r="F458" s="2" t="n">
-        <v>902.4881176066978</v>
+        <v>675711222.6800796</v>
       </c>
     </row>
     <row r="459">
@@ -9259,10 +9259,10 @@
         </is>
       </c>
       <c r="E459" s="2" t="n">
-        <v>256.2621744766313</v>
+        <v>1146322693.194041</v>
       </c>
       <c r="F459" s="2" t="n">
-        <v>752.7900524138739</v>
+        <v>671785677.7662393</v>
       </c>
     </row>
     <row r="460">
@@ -9285,10 +9285,10 @@
         </is>
       </c>
       <c r="E460" s="2" t="n">
-        <v>250.9407981737039</v>
+        <v>1365840459.634722</v>
       </c>
       <c r="F460" s="2" t="n">
-        <v>648.2550669219886</v>
+        <v>689509125.9290614</v>
       </c>
     </row>
     <row r="461">
@@ -9311,10 +9311,10 @@
         </is>
       </c>
       <c r="E461" s="2" t="n">
-        <v>251.3155506939212</v>
+        <v>1664387234.452982</v>
       </c>
       <c r="F461" s="2" t="n">
-        <v>571.1654566467648</v>
+        <v>724091187.8307656</v>
       </c>
     </row>
     <row r="462">
@@ -9337,10 +9337,10 @@
         </is>
       </c>
       <c r="E462" s="2" t="n">
-        <v>256</v>
+        <v>2062914813.819247</v>
       </c>
       <c r="F462" s="2" t="n">
-        <v>512</v>
+        <v>773639291.8273966</v>
       </c>
     </row>
     <row r="463">
@@ -9363,10 +9363,10 @@
         </is>
       </c>
       <c r="E463" s="2" t="n">
-        <v>256</v>
+        <v>2062914813.819247</v>
       </c>
       <c r="F463" s="2" t="n">
-        <v>512</v>
+        <v>773639291.8273966</v>
       </c>
     </row>
     <row r="464">
@@ -9389,10 +9389,10 @@
         </is>
       </c>
       <c r="E464" s="2" t="n">
-        <v>108.0017740826299</v>
+        <v>1322763995.548106</v>
       </c>
       <c r="F464" s="2" t="n">
-        <v>202.144749121721</v>
+        <v>444225268.8096915</v>
       </c>
     </row>
     <row r="465">
@@ -9415,10 +9415,10 @@
         </is>
       </c>
       <c r="E465" s="2" t="n">
-        <v>69.34180216208662</v>
+        <v>1290793432.415621</v>
       </c>
       <c r="F465" s="2" t="n">
-        <v>126.4547741947134</v>
+        <v>404155283.8286686</v>
       </c>
     </row>
     <row r="466">
@@ -9441,10 +9441,10 @@
         </is>
       </c>
       <c r="E466" s="2" t="n">
-        <v>51.55185107897695</v>
+        <v>1458532239.463664</v>
       </c>
       <c r="F466" s="2" t="n">
-        <v>92.28122413600921</v>
+        <v>428942041.0554438</v>
       </c>
     </row>
     <row r="467">
@@ -9467,10 +9467,10 @@
         </is>
       </c>
       <c r="E467" s="2" t="n">
-        <v>41.33264956510073</v>
+        <v>1777359016.136873</v>
       </c>
       <c r="F467" s="2" t="n">
-        <v>72.81919686751712</v>
+        <v>492270020.9630268</v>
       </c>
     </row>
     <row r="468">
@@ -9493,10 +9493,10 @@
         </is>
       </c>
       <c r="E468" s="2" t="n">
-        <v>34.70516056072824</v>
+        <v>2268224934.171155</v>
       </c>
       <c r="F468" s="2" t="n">
-        <v>60.25244476556771</v>
+        <v>592385491.2388648</v>
       </c>
     </row>
     <row r="469">
@@ -9519,10 +9519,10 @@
         </is>
       </c>
       <c r="E469" s="2" t="n">
-        <v>30.06316735633945</v>
+        <v>2986324129.519697</v>
       </c>
       <c r="F469" s="2" t="n">
-        <v>51.46869197815998</v>
+        <v>735944573.9449331</v>
       </c>
     </row>
     <row r="470">
@@ -9545,10 +9545,10 @@
         </is>
       </c>
       <c r="E470" s="2" t="n">
-        <v>26.63402053600463</v>
+        <v>4021139000.028463</v>
       </c>
       <c r="F470" s="2" t="n">
-        <v>44.98373942487196</v>
+        <v>935469791.32731</v>
       </c>
     </row>
     <row r="471">
@@ -9571,10 +9571,10 @@
         </is>
       </c>
       <c r="E471" s="2" t="n">
-        <v>24</v>
+        <v>5507236713.11497</v>
       </c>
       <c r="F471" s="2" t="n">
-        <v>40</v>
+        <v>1209780111.624298</v>
       </c>
     </row>
     <row r="472">
@@ -9597,10 +9597,10 @@
         </is>
       </c>
       <c r="E472" s="2" t="n">
-        <v>24</v>
+        <v>5507236713.11497</v>
       </c>
       <c r="F472" s="2" t="n">
-        <v>40</v>
+        <v>1209780111.624298</v>
       </c>
     </row>
     <row r="473">
@@ -9623,10 +9623,10 @@
         </is>
       </c>
       <c r="E473" s="2" t="n">
-        <v>4.61404717992635</v>
+        <v>2443821882.72761</v>
       </c>
       <c r="F473" s="2" t="n">
-        <v>6.793413216515661</v>
+        <v>434271245.7290222</v>
       </c>
     </row>
     <row r="474">
@@ -9649,10 +9649,10 @@
         </is>
       </c>
       <c r="E474" s="2" t="n">
-        <v>2.678561477405338</v>
+        <v>3274569052.8913</v>
       </c>
       <c r="F474" s="2" t="n">
-        <v>3.713200530214782</v>
+        <v>501704550.2673191</v>
       </c>
     </row>
     <row r="475">
@@ -9675,10 +9675,10 @@
         </is>
       </c>
       <c r="E475" s="2" t="n">
-        <v>1.949561306027979</v>
+        <v>5501162163.562591</v>
       </c>
       <c r="F475" s="2" t="n">
-        <v>2.555426031861377</v>
+        <v>729775945.328842</v>
       </c>
     </row>
     <row r="476">
@@ -9701,10 +9701,10 @@
         </is>
       </c>
       <c r="E476" s="2" t="n">
-        <v>1.570142448033869</v>
+        <v>10226372819.29995</v>
       </c>
       <c r="F476" s="2" t="n">
-        <v>1.948384751261965</v>
+        <v>1176054762.613422</v>
       </c>
     </row>
     <row r="477">
@@ -9727,10 +9727,10 @@
         </is>
       </c>
       <c r="E477" s="2" t="n">
-        <v>1.339695023226408</v>
+        <v>20139724582.75352</v>
       </c>
       <c r="F477" s="2" t="n">
-        <v>1.574619863309849</v>
+        <v>2008885305.812436</v>
       </c>
     </row>
     <row r="478">
@@ -9753,10 +9753,10 @@
         </is>
       </c>
       <c r="E478" s="2" t="n">
-        <v>1.186570383980938</v>
+        <v>41172392447.82437</v>
       </c>
       <c r="F478" s="2" t="n">
-        <v>1.321337309095369</v>
+        <v>3563031876.379255</v>
       </c>
     </row>
     <row r="479">
@@ -9779,10 +9779,10 @@
         </is>
       </c>
       <c r="E479" s="2" t="n">
-        <v>1.078807368523075</v>
+        <v>86401547228.57439</v>
       </c>
       <c r="F479" s="2" t="n">
-        <v>1.138367375927505</v>
+        <v>6488062791.278718</v>
       </c>
     </row>
     <row r="480">
@@ -9805,10 +9805,10 @@
         </is>
       </c>
       <c r="E480" s="2" t="n">
-        <v>1</v>
+        <v>184859865072.0317</v>
       </c>
       <c r="F480" s="2" t="n">
-        <v>1</v>
+        <v>12046453173.55365</v>
       </c>
     </row>
     <row r="481">

</xml_diff>

<commit_message>
balance: soften stage14 elite salvo cliff with reproducible local attack shape
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/monGroup.xlsx
+++ b/space-battleship/config_excel/monGroup.xlsx
@@ -1013,7 +1013,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2280"/>
+  <dimension ref="A1:G2280"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.888888888888889" defaultRowHeight="14.4"/>
   <cols>
     <col width="50.7777777777778" customWidth="1" style="3" min="2" max="2"/>
@@ -1051,6 +1051,11 @@
           <t>lifeMultiplier</t>
         </is>
       </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>authorAtkScale</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1083,6 +1088,11 @@
           <t>本波生命及护盾倍率；空白为1，不改变资源和跨关插值锚点</t>
         </is>
       </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Author-only attack shape; not projected. Tail multiplier includes this factor.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1111,6 +1121,11 @@
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>float</t>
         </is>
@@ -8323,10 +8338,13 @@
         </is>
       </c>
       <c r="E423" s="2" t="n">
-        <v>5014.690810225376</v>
+        <v>626.8363512781719</v>
       </c>
       <c r="F423" s="2" t="n">
         <v>16831.09401287439</v>
+      </c>
+      <c r="G423" s="2" t="n">
+        <v>0.125</v>
       </c>
     </row>
     <row r="424">
@@ -8349,10 +8367,13 @@
         </is>
       </c>
       <c r="E424" s="2" t="n">
-        <v>9949.311847531131</v>
+        <v>1243.663980941391</v>
       </c>
       <c r="F424" s="2" t="n">
         <v>39119.06587803794</v>
+      </c>
+      <c r="G424" s="2" t="n">
+        <v>0.125</v>
       </c>
     </row>
     <row r="425">
@@ -8375,10 +8396,13 @@
         </is>
       </c>
       <c r="E425" s="2" t="n">
-        <v>20200.74957401707</v>
+        <v>2525.093696752134</v>
       </c>
       <c r="F425" s="2" t="n">
         <v>93168.83992096882</v>
+      </c>
+      <c r="G425" s="2" t="n">
+        <v>0.125</v>
       </c>
     </row>
     <row r="426">
@@ -8401,10 +8425,13 @@
         </is>
       </c>
       <c r="E426" s="2" t="n">
-        <v>41733.72776251628</v>
+        <v>5216.715970314535</v>
       </c>
       <c r="F426" s="2" t="n">
         <v>225982.3092077873</v>
+      </c>
+      <c r="G426" s="2" t="n">
+        <v>0.125</v>
       </c>
     </row>
     <row r="427">
@@ -8427,7 +8454,7 @@
         </is>
       </c>
       <c r="E427" s="2" t="n">
-        <v>41733.72776251628</v>
+        <v>5216.715970314535</v>
       </c>
       <c r="F427" s="2" t="n">
         <v>225982.3092077873</v>
@@ -8453,7 +8480,7 @@
         </is>
       </c>
       <c r="E428" s="2" t="n">
-        <v>30633.82530427614</v>
+        <v>4965.894545606789</v>
       </c>
       <c r="F428" s="2" t="n">
         <v>161169.1054540616</v>
@@ -8479,7 +8506,7 @@
         </is>
       </c>
       <c r="E429" s="2" t="n">
-        <v>34220.67683617786</v>
+        <v>7194.011119774445</v>
       </c>
       <c r="F429" s="2" t="n">
         <v>182124.9354110597</v>
@@ -8505,7 +8532,7 @@
         </is>
       </c>
       <c r="E430" s="2" t="n">
-        <v>44265.04021406242</v>
+        <v>12067.84216004341</v>
       </c>
       <c r="F430" s="2" t="n">
         <v>240083.5348901573</v>
@@ -8531,7 +8558,7 @@
         </is>
       </c>
       <c r="E431" s="2" t="n">
-        <v>61749.43289317845</v>
+        <v>21831.72136659507</v>
       </c>
       <c r="F431" s="2" t="n">
         <v>342223.4492537044</v>
@@ -8557,7 +8584,7 @@
         </is>
       </c>
       <c r="E432" s="2" t="n">
-        <v>90210.46343745851</v>
+        <v>41361.67985575831</v>
       </c>
       <c r="F432" s="2" t="n">
         <v>511509.1446189569</v>
@@ -8583,7 +8610,7 @@
         </is>
       </c>
       <c r="E433" s="2" t="n">
-        <v>135962.9938345435</v>
+        <v>80844.07982255514</v>
       </c>
       <c r="F433" s="2" t="n">
         <v>789290.1987877744</v>
@@ -8609,7 +8636,7 @@
         </is>
       </c>
       <c r="E434" s="2" t="n">
-        <v>209578.07318589</v>
+        <v>161606.7866177086</v>
       </c>
       <c r="F434" s="2" t="n">
         <v>1246131.811672945</v>

</xml_diff>

<commit_message>
fix: validate mixed fleet geometry and isolate hyperspace reward references
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/monGroup.xlsx
+++ b/space-battleship/config_excel/monGroup.xlsx
@@ -1061,7 +1061,7 @@
           <t>rewardBinding</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>formation_positions</t>
         </is>
@@ -1108,7 +1108,7 @@
           <t>Optional existing candidate reward contract</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Optional explicit existing formation contract</t>
         </is>
@@ -1155,7 +1155,7 @@
           <t>json</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>json</t>
         </is>
@@ -45901,9 +45901,9 @@
           <t>{"status":"BOUND","referenceGroupId":34146,"levelId":14,"resRatio":561545.6675019113,"jewelRatio":3.6}</t>
         </is>
       </c>
-      <c r="I2281" t="inlineStr">
-        <is>
-          <t>[null,[106,220],[226,220],[346,220],null,null,[466,220],[286,110],[106,330],null,null,[226,330],[346,330],[466,330],null]</t>
+      <c r="I2281" s="2" t="inlineStr">
+        <is>
+          <t>[null,[106,270],[226,270],[346,270],null,null,[466,270],[286,110],[106,350],null,null,[226,350],[346,350],[466,350],null]</t>
         </is>
       </c>
     </row>
@@ -45940,9 +45940,9 @@
           <t>{"status":"BOUND","referenceGroupId":34147,"levelId":14,"resRatio":561545.6675019113,"jewelRatio":3.6}</t>
         </is>
       </c>
-      <c r="I2282" t="inlineStr">
-        <is>
-          <t>[null,[106,220],[226,220],[346,220],null,null,[466,220],[286,110],[106,330],null,null,[226,330],[346,330],[466,330],null]</t>
+      <c r="I2282" s="2" t="inlineStr">
+        <is>
+          <t>[null,[106,270],[226,270],[346,270],null,null,[466,270],[286,110],[106,350],null,null,[226,350],[346,350],[466,350],null]</t>
         </is>
       </c>
     </row>
@@ -45979,9 +45979,9 @@
           <t>{"status":"BOUND","referenceGroupId":34148,"levelId":14,"resRatio":561545.6675019113,"jewelRatio":3.6}</t>
         </is>
       </c>
-      <c r="I2283" t="inlineStr">
-        <is>
-          <t>[null,[106,220],[226,220],[346,220],null,null,[466,220],[286,110],[106,330],null,null,[226,330],[346,330],[466,330],null]</t>
+      <c r="I2283" s="2" t="inlineStr">
+        <is>
+          <t>[null,[106,270],[226,270],[346,270],null,null,[466,270],[286,110],[106,350],null,null,[226,350],[346,350],[466,350],null]</t>
         </is>
       </c>
     </row>
@@ -46018,9 +46018,9 @@
           <t>{"status":"BOUND","referenceGroupId":34149,"levelId":14,"resRatio":561545.6675019113,"jewelRatio":3.6}</t>
         </is>
       </c>
-      <c r="I2284" t="inlineStr">
-        <is>
-          <t>[null,null,null,null,null,null,[126,250],[286,100],[446,250],null,null,null,null,null,null]</t>
+      <c r="I2284" s="2" t="inlineStr">
+        <is>
+          <t>[null,null,null,null,null,null,[126,350],[286,160],[446,350],null,null,null,null,null,null]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
balance: connect stage15 patrols mixed escorts and boss pressure
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/monGroup.xlsx
+++ b/space-battleship/config_excel/monGroup.xlsx
@@ -8600,7 +8600,7 @@
       </c>
       <c r="B432" s="2" t="inlineStr">
         <is>
-          <t>第15关第6战点</t>
+          <t>第15关第6战点：主舰与混合护卫</t>
         </is>
       </c>
       <c r="C432" s="2" t="inlineStr">
@@ -8618,6 +8618,11 @@
       </c>
       <c r="F432" s="2" t="n">
         <v>511509.1446189569</v>
+      </c>
+      <c r="I432" s="2" t="inlineStr">
+        <is>
+          <t>[null,null,null,null,null,[126,350],null,[286,110],null,[446,350],null,null,null,null,null]</t>
+        </is>
       </c>
     </row>
     <row r="433">
@@ -8626,7 +8631,7 @@
       </c>
       <c r="B433" s="2" t="inlineStr">
         <is>
-          <t>第15关第7战点</t>
+          <t>第15关第7战点：主舰与混合护卫</t>
         </is>
       </c>
       <c r="C433" s="2" t="inlineStr">
@@ -8644,6 +8649,11 @@
       </c>
       <c r="F433" s="2" t="n">
         <v>789290.1987877744</v>
+      </c>
+      <c r="I433" s="2" t="inlineStr">
+        <is>
+          <t>[null,null,null,null,null,[126,350],null,[286,110],null,[446,350],null,null,null,null,null]</t>
+        </is>
       </c>
     </row>
     <row r="434">
@@ -8652,7 +8662,7 @@
       </c>
       <c r="B434" s="2" t="inlineStr">
         <is>
-          <t>第15关第8战点</t>
+          <t>第15关第8战点：主舰与混合护卫</t>
         </is>
       </c>
       <c r="C434" s="2" t="inlineStr">
@@ -8670,6 +8680,11 @@
       </c>
       <c r="F434" s="2" t="n">
         <v>1246131.811672945</v>
+      </c>
+      <c r="I434" s="2" t="inlineStr">
+        <is>
+          <t>[null,null,null,null,null,[126,350],null,[286,110],null,[446,350],null,null,null,null,null]</t>
+        </is>
       </c>
     </row>
     <row r="435">

</xml_diff>

<commit_message>
balance: connect mid-stage weapon budgets and shorten overlong life gates
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/monGroup.xlsx
+++ b/space-battleship/config_excel/monGroup.xlsx
@@ -8513,7 +8513,7 @@
         <v>4965.894545606789</v>
       </c>
       <c r="F428" s="2" t="n">
-        <v>161169.1054540616</v>
+        <v>124278.3695762839</v>
       </c>
     </row>
     <row r="429">
@@ -8539,7 +8539,7 @@
         <v>7194.011119774445</v>
       </c>
       <c r="F429" s="2" t="n">
-        <v>182124.9354110597</v>
+        <v>108292.1345051216</v>
       </c>
     </row>
     <row r="430">
@@ -8565,7 +8565,7 @@
         <v>12067.84216004341</v>
       </c>
       <c r="F430" s="2" t="n">
-        <v>240083.5348901573</v>
+        <v>110078.786100572</v>
       </c>
     </row>
     <row r="431">
@@ -8591,7 +8591,7 @@
         <v>21831.72136659507</v>
       </c>
       <c r="F431" s="2" t="n">
-        <v>342223.4492537044</v>
+        <v>120994.2608241724</v>
       </c>
     </row>
     <row r="432">
@@ -8617,7 +8617,7 @@
         <v>41361.67985575831</v>
       </c>
       <c r="F432" s="2" t="n">
-        <v>511509.1446189569</v>
+        <v>139451.169383991</v>
       </c>
       <c r="I432" s="2" t="inlineStr">
         <is>
@@ -8648,7 +8648,7 @@
         <v>80844.07982255514</v>
       </c>
       <c r="F433" s="2" t="n">
-        <v>789290.1987877744</v>
+        <v>165927.8246888828</v>
       </c>
       <c r="I433" s="2" t="inlineStr">
         <is>
@@ -8679,7 +8679,7 @@
         <v>161606.7866177086</v>
       </c>
       <c r="F434" s="2" t="n">
-        <v>1246131.811672945</v>
+        <v>202004.1279607996</v>
       </c>
       <c r="I434" s="2" t="inlineStr">
         <is>
@@ -8710,7 +8710,7 @@
         <v>328581.7839565452</v>
       </c>
       <c r="F435" s="2" t="n">
-        <v>2001627.546075745</v>
+        <v>250203.4432594681</v>
       </c>
     </row>
     <row r="436">
@@ -8736,7 +8736,7 @@
         <v>328581.7839565452</v>
       </c>
       <c r="F436" s="2" t="n">
-        <v>2001627.546075745</v>
+        <v>250203.4432594681</v>
       </c>
     </row>
     <row r="437">
@@ -8762,7 +8762,7 @@
         <v>156201.3328787747</v>
       </c>
       <c r="F437" s="2" t="n">
-        <v>865988.9475631206</v>
+        <v>140381.0901363067</v>
       </c>
     </row>
     <row r="438">
@@ -8788,7 +8788,7 @@
         <v>113005.4264854566</v>
       </c>
       <c r="F438" s="2" t="n">
-        <v>593637.9975864481</v>
+        <v>124797.0160322093</v>
       </c>
     </row>
     <row r="439">
@@ -8814,7 +8814,7 @@
         <v>94667.03309593175</v>
       </c>
       <c r="F439" s="2" t="n">
-        <v>474718.7489707069</v>
+        <v>129421.1166484333</v>
       </c>
     </row>
     <row r="440">
@@ -8840,7 +8840,7 @@
         <v>85525.9833469116</v>
       </c>
       <c r="F440" s="2" t="n">
-        <v>410492.7572049934</v>
+        <v>145131.1061238069</v>
       </c>
     </row>
     <row r="441">
@@ -8866,7 +8866,7 @@
         <v>80918.75950932644</v>
       </c>
       <c r="F441" s="2" t="n">
-        <v>372195.2821115094</v>
+        <v>170652.2892789786</v>
       </c>
     </row>
     <row r="442">
@@ -8892,7 +8892,7 @@
         <v>78984.19951064256</v>
       </c>
       <c r="F442" s="2" t="n">
-        <v>348398.1965499314</v>
+        <v>207158.8070956474</v>
       </c>
     </row>
     <row r="443">
@@ -8918,7 +8918,7 @@
         <v>78848.33825134594</v>
       </c>
       <c r="F443" s="2" t="n">
-        <v>333675.9443618188</v>
+        <v>257299.3267865074</v>
       </c>
     </row>
     <row r="444">
@@ -9695,10 +9695,10 @@
         </is>
       </c>
       <c r="E473" s="2" t="n">
-        <v>6215058.952198651</v>
+        <v>5226220.793494353</v>
       </c>
       <c r="F473" s="2" t="n">
-        <v>6193676.665663028</v>
+        <v>4379590.770767212</v>
       </c>
     </row>
     <row r="474">
@@ -9721,10 +9721,10 @@
         </is>
       </c>
       <c r="E474" s="2" t="n">
-        <v>6618612.912963974</v>
+        <v>4680066.072805675</v>
       </c>
       <c r="F474" s="2" t="n">
-        <v>6210278.03366101</v>
+        <v>3105139.016830505</v>
       </c>
     </row>
     <row r="475">
@@ -9747,10 +9747,10 @@
         </is>
       </c>
       <c r="E475" s="2" t="n">
-        <v>8836990.792871492</v>
+        <v>5254506.163048157</v>
       </c>
       <c r="F475" s="2" t="n">
-        <v>7840217.249174365</v>
+        <v>2771935.391433466</v>
       </c>
     </row>
     <row r="476">
@@ -9773,10 +9773,10 @@
         </is>
       </c>
       <c r="E476" s="2" t="n">
-        <v>13055956.75314689</v>
+        <v>6527978.376573443</v>
       </c>
       <c r="F476" s="2" t="n">
-        <v>10965833.47744089</v>
+        <v>2741458.369360223</v>
       </c>
     </row>
     <row r="477">
@@ -9799,10 +9799,10 @@
         </is>
       </c>
       <c r="E477" s="2" t="n">
-        <v>20435145.50667887</v>
+        <v>8591920.300877156</v>
       </c>
       <c r="F477" s="2" t="n">
-        <v>16257164.20991712</v>
+        <v>2873887.763923908</v>
       </c>
     </row>
     <row r="478">
@@ -9825,10 +9825,10 @@
         </is>
       </c>
       <c r="E478" s="2" t="n">
-        <v>33202244.01616731</v>
+        <v>11738765.94722118</v>
       </c>
       <c r="F478" s="2" t="n">
-        <v>25025623.52386186</v>
+        <v>3128202.940482732</v>
       </c>
     </row>
     <row r="479">
@@ -9851,10 +9851,10 @@
         </is>
       </c>
       <c r="E479" s="2" t="n">
-        <v>55375795.60839046</v>
+        <v>16463322.53410859</v>
       </c>
       <c r="F479" s="2" t="n">
-        <v>39550847.33806602</v>
+        <v>3495834.04430255</v>
       </c>
     </row>
     <row r="480">
@@ -9877,10 +9877,10 @@
         </is>
       </c>
       <c r="E480" s="2" t="n">
-        <v>94162551.30680417</v>
+        <v>23540637.82670104</v>
       </c>
       <c r="F480" s="2" t="n">
-        <v>63734633.61066098</v>
+        <v>3983414.600666311</v>
       </c>
     </row>
     <row r="481">

</xml_diff>

<commit_message>
balance: shorten measured stage17 shield-life progression
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/monGroup.xlsx
+++ b/space-battleship/config_excel/monGroup.xlsx
@@ -8996,7 +8996,7 @@
         <v>73669.77095405322</v>
       </c>
       <c r="F446" s="2" t="n">
-        <v>286442.2534907912</v>
+        <v>220877.1720938719</v>
       </c>
     </row>
     <row r="447">
@@ -9022,7 +9022,7 @@
         <v>103165.5186192836</v>
       </c>
       <c r="F447" s="2" t="n">
-        <v>399842.0949667247</v>
+        <v>237747.5321060114</v>
       </c>
     </row>
     <row r="448">
@@ -9048,7 +9048,7 @@
         <v>167287.9720057605</v>
       </c>
       <c r="F448" s="2" t="n">
-        <v>651096.4051923612</v>
+        <v>298529.0180387111</v>
       </c>
     </row>
     <row r="449">
@@ -9074,7 +9074,7 @@
         <v>292546.3669700471</v>
       </c>
       <c r="F449" s="2" t="n">
-        <v>1146453.652119232</v>
+        <v>405332.5758647961</v>
       </c>
     </row>
     <row r="450">
@@ -9100,7 +9100,7 @@
         <v>535767.7056266126</v>
       </c>
       <c r="F450" s="2" t="n">
-        <v>2116722.652082936</v>
+        <v>577075.6050010385</v>
       </c>
     </row>
     <row r="451">
@@ -9126,7 +9126,7 @@
         <v>1012274.320400161</v>
       </c>
       <c r="F451" s="2" t="n">
-        <v>4034698.456719378</v>
+        <v>848190.8672212551</v>
       </c>
     </row>
     <row r="452">
@@ -9152,7 +9152,7 @@
         <v>1956055.740709604</v>
       </c>
       <c r="F452" s="2" t="n">
-        <v>7868685.22739314</v>
+        <v>1275552.780747687</v>
       </c>
     </row>
     <row r="453">
@@ -9178,7 +9178,7 @@
         <v>3844472.413788395</v>
       </c>
       <c r="F453" s="2" t="n">
-        <v>15612961.03293186</v>
+        <v>1951620.129116483</v>
       </c>
     </row>
     <row r="454">
@@ -9204,7 +9204,7 @@
         <v>3844472.413788395</v>
       </c>
       <c r="F454" s="2" t="n">
-        <v>15612961.03293186</v>
+        <v>1951620.129116483</v>
       </c>
     </row>
     <row r="455">
@@ -9230,7 +9230,7 @@
         <v>2315021.608712353</v>
       </c>
       <c r="F455" s="2" t="n">
-        <v>7846259.264164844</v>
+        <v>1271917.421226987</v>
       </c>
     </row>
     <row r="456">
@@ -9256,7 +9256,7 @@
         <v>2121517.704119835</v>
       </c>
       <c r="F456" s="2" t="n">
-        <v>6247701.835633707</v>
+        <v>1313417.51928961</v>
       </c>
     </row>
     <row r="457">
@@ -9282,7 +9282,7 @@
         <v>2251247.149590914</v>
       </c>
       <c r="F457" s="2" t="n">
-        <v>5803410.439569656</v>
+        <v>1582165.990045249</v>
       </c>
     </row>
     <row r="458">
@@ -9308,7 +9308,7 @@
         <v>2576318.391251266</v>
       </c>
       <c r="F458" s="2" t="n">
-        <v>5829089.176058053</v>
+        <v>2060894.242265878</v>
       </c>
     </row>
     <row r="459">
@@ -9334,7 +9334,7 @@
         <v>3087647.559750664</v>
       </c>
       <c r="F459" s="2" t="n">
-        <v>6139236.485866043</v>
+        <v>2814852.3398644</v>
       </c>
     </row>
     <row r="460">
@@ -9360,7 +9360,7 @@
         <v>3817647.050025986</v>
       </c>
       <c r="F460" s="2" t="n">
-        <v>6675252.465644834</v>
+        <v>3969128.863292147</v>
       </c>
     </row>
     <row r="461">
@@ -9386,7 +9386,7 @@
         <v>4827531.833205524</v>
       </c>
       <c r="F461" s="2" t="n">
-        <v>7426171.837749272</v>
+        <v>5726361.299758255</v>
       </c>
     </row>
     <row r="462">

</xml_diff>

<commit_message>
balance: remove stage18 guard damage wall and taper late-stage curves
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/monGroup.xlsx
+++ b/space-battleship/config_excel/monGroup.xlsx
@@ -9227,10 +9227,10 @@
         </is>
       </c>
       <c r="E455" s="2" t="n">
-        <v>2315021.608712353</v>
+        <v>1946693.372001105</v>
       </c>
       <c r="F455" s="2" t="n">
-        <v>1271917.421226987</v>
+        <v>980782.4080206057</v>
       </c>
     </row>
     <row r="456">
@@ -9253,10 +9253,10 @@
         </is>
       </c>
       <c r="E456" s="2" t="n">
-        <v>2121517.704119835</v>
+        <v>1500139.55499045</v>
       </c>
       <c r="F456" s="2" t="n">
-        <v>1313417.51928961</v>
+        <v>780962.7294542136</v>
       </c>
     </row>
     <row r="457">
@@ -9279,10 +9279,10 @@
         </is>
       </c>
       <c r="E457" s="2" t="n">
-        <v>2251247.149590914</v>
+        <v>1338599.563961555</v>
       </c>
       <c r="F457" s="2" t="n">
-        <v>1582165.990045249</v>
+        <v>725426.3049462072</v>
       </c>
     </row>
     <row r="458">
@@ -9305,10 +9305,10 @@
         </is>
       </c>
       <c r="E458" s="2" t="n">
-        <v>2576318.391251266</v>
+        <v>1288159.195625633</v>
       </c>
       <c r="F458" s="2" t="n">
-        <v>2060894.242265878</v>
+        <v>728636.1470072566</v>
       </c>
     </row>
     <row r="459">
@@ -9331,10 +9331,10 @@
         </is>
       </c>
       <c r="E459" s="2" t="n">
-        <v>3087647.559750664</v>
+        <v>1298195.882280606</v>
       </c>
       <c r="F459" s="2" t="n">
-        <v>2814852.3398644</v>
+        <v>767404.5607332553</v>
       </c>
     </row>
     <row r="460">
@@ -9357,10 +9357,10 @@
         </is>
       </c>
       <c r="E460" s="2" t="n">
-        <v>3817647.050025986</v>
+        <v>1349742.058625097</v>
       </c>
       <c r="F460" s="2" t="n">
-        <v>3969128.863292147</v>
+        <v>834406.5582056041</v>
       </c>
     </row>
     <row r="461">
@@ -9383,10 +9383,10 @@
         </is>
       </c>
       <c r="E461" s="2" t="n">
-        <v>4827531.833205524</v>
+        <v>1435233.800987535</v>
       </c>
       <c r="F461" s="2" t="n">
-        <v>5726361.299758255</v>
+        <v>928271.479718659</v>
       </c>
     </row>
     <row r="462">
@@ -9409,10 +9409,10 @@
         </is>
       </c>
       <c r="E462" s="2" t="n">
-        <v>6209076.829557999</v>
+        <v>1552269.2073895</v>
       </c>
       <c r="F462" s="2" t="n">
-        <v>8405321.038996274</v>
+        <v>1050665.129874534</v>
       </c>
     </row>
     <row r="463">
@@ -9435,10 +9435,10 @@
         </is>
       </c>
       <c r="E463" s="2" t="n">
-        <v>6209076.829557999</v>
+        <v>1552269.2073895</v>
       </c>
       <c r="F463" s="2" t="n">
-        <v>8405321.038996274</v>
+        <v>1050665.129874534</v>
       </c>
     </row>
     <row r="464">
@@ -9461,10 +9461,10 @@
         </is>
       </c>
       <c r="E464" s="2" t="n">
-        <v>4011919.490687458</v>
+        <v>1002979.872671865</v>
       </c>
       <c r="F464" s="2" t="n">
-        <v>5082542.991611379</v>
+        <v>635317.8739514224</v>
       </c>
     </row>
     <row r="465">
@@ -9487,10 +9487,10 @@
         </is>
       </c>
       <c r="E465" s="2" t="n">
-        <v>3945033.502259679</v>
+        <v>986258.3755649199</v>
       </c>
       <c r="F465" s="2" t="n">
-        <v>4869541.573952398</v>
+        <v>608692.6967440498</v>
       </c>
     </row>
     <row r="466">
@@ -9513,10 +9513,10 @@
         </is>
       </c>
       <c r="E466" s="2" t="n">
-        <v>4491941.447956745</v>
+        <v>1122985.361989187</v>
       </c>
       <c r="F466" s="2" t="n">
-        <v>5442525.165719046</v>
+        <v>680315.6457148808</v>
       </c>
     </row>
     <row r="467">
@@ -9539,10 +9539,10 @@
         </is>
       </c>
       <c r="E467" s="2" t="n">
-        <v>5515911.884082857</v>
+        <v>1378977.971020714</v>
       </c>
       <c r="F467" s="2" t="n">
-        <v>6577596.601022505</v>
+        <v>822199.5751278132</v>
       </c>
     </row>
     <row r="468">
@@ -9565,10 +9565,10 @@
         </is>
       </c>
       <c r="E468" s="2" t="n">
-        <v>7093366.232010648</v>
+        <v>1773341.558002662</v>
       </c>
       <c r="F468" s="2" t="n">
-        <v>8335473.495320463</v>
+        <v>1041934.186915058</v>
       </c>
     </row>
     <row r="469">
@@ -9591,10 +9591,10 @@
         </is>
       </c>
       <c r="E469" s="2" t="n">
-        <v>9410816.624785341</v>
+        <v>2352704.156196336</v>
       </c>
       <c r="F469" s="2" t="n">
-        <v>10905183.66204279</v>
+        <v>1363147.957755349</v>
       </c>
     </row>
     <row r="470">
@@ -9617,10 +9617,10 @@
         </is>
       </c>
       <c r="E470" s="2" t="n">
-        <v>12769196.14545644</v>
+        <v>3192299.036364111</v>
       </c>
       <c r="F470" s="2" t="n">
-        <v>14597539.50090802</v>
+        <v>1824692.437613503</v>
       </c>
     </row>
     <row r="471">
@@ -9643,10 +9643,10 @@
         </is>
       </c>
       <c r="E471" s="2" t="n">
-        <v>17622694.8409208</v>
+        <v>4405673.7102302</v>
       </c>
       <c r="F471" s="2" t="n">
-        <v>19880090.03811214</v>
+        <v>2485011.254764018</v>
       </c>
     </row>
     <row r="472">
@@ -9669,10 +9669,10 @@
         </is>
       </c>
       <c r="E472" s="2" t="n">
-        <v>17622694.8409208</v>
+        <v>4405673.7102302</v>
       </c>
       <c r="F472" s="2" t="n">
-        <v>19880090.03811214</v>
+        <v>2485011.254764018</v>
       </c>
     </row>
     <row r="473">
@@ -9695,10 +9695,10 @@
         </is>
       </c>
       <c r="E473" s="2" t="n">
-        <v>5226220.793494353</v>
+        <v>1306555.198373588</v>
       </c>
       <c r="F473" s="2" t="n">
-        <v>4379590.770767212</v>
+        <v>547448.8463459016</v>
       </c>
     </row>
     <row r="474">
@@ -9721,10 +9721,10 @@
         </is>
       </c>
       <c r="E474" s="2" t="n">
-        <v>4680066.072805675</v>
+        <v>1170016.518201419</v>
       </c>
       <c r="F474" s="2" t="n">
-        <v>3105139.016830505</v>
+        <v>388142.3771038132</v>
       </c>
     </row>
     <row r="475">
@@ -9747,10 +9747,10 @@
         </is>
       </c>
       <c r="E475" s="2" t="n">
-        <v>5254506.163048157</v>
+        <v>1313626.540762039</v>
       </c>
       <c r="F475" s="2" t="n">
-        <v>2771935.391433466</v>
+        <v>346491.9239291833</v>
       </c>
     </row>
     <row r="476">
@@ -9773,10 +9773,10 @@
         </is>
       </c>
       <c r="E476" s="2" t="n">
-        <v>6527978.376573443</v>
+        <v>1631994.594143361</v>
       </c>
       <c r="F476" s="2" t="n">
-        <v>2741458.369360223</v>
+        <v>342682.2961700279</v>
       </c>
     </row>
     <row r="477">
@@ -9799,10 +9799,10 @@
         </is>
       </c>
       <c r="E477" s="2" t="n">
-        <v>8591920.300877156</v>
+        <v>2147980.075219289</v>
       </c>
       <c r="F477" s="2" t="n">
-        <v>2873887.763923908</v>
+        <v>359235.9704904885</v>
       </c>
     </row>
     <row r="478">
@@ -9825,10 +9825,10 @@
         </is>
       </c>
       <c r="E478" s="2" t="n">
-        <v>11738765.94722118</v>
+        <v>2934691.486805297</v>
       </c>
       <c r="F478" s="2" t="n">
-        <v>3128202.940482732</v>
+        <v>391025.3675603415</v>
       </c>
     </row>
     <row r="479">
@@ -9851,10 +9851,10 @@
         </is>
       </c>
       <c r="E479" s="2" t="n">
-        <v>16463322.53410859</v>
+        <v>4115830.633527148</v>
       </c>
       <c r="F479" s="2" t="n">
-        <v>3495834.04430255</v>
+        <v>436979.2555378187</v>
       </c>
     </row>
     <row r="480">
@@ -9877,10 +9877,10 @@
         </is>
       </c>
       <c r="E480" s="2" t="n">
-        <v>23540637.82670104</v>
+        <v>5885159.45667526</v>
       </c>
       <c r="F480" s="2" t="n">
-        <v>3983414.600666311</v>
+        <v>497926.8250832889</v>
       </c>
     </row>
     <row r="481">

</xml_diff>

<commit_message>
balance: reduce stage17 growth budget and reconnect stage18 entry
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/monGroup.xlsx
+++ b/space-battleship/config_excel/monGroup.xlsx
@@ -8993,10 +8993,10 @@
         </is>
       </c>
       <c r="E446" s="2" t="n">
-        <v>73669.77095405322</v>
+        <v>67555.47782682885</v>
       </c>
       <c r="F446" s="2" t="n">
-        <v>220877.1720938719</v>
+        <v>185734.8222251147</v>
       </c>
     </row>
     <row r="447">
@@ -9019,10 +9019,10 @@
         </is>
       </c>
       <c r="E447" s="2" t="n">
-        <v>103165.5186192836</v>
+        <v>86751.51478474596</v>
       </c>
       <c r="F447" s="2" t="n">
-        <v>237747.5321060114</v>
+        <v>168112.8921625271</v>
       </c>
     </row>
     <row r="448">
@@ -9045,10 +9045,10 @@
         </is>
       </c>
       <c r="E448" s="2" t="n">
-        <v>167287.9720057605</v>
+        <v>128996.6606939122</v>
       </c>
       <c r="F448" s="2" t="n">
-        <v>298529.0180387111</v>
+        <v>177506.4161432054</v>
       </c>
     </row>
     <row r="449">
@@ -9071,10 +9071,10 @@
         </is>
       </c>
       <c r="E449" s="2" t="n">
-        <v>292546.3669700471</v>
+        <v>206861.5198960085</v>
       </c>
       <c r="F449" s="2" t="n">
-        <v>405332.5758647961</v>
+        <v>202666.2879323981</v>
       </c>
     </row>
     <row r="450">
@@ -9097,10 +9097,10 @@
         </is>
       </c>
       <c r="E450" s="2" t="n">
-        <v>535767.7056266126</v>
+        <v>347402.3763806049</v>
       </c>
       <c r="F450" s="2" t="n">
-        <v>577075.6050010385</v>
+        <v>242630.4037878709</v>
       </c>
     </row>
     <row r="451">
@@ -9123,10 +9123,10 @@
         </is>
       </c>
       <c r="E451" s="2" t="n">
-        <v>1012274.320400161</v>
+        <v>601901.9120772079</v>
       </c>
       <c r="F451" s="2" t="n">
-        <v>848190.8672212551</v>
+        <v>299880.756976324</v>
       </c>
     </row>
     <row r="452">
@@ -9149,10 +9149,10 @@
         </is>
       </c>
       <c r="E452" s="2" t="n">
-        <v>1956055.740709604</v>
+        <v>1066546.955384046</v>
       </c>
       <c r="F452" s="2" t="n">
-        <v>1275552.780747687</v>
+        <v>379224.110606664</v>
       </c>
     </row>
     <row r="453">
@@ -9175,10 +9175,10 @@
         </is>
       </c>
       <c r="E453" s="2" t="n">
-        <v>3844472.413788395</v>
+        <v>1922236.206894198</v>
       </c>
       <c r="F453" s="2" t="n">
-        <v>1951620.129116483</v>
+        <v>487905.0322791208</v>
       </c>
     </row>
     <row r="454">
@@ -9201,10 +9201,10 @@
         </is>
       </c>
       <c r="E454" s="2" t="n">
-        <v>3844472.413788395</v>
+        <v>1922236.206894198</v>
       </c>
       <c r="F454" s="2" t="n">
-        <v>1951620.129116483</v>
+        <v>487905.0322791208</v>
       </c>
     </row>
     <row r="455">
@@ -9227,10 +9227,10 @@
         </is>
       </c>
       <c r="E455" s="2" t="n">
-        <v>1946693.372001105</v>
+        <v>1061442.087647705</v>
       </c>
       <c r="F455" s="2" t="n">
-        <v>980782.4080206057</v>
+        <v>291588.3544719016</v>
       </c>
     </row>
     <row r="456">
@@ -9253,10 +9253,10 @@
         </is>
       </c>
       <c r="E456" s="2" t="n">
-        <v>1500139.55499045</v>
+        <v>891988.3161458297</v>
       </c>
       <c r="F456" s="2" t="n">
-        <v>780962.7294542136</v>
+        <v>276112.0209255147</v>
       </c>
     </row>
     <row r="457">
@@ -9279,10 +9279,10 @@
         </is>
       </c>
       <c r="E457" s="2" t="n">
-        <v>1338599.563961555</v>
+        <v>867974.4311919694</v>
       </c>
       <c r="F457" s="2" t="n">
-        <v>725426.3049462072</v>
+        <v>305004.1896800068</v>
       </c>
     </row>
     <row r="458">
@@ -9305,10 +9305,10 @@
         </is>
       </c>
       <c r="E458" s="2" t="n">
-        <v>1288159.195625633</v>
+        <v>910866.1024746936</v>
       </c>
       <c r="F458" s="2" t="n">
-        <v>728636.1470072566</v>
+        <v>364318.0735036284</v>
       </c>
     </row>
     <row r="459">
@@ -9331,10 +9331,10 @@
         </is>
       </c>
       <c r="E459" s="2" t="n">
-        <v>1298195.882280606</v>
+        <v>1001045.871576582</v>
       </c>
       <c r="F459" s="2" t="n">
-        <v>767404.5607332553</v>
+        <v>456301.4818547625</v>
       </c>
     </row>
     <row r="460">
@@ -9357,10 +9357,10 @@
         </is>
       </c>
       <c r="E460" s="2" t="n">
-        <v>1349742.058625097</v>
+        <v>1134993.258615013</v>
       </c>
       <c r="F460" s="2" t="n">
-        <v>834406.5582056041</v>
+        <v>590014.5355737103</v>
       </c>
     </row>
     <row r="461">
@@ -9383,10 +9383,10 @@
         </is>
       </c>
       <c r="E461" s="2" t="n">
-        <v>1435233.800987535</v>
+        <v>1316115.198449578</v>
       </c>
       <c r="F461" s="2" t="n">
-        <v>928271.479718659</v>
+        <v>780580.1596776814</v>
       </c>
     </row>
     <row r="462">

</xml_diff>

<commit_message>
balance: connect late fleet budgets and release accumulated growth
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/monGroup.xlsx
+++ b/space-battleship/config_excel/monGroup.xlsx
@@ -9461,10 +9461,10 @@
         </is>
       </c>
       <c r="E464" s="2" t="n">
-        <v>1002979.872671865</v>
+        <v>843402.179501398</v>
       </c>
       <c r="F464" s="2" t="n">
-        <v>635317.8739514224</v>
+        <v>346409.5271222388</v>
       </c>
     </row>
     <row r="465">
@@ -9487,10 +9487,10 @@
         </is>
       </c>
       <c r="E465" s="2" t="n">
-        <v>986258.3755649199</v>
+        <v>697389.9853639835</v>
       </c>
       <c r="F465" s="2" t="n">
-        <v>608692.6967440498</v>
+        <v>180965.4214545544</v>
       </c>
     </row>
     <row r="466">
@@ -9513,10 +9513,10 @@
         </is>
       </c>
       <c r="E466" s="2" t="n">
-        <v>1122985.361989187</v>
+        <v>667731.0912607233</v>
       </c>
       <c r="F466" s="2" t="n">
-        <v>680315.6457148808</v>
+        <v>110282.529876375</v>
       </c>
     </row>
     <row r="467">
@@ -9539,10 +9539,10 @@
         </is>
       </c>
       <c r="E467" s="2" t="n">
-        <v>1378977.971020714</v>
+        <v>689488.9855103572</v>
       </c>
       <c r="F467" s="2" t="n">
-        <v>822199.5751278132</v>
+        <v>72672.86188269686</v>
       </c>
     </row>
     <row r="468">
@@ -9565,10 +9565,10 @@
         </is>
       </c>
       <c r="E468" s="2" t="n">
-        <v>1773341.558002662</v>
+        <v>745598.2795724379</v>
       </c>
       <c r="F468" s="2" t="n">
-        <v>1041934.186915058</v>
+        <v>50215.06820071946</v>
       </c>
     </row>
     <row r="469">
@@ -9591,10 +9591,10 @@
         </is>
       </c>
       <c r="E469" s="2" t="n">
-        <v>2352704.156196336</v>
+        <v>831806.5314861018</v>
       </c>
       <c r="F469" s="2" t="n">
-        <v>1363147.957755349</v>
+        <v>35820.81972302797</v>
       </c>
     </row>
     <row r="470">
@@ -9617,10 +9617,10 @@
         </is>
       </c>
       <c r="E470" s="2" t="n">
-        <v>3192299.036364111</v>
+        <v>949076.1818151328</v>
       </c>
       <c r="F470" s="2" t="n">
-        <v>1824692.437613503</v>
+        <v>26144.5366077589</v>
       </c>
     </row>
     <row r="471">
@@ -9643,10 +9643,10 @@
         </is>
       </c>
       <c r="E471" s="2" t="n">
-        <v>4405673.7102302</v>
+        <v>1101418.42755755</v>
       </c>
       <c r="F471" s="2" t="n">
-        <v>2485011.254764018</v>
+        <v>19414.15042784389</v>
       </c>
     </row>
     <row r="472">
@@ -9669,10 +9669,10 @@
         </is>
       </c>
       <c r="E472" s="2" t="n">
-        <v>4405673.7102302</v>
+        <v>1101418.42755755</v>
       </c>
       <c r="F472" s="2" t="n">
-        <v>2485011.254764018</v>
+        <v>19414.15042784389</v>
       </c>
     </row>
     <row r="473">
@@ -9695,10 +9695,10 @@
         </is>
       </c>
       <c r="E473" s="2" t="n">
-        <v>1306555.198373588</v>
+        <v>326638.799593397</v>
       </c>
       <c r="F473" s="2" t="n">
-        <v>547448.8463459016</v>
+        <v>4276.944112077356</v>
       </c>
     </row>
     <row r="474">
@@ -9721,10 +9721,10 @@
         </is>
       </c>
       <c r="E474" s="2" t="n">
-        <v>1170016.518201419</v>
+        <v>292504.1295503547</v>
       </c>
       <c r="F474" s="2" t="n">
-        <v>388142.3771038132</v>
+        <v>3032.362321123541</v>
       </c>
     </row>
     <row r="475">
@@ -9747,10 +9747,10 @@
         </is>
       </c>
       <c r="E475" s="2" t="n">
-        <v>1313626.540762039</v>
+        <v>328406.6351905098</v>
       </c>
       <c r="F475" s="2" t="n">
-        <v>346491.9239291833</v>
+        <v>2706.968155696744</v>
       </c>
     </row>
     <row r="476">
@@ -9773,10 +9773,10 @@
         </is>
       </c>
       <c r="E476" s="2" t="n">
-        <v>1631994.594143361</v>
+        <v>407998.6485358402</v>
       </c>
       <c r="F476" s="2" t="n">
-        <v>342682.2961700279</v>
+        <v>2677.205438828343</v>
       </c>
     </row>
     <row r="477">
@@ -9799,10 +9799,10 @@
         </is>
       </c>
       <c r="E477" s="2" t="n">
-        <v>2147980.075219289</v>
+        <v>536995.0188048223</v>
       </c>
       <c r="F477" s="2" t="n">
-        <v>359235.9704904885</v>
+        <v>2806.531019456942</v>
       </c>
     </row>
     <row r="478">
@@ -9825,10 +9825,10 @@
         </is>
       </c>
       <c r="E478" s="2" t="n">
-        <v>2934691.486805297</v>
+        <v>733672.871701324</v>
       </c>
       <c r="F478" s="2" t="n">
-        <v>391025.3675603415</v>
+        <v>3054.885684065168</v>
       </c>
     </row>
     <row r="479">
@@ -9851,10 +9851,10 @@
         </is>
       </c>
       <c r="E479" s="2" t="n">
-        <v>4115830.633527148</v>
+        <v>1028957.658381787</v>
       </c>
       <c r="F479" s="2" t="n">
-        <v>436979.2555378187</v>
+        <v>3413.900433889209</v>
       </c>
     </row>
     <row r="480">
@@ -9877,10 +9877,10 @@
         </is>
       </c>
       <c r="E480" s="2" t="n">
-        <v>5885159.45667526</v>
+        <v>1471289.864168815</v>
       </c>
       <c r="F480" s="2" t="n">
-        <v>497926.8250832889</v>
+        <v>3890.053320963194</v>
       </c>
     </row>
     <row r="481">

</xml_diff>

<commit_message>
balance: shorten shield fleet endurance and connect the twentieth boss
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/monGroup.xlsx
+++ b/space-battleship/config_excel/monGroup.xlsx
@@ -8996,7 +8996,7 @@
         <v>67555.47782682885</v>
       </c>
       <c r="F446" s="2" t="n">
-        <v>185734.8222251147</v>
+        <v>156183.7461968849</v>
       </c>
     </row>
     <row r="447">
@@ -9022,7 +9022,7 @@
         <v>86751.51478474596</v>
       </c>
       <c r="F447" s="2" t="n">
-        <v>168112.8921625271</v>
+        <v>118873.7660530057</v>
       </c>
     </row>
     <row r="448">
@@ -9048,7 +9048,7 @@
         <v>128996.6606939122</v>
       </c>
       <c r="F448" s="2" t="n">
-        <v>177506.4161432054</v>
+        <v>105545.9465180669</v>
       </c>
     </row>
     <row r="449">
@@ -9074,7 +9074,7 @@
         <v>206861.5198960085</v>
       </c>
       <c r="F449" s="2" t="n">
-        <v>202666.2879323981</v>
+        <v>101333.143966199</v>
       </c>
     </row>
     <row r="450">
@@ -9100,7 +9100,7 @@
         <v>347402.3763806049</v>
       </c>
       <c r="F450" s="2" t="n">
-        <v>242630.4037878709</v>
+        <v>102013.518388391</v>
       </c>
     </row>
     <row r="451">
@@ -9126,7 +9126,7 @@
         <v>601901.9120772079</v>
       </c>
       <c r="F451" s="2" t="n">
-        <v>299880.756976324</v>
+        <v>106023.8584026569</v>
       </c>
     </row>
     <row r="452">
@@ -9152,7 +9152,7 @@
         <v>1066546.955384046</v>
       </c>
       <c r="F452" s="2" t="n">
-        <v>379224.110606664</v>
+        <v>112744.0026285059</v>
       </c>
     </row>
     <row r="453">
@@ -9178,7 +9178,7 @@
         <v>1922236.206894198</v>
       </c>
       <c r="F453" s="2" t="n">
-        <v>487905.0322791208</v>
+        <v>121976.2580697802</v>
       </c>
     </row>
     <row r="454">
@@ -9204,7 +9204,7 @@
         <v>1922236.206894198</v>
       </c>
       <c r="F454" s="2" t="n">
-        <v>487905.0322791208</v>
+        <v>121976.2580697802</v>
       </c>
     </row>
     <row r="455">
@@ -9230,7 +9230,7 @@
         <v>1061442.087647705</v>
       </c>
       <c r="F455" s="2" t="n">
-        <v>291588.3544719016</v>
+        <v>72897.0886179754</v>
       </c>
     </row>
     <row r="456">
@@ -9256,7 +9256,7 @@
         <v>891988.3161458297</v>
       </c>
       <c r="F456" s="2" t="n">
-        <v>276112.0209255147</v>
+        <v>69028.0052313787</v>
       </c>
     </row>
     <row r="457">
@@ -9282,7 +9282,7 @@
         <v>867974.4311919694</v>
       </c>
       <c r="F457" s="2" t="n">
-        <v>305004.1896800068</v>
+        <v>76251.04742000171</v>
       </c>
     </row>
     <row r="458">
@@ -9308,7 +9308,7 @@
         <v>910866.1024746936</v>
       </c>
       <c r="F458" s="2" t="n">
-        <v>364318.0735036284</v>
+        <v>91079.51837590709</v>
       </c>
     </row>
     <row r="459">
@@ -9334,7 +9334,7 @@
         <v>1001045.871576582</v>
       </c>
       <c r="F459" s="2" t="n">
-        <v>456301.4818547625</v>
+        <v>114075.3704636906</v>
       </c>
     </row>
     <row r="460">
@@ -9360,7 +9360,7 @@
         <v>1134993.258615013</v>
       </c>
       <c r="F460" s="2" t="n">
-        <v>590014.5355737103</v>
+        <v>147503.6338934276</v>
       </c>
     </row>
     <row r="461">
@@ -9386,7 +9386,7 @@
         <v>1316115.198449578</v>
       </c>
       <c r="F461" s="2" t="n">
-        <v>780580.1596776814</v>
+        <v>195145.0399194203</v>
       </c>
     </row>
     <row r="462">
@@ -9412,7 +9412,7 @@
         <v>1552269.2073895</v>
       </c>
       <c r="F462" s="2" t="n">
-        <v>1050665.129874534</v>
+        <v>262666.2824686335</v>
       </c>
     </row>
     <row r="463">
@@ -9438,7 +9438,7 @@
         <v>1552269.2073895</v>
       </c>
       <c r="F463" s="2" t="n">
-        <v>1050665.129874534</v>
+        <v>262666.2824686335</v>
       </c>
     </row>
     <row r="464">
@@ -9464,7 +9464,7 @@
         <v>843402.179501398</v>
       </c>
       <c r="F464" s="2" t="n">
-        <v>346409.5271222388</v>
+        <v>102988.1685896236</v>
       </c>
     </row>
     <row r="465">
@@ -9490,7 +9490,7 @@
         <v>697389.9853639835</v>
       </c>
       <c r="F465" s="2" t="n">
-        <v>180965.4214545544</v>
+        <v>63980.93833539847</v>
       </c>
     </row>
     <row r="466">
@@ -9516,7 +9516,7 @@
         <v>667731.0912607233</v>
       </c>
       <c r="F466" s="2" t="n">
-        <v>110282.529876375</v>
+        <v>46368.0920190772</v>
       </c>
     </row>
     <row r="467">
@@ -9542,7 +9542,7 @@
         <v>689488.9855103572</v>
       </c>
       <c r="F467" s="2" t="n">
-        <v>72672.86188269686</v>
+        <v>36336.43094134843</v>
       </c>
     </row>
     <row r="468">
@@ -9568,7 +9568,7 @@
         <v>745598.2795724379</v>
       </c>
       <c r="F468" s="2" t="n">
-        <v>50215.06820071946</v>
+        <v>29858.05819232124</v>
       </c>
     </row>
     <row r="469">
@@ -9594,7 +9594,7 @@
         <v>831806.5314861018</v>
       </c>
       <c r="F469" s="2" t="n">
-        <v>35820.81972302797</v>
+        <v>25329.1445338139</v>
       </c>
     </row>
     <row r="470">
@@ -9620,7 +9620,7 @@
         <v>949076.1818151328</v>
       </c>
       <c r="F470" s="2" t="n">
-        <v>26144.5366077589</v>
+        <v>21984.84711193397</v>
       </c>
     </row>
     <row r="471">

</xml_diff>

<commit_message>
Balance stages 4-7 for AI progression and first evolution material
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/monGroup.xlsx
+++ b/space-battleship/config_excel/monGroup.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="17700" windowHeight="13908" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="monGroup" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="monGroup" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -45602,700 +45602,700 @@
       </c>
     </row>
     <row r="2299">
-      <c r="A2299" t="n">
+      <c r="A2299" s="2" t="n">
         <v>90401</v>
       </c>
-      <c r="B2299" t="inlineStr">
-        <is>
-          <t>第4关第1点重堡</t>
-        </is>
-      </c>
-      <c r="C2299" t="inlineStr">
+      <c r="B2299" s="2" t="inlineStr">
+        <is>
+          <t>磁轨壁垒</t>
+        </is>
+      </c>
+      <c r="C2299" s="2" t="inlineStr">
         <is>
           <t>{null,null,null,null,null,null,null,400001,null,null,null,null,null,null,null}</t>
         </is>
       </c>
-      <c r="D2299" t="inlineStr">
+      <c r="D2299" s="2" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
     </row>
     <row r="2300">
-      <c r="A2300" t="n">
+      <c r="A2300" s="2" t="n">
         <v>90402</v>
       </c>
-      <c r="B2300" t="inlineStr">
-        <is>
-          <t>第4关第2点哨卫</t>
-        </is>
-      </c>
-      <c r="C2300" t="inlineStr">
+      <c r="B2300" s="2" t="inlineStr">
+        <is>
+          <t>能量哨卫</t>
+        </is>
+      </c>
+      <c r="C2300" s="2" t="inlineStr">
         <is>
           <t>{null,null,null,null,null,null,400002,400002,400002,null,null,null,null,null,null}</t>
         </is>
       </c>
-      <c r="D2300" t="inlineStr">
+      <c r="D2300" s="2" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
     </row>
     <row r="2301">
-      <c r="A2301" t="n">
+      <c r="A2301" s="2" t="n">
         <v>90403</v>
       </c>
-      <c r="B2301" t="inlineStr">
-        <is>
-          <t>第4关第3点重堡</t>
-        </is>
-      </c>
-      <c r="C2301" t="inlineStr">
+      <c r="B2301" s="2" t="inlineStr">
+        <is>
+          <t>轨道重堡</t>
+        </is>
+      </c>
+      <c r="C2301" s="2" t="inlineStr">
         <is>
           <t>{null,null,null,null,null,null,null,400003,null,null,null,null,null,null,null}</t>
         </is>
       </c>
-      <c r="D2301" t="inlineStr">
+      <c r="D2301" s="2" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
     </row>
     <row r="2302">
-      <c r="A2302" t="n">
+      <c r="A2302" s="2" t="n">
         <v>90404</v>
       </c>
-      <c r="B2302" t="inlineStr">
-        <is>
-          <t>第4关第4点蜂群</t>
-        </is>
-      </c>
-      <c r="C2302" t="inlineStr">
+      <c r="B2302" s="2" t="inlineStr">
+        <is>
+          <t>蜂群巡防群</t>
+        </is>
+      </c>
+      <c r="C2302" s="2" t="inlineStr">
         <is>
           <t>{null,null,400004,400004,400004,400004,400004,400004,400004,400004,400004,400004,null,null,null}</t>
         </is>
       </c>
-      <c r="D2302" t="inlineStr">
+      <c r="D2302" s="2" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
     </row>
     <row r="2303">
-      <c r="A2303" t="n">
+      <c r="A2303" s="2" t="n">
         <v>90405</v>
       </c>
-      <c r="B2303" t="inlineStr">
-        <is>
-          <t>第4关第5点重堡</t>
-        </is>
-      </c>
-      <c r="C2303" t="inlineStr">
+      <c r="B2303" s="2" t="inlineStr">
+        <is>
+          <t>合金堡垒</t>
+        </is>
+      </c>
+      <c r="C2303" s="2" t="inlineStr">
         <is>
           <t>{null,null,null,null,null,null,null,400005,null,null,null,null,null,null,null}</t>
         </is>
       </c>
-      <c r="D2303" t="inlineStr">
+      <c r="D2303" s="2" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
     </row>
     <row r="2304">
-      <c r="A2304" t="n">
+      <c r="A2304" s="2" t="n">
         <v>90406</v>
       </c>
-      <c r="B2304" t="inlineStr">
-        <is>
-          <t>第4关第6点哨卫</t>
-        </is>
-      </c>
-      <c r="C2304" t="inlineStr">
+      <c r="B2304" s="2" t="inlineStr">
+        <is>
+          <t>脉冲哨卫</t>
+        </is>
+      </c>
+      <c r="C2304" s="2" t="inlineStr">
         <is>
           <t>{null,null,null,null,null,null,400006,400006,400006,null,null,null,null,null,null}</t>
         </is>
       </c>
-      <c r="D2304" t="inlineStr">
+      <c r="D2304" s="2" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
     </row>
     <row r="2305">
-      <c r="A2305" t="n">
+      <c r="A2305" s="2" t="n">
         <v>90407</v>
       </c>
-      <c r="B2305" t="inlineStr">
-        <is>
-          <t>第4关第7点重堡</t>
-        </is>
-      </c>
-      <c r="C2305" t="inlineStr">
+      <c r="B2305" s="2" t="inlineStr">
+        <is>
+          <t>重炮壁垒</t>
+        </is>
+      </c>
+      <c r="C2305" s="2" t="inlineStr">
         <is>
           <t>{null,null,null,null,null,null,null,400007,null,null,null,null,null,null,null}</t>
         </is>
       </c>
-      <c r="D2305" t="inlineStr">
+      <c r="D2305" s="2" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
     </row>
     <row r="2306">
-      <c r="A2306" t="n">
+      <c r="A2306" s="2" t="n">
         <v>90408</v>
       </c>
-      <c r="B2306" t="inlineStr">
-        <is>
-          <t>第4关第8点重堡</t>
-        </is>
-      </c>
-      <c r="C2306" t="inlineStr">
+      <c r="B2306" s="2" t="inlineStr">
+        <is>
+          <t>关隘核心</t>
+        </is>
+      </c>
+      <c r="C2306" s="2" t="inlineStr">
         <is>
           <t>{null,null,null,null,null,null,null,400008,null,null,null,null,null,null,null}</t>
         </is>
       </c>
-      <c r="D2306" t="inlineStr">
+      <c r="D2306" s="2" t="inlineStr">
         <is>
           <t>elite</t>
         </is>
       </c>
     </row>
     <row r="2307">
-      <c r="A2307" t="n">
+      <c r="A2307" s="2" t="n">
         <v>90501</v>
       </c>
-      <c r="B2307" t="inlineStr">
-        <is>
-          <t>第5关第1点哨卫</t>
-        </is>
-      </c>
-      <c r="C2307" t="inlineStr">
+      <c r="B2307" s="2" t="inlineStr">
+        <is>
+          <t>哨卫巡逻队</t>
+        </is>
+      </c>
+      <c r="C2307" s="2" t="inlineStr">
         <is>
           <t>{null,null,null,null,null,null,500001,500001,500001,null,null,null,null,null,null}</t>
         </is>
       </c>
-      <c r="D2307" t="inlineStr">
+      <c r="D2307" s="2" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
     </row>
     <row r="2308">
-      <c r="A2308" t="n">
+      <c r="A2308" s="2" t="n">
         <v>90502</v>
       </c>
-      <c r="B2308" t="inlineStr">
-        <is>
-          <t>第5关第2点哨卫</t>
-        </is>
-      </c>
-      <c r="C2308" t="inlineStr">
+      <c r="B2308" s="2" t="inlineStr">
+        <is>
+          <t>哨卫阻截队</t>
+        </is>
+      </c>
+      <c r="C2308" s="2" t="inlineStr">
         <is>
           <t>{null,null,null,null,null,null,500002,500002,500002,null,null,null,null,null,null}</t>
         </is>
       </c>
-      <c r="D2308" t="inlineStr">
+      <c r="D2308" s="2" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
     </row>
     <row r="2309">
-      <c r="A2309" t="n">
+      <c r="A2309" s="2" t="n">
         <v>90503</v>
       </c>
-      <c r="B2309" t="inlineStr">
-        <is>
-          <t>第5关第3点蜂群</t>
-        </is>
-      </c>
-      <c r="C2309" t="inlineStr">
+      <c r="B2309" s="2" t="inlineStr">
+        <is>
+          <t>蜂群散阵</t>
+        </is>
+      </c>
+      <c r="C2309" s="2" t="inlineStr">
         <is>
           <t>{null,null,500003,500003,500003,500003,500003,500003,500003,500003,500003,500003,null,null,null}</t>
         </is>
       </c>
-      <c r="D2309" t="inlineStr">
+      <c r="D2309" s="2" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
     </row>
     <row r="2310">
-      <c r="A2310" t="n">
+      <c r="A2310" s="2" t="n">
         <v>90504</v>
       </c>
-      <c r="B2310" t="inlineStr">
-        <is>
-          <t>第5关第4点蜂群</t>
-        </is>
-      </c>
-      <c r="C2310" t="inlineStr">
+      <c r="B2310" s="2" t="inlineStr">
+        <is>
+          <t>蜂群密阵</t>
+        </is>
+      </c>
+      <c r="C2310" s="2" t="inlineStr">
         <is>
           <t>{null,null,500004,500004,500004,500004,500004,500004,500004,500004,500004,500004,null,null,null}</t>
         </is>
       </c>
-      <c r="D2310" t="inlineStr">
+      <c r="D2310" s="2" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
     </row>
     <row r="2311">
-      <c r="A2311" t="n">
+      <c r="A2311" s="2" t="n">
         <v>90505</v>
       </c>
-      <c r="B2311" t="inlineStr">
-        <is>
-          <t>第5关第5点重堡</t>
-        </is>
-      </c>
-      <c r="C2311" t="inlineStr">
+      <c r="B2311" s="2" t="inlineStr">
+        <is>
+          <t>重甲堡垒</t>
+        </is>
+      </c>
+      <c r="C2311" s="2" t="inlineStr">
         <is>
           <t>{null,null,null,null,null,null,null,500005,null,null,null,null,null,null,null}</t>
         </is>
       </c>
-      <c r="D2311" t="inlineStr">
+      <c r="D2311" s="2" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
     </row>
     <row r="2312">
-      <c r="A2312" t="n">
+      <c r="A2312" s="2" t="n">
         <v>90506</v>
       </c>
-      <c r="B2312" t="inlineStr">
-        <is>
-          <t>第5关第6点重堡</t>
-        </is>
-      </c>
-      <c r="C2312" t="inlineStr">
+      <c r="B2312" s="2" t="inlineStr">
+        <is>
+          <t>重炮堡垒</t>
+        </is>
+      </c>
+      <c r="C2312" s="2" t="inlineStr">
         <is>
           <t>{null,null,null,null,null,null,null,500006,null,null,null,null,null,null,null}</t>
         </is>
       </c>
-      <c r="D2312" t="inlineStr">
+      <c r="D2312" s="2" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
     </row>
     <row r="2313">
-      <c r="A2313" t="n">
+      <c r="A2313" s="2" t="n">
         <v>90507</v>
       </c>
-      <c r="B2313" t="inlineStr">
-        <is>
-          <t>第5关第7点哨卫</t>
-        </is>
-      </c>
-      <c r="C2313" t="inlineStr">
+      <c r="B2313" s="2" t="inlineStr">
+        <is>
+          <t>能量哨卫群</t>
+        </is>
+      </c>
+      <c r="C2313" s="2" t="inlineStr">
         <is>
           <t>{null,null,null,null,null,null,500007,500007,500007,null,null,null,null,null,null}</t>
         </is>
       </c>
-      <c r="D2313" t="inlineStr">
+      <c r="D2313" s="2" t="inlineStr">
         <is>
           <t>elite</t>
         </is>
       </c>
     </row>
     <row r="2314">
-      <c r="A2314" t="n">
+      <c r="A2314" s="2" t="n">
         <v>90508</v>
       </c>
-      <c r="B2314" t="inlineStr">
-        <is>
-          <t>第5关第8点蜂群</t>
-        </is>
-      </c>
-      <c r="C2314" t="inlineStr">
+      <c r="B2314" s="2" t="inlineStr">
+        <is>
+          <t>蜂群终阵</t>
+        </is>
+      </c>
+      <c r="C2314" s="2" t="inlineStr">
         <is>
           <t>{null,null,500008,500008,500008,500008,500008,500008,500008,500008,500008,500008,null,null,null}</t>
         </is>
       </c>
-      <c r="D2314" t="inlineStr">
+      <c r="D2314" s="2" t="inlineStr">
         <is>
           <t>elite</t>
         </is>
       </c>
     </row>
     <row r="2315">
-      <c r="A2315" t="n">
+      <c r="A2315" s="2" t="n">
         <v>90509</v>
       </c>
-      <c r="B2315" t="inlineStr">
-        <is>
-          <t>第5关第9点重堡</t>
-        </is>
-      </c>
-      <c r="C2315" t="inlineStr">
+      <c r="B2315" s="2" t="inlineStr">
+        <is>
+          <t>深空重堡</t>
+        </is>
+      </c>
+      <c r="C2315" s="2" t="inlineStr">
         <is>
           <t>{null,null,null,null,null,null,null,500009,null,null,null,null,null,null,null}</t>
         </is>
       </c>
-      <c r="D2315" t="inlineStr">
+      <c r="D2315" s="2" t="inlineStr">
         <is>
           <t>elite</t>
         </is>
       </c>
     </row>
     <row r="2316">
-      <c r="A2316" t="n">
+      <c r="A2316" s="2" t="n">
         <v>90601</v>
       </c>
-      <c r="B2316" t="inlineStr">
-        <is>
-          <t>第6关第1点光束靶舰</t>
-        </is>
-      </c>
-      <c r="C2316" t="inlineStr">
+      <c r="B2316" s="2" t="inlineStr">
+        <is>
+          <t>锁定侦察艇</t>
+        </is>
+      </c>
+      <c r="C2316" s="2" t="inlineStr">
         <is>
           <t>{null,null,null,null,null,null,null,600001,null,null,null,null,null,null,null}</t>
         </is>
       </c>
-      <c r="D2316" t="inlineStr">
+      <c r="D2316" s="2" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
     </row>
     <row r="2317">
-      <c r="A2317" t="n">
+      <c r="A2317" s="2" t="n">
         <v>90602</v>
       </c>
-      <c r="B2317" t="inlineStr">
-        <is>
-          <t>第6关第2点光束靶舰</t>
-        </is>
-      </c>
-      <c r="C2317" t="inlineStr">
+      <c r="B2317" s="2" t="inlineStr">
+        <is>
+          <t>重脉冲哨卫</t>
+        </is>
+      </c>
+      <c r="C2317" s="2" t="inlineStr">
         <is>
           <t>{null,null,null,null,null,null,null,600002,null,null,null,null,null,null,null}</t>
         </is>
       </c>
-      <c r="D2317" t="inlineStr">
+      <c r="D2317" s="2" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
     </row>
     <row r="2318">
-      <c r="A2318" t="n">
+      <c r="A2318" s="2" t="n">
         <v>90603</v>
       </c>
-      <c r="B2318" t="inlineStr">
-        <is>
-          <t>第6关第3点光束靶舰</t>
-        </is>
-      </c>
-      <c r="C2318" t="inlineStr">
-        <is>
-          <t>{null,null,null,null,null,null,null,600003,null,null,null,null,null,null,null}</t>
-        </is>
-      </c>
-      <c r="D2318" t="inlineStr">
+      <c r="B2318" s="2" t="inlineStr">
+        <is>
+          <t>双机警戒线</t>
+        </is>
+      </c>
+      <c r="C2318" s="2" t="inlineStr">
+        <is>
+          <t>{null,null,null,null,null,960003,null,600003,null,null,null,null,null,null,null}</t>
+        </is>
+      </c>
+      <c r="D2318" s="2" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
     </row>
     <row r="2319">
-      <c r="A2319" t="n">
+      <c r="A2319" s="2" t="n">
         <v>90604</v>
       </c>
-      <c r="B2319" t="inlineStr">
-        <is>
-          <t>第6关第4点光束靶舰</t>
-        </is>
-      </c>
-      <c r="C2319" t="inlineStr">
+      <c r="B2319" s="2" t="inlineStr">
+        <is>
+          <t>回充护卫舰</t>
+        </is>
+      </c>
+      <c r="C2319" s="2" t="inlineStr">
         <is>
           <t>{null,null,null,null,null,null,null,600004,null,null,null,null,null,null,null}</t>
         </is>
       </c>
-      <c r="D2319" t="inlineStr">
+      <c r="D2319" s="2" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
     </row>
     <row r="2320">
-      <c r="A2320" t="n">
+      <c r="A2320" s="2" t="n">
         <v>90605</v>
       </c>
-      <c r="B2320" t="inlineStr">
-        <is>
-          <t>第6关第5点光束靶舰</t>
-        </is>
-      </c>
-      <c r="C2320" t="inlineStr">
+      <c r="B2320" s="2" t="inlineStr">
+        <is>
+          <t>重击炮艇</t>
+        </is>
+      </c>
+      <c r="C2320" s="2" t="inlineStr">
         <is>
           <t>{null,null,null,null,null,null,null,600005,null,null,null,null,null,null,null}</t>
         </is>
       </c>
-      <c r="D2320" t="inlineStr">
+      <c r="D2320" s="2" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
     </row>
     <row r="2321">
-      <c r="A2321" t="n">
+      <c r="A2321" s="2" t="n">
         <v>90606</v>
       </c>
-      <c r="B2321" t="inlineStr">
-        <is>
-          <t>第6关第6点光束靶舰</t>
-        </is>
-      </c>
-      <c r="C2321" t="inlineStr">
-        <is>
-          <t>{null,null,null,null,null,null,null,600006,null,null,null,null,null,null,null}</t>
-        </is>
-      </c>
-      <c r="D2321" t="inlineStr">
+      <c r="B2321" s="2" t="inlineStr">
+        <is>
+          <t>双翼巡防阵</t>
+        </is>
+      </c>
+      <c r="C2321" s="2" t="inlineStr">
+        <is>
+          <t>{null,null,null,null,null,null,null,600006,null,960006,null,null,null,null,null}</t>
+        </is>
+      </c>
+      <c r="D2321" s="2" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
     </row>
     <row r="2322">
-      <c r="A2322" t="n">
+      <c r="A2322" s="2" t="n">
         <v>90607</v>
       </c>
-      <c r="B2322" t="inlineStr">
-        <is>
-          <t>第6关第7点光束靶舰</t>
-        </is>
-      </c>
-      <c r="C2322" t="inlineStr">
+      <c r="B2322" s="2" t="inlineStr">
+        <is>
+          <t>再生护卫舰</t>
+        </is>
+      </c>
+      <c r="C2322" s="2" t="inlineStr">
         <is>
           <t>{null,null,null,null,null,null,null,600007,null,null,null,null,null,null,null}</t>
         </is>
       </c>
-      <c r="D2322" t="inlineStr">
+      <c r="D2322" s="2" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
     </row>
     <row r="2323">
-      <c r="A2323" t="n">
+      <c r="A2323" s="2" t="n">
         <v>90608</v>
       </c>
-      <c r="B2323" t="inlineStr">
-        <is>
-          <t>第6关第8点光束靶舰</t>
-        </is>
-      </c>
-      <c r="C2323" t="inlineStr">
+      <c r="B2323" s="2" t="inlineStr">
+        <is>
+          <t>远程炮台</t>
+        </is>
+      </c>
+      <c r="C2323" s="2" t="inlineStr">
         <is>
           <t>{null,null,null,null,null,null,null,600008,null,null,null,null,null,null,null}</t>
         </is>
       </c>
-      <c r="D2323" t="inlineStr">
+      <c r="D2323" s="2" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
     </row>
     <row r="2324">
-      <c r="A2324" t="n">
+      <c r="A2324" s="2" t="n">
         <v>90609</v>
       </c>
-      <c r="B2324" t="inlineStr">
-        <is>
-          <t>第6关第9点光束靶舰</t>
-        </is>
-      </c>
-      <c r="C2324" t="inlineStr">
+      <c r="B2324" s="2" t="inlineStr">
+        <is>
+          <t>束流壁垒</t>
+        </is>
+      </c>
+      <c r="C2324" s="2" t="inlineStr">
         <is>
           <t>{null,null,null,null,null,null,null,600009,null,null,null,null,null,null,null}</t>
         </is>
       </c>
-      <c r="D2324" t="inlineStr">
+      <c r="D2324" s="2" t="inlineStr">
         <is>
           <t>boss</t>
         </is>
       </c>
     </row>
     <row r="2325">
-      <c r="A2325" t="n">
+      <c r="A2325" s="2" t="n">
         <v>90701</v>
       </c>
-      <c r="B2325" t="inlineStr">
-        <is>
-          <t>第7关第1点光束靶舰</t>
-        </is>
-      </c>
-      <c r="C2325" t="inlineStr">
+      <c r="B2325" s="2" t="inlineStr">
+        <is>
+          <t>深空屏障舰</t>
+        </is>
+      </c>
+      <c r="C2325" s="2" t="inlineStr">
         <is>
           <t>{null,null,null,null,null,null,null,700001,null,null,null,null,null,null,null}</t>
         </is>
       </c>
-      <c r="D2325" t="inlineStr">
+      <c r="D2325" s="2" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
     </row>
     <row r="2326">
-      <c r="A2326" t="n">
+      <c r="A2326" s="2" t="n">
         <v>90702</v>
       </c>
-      <c r="B2326" t="inlineStr">
-        <is>
-          <t>第7关第2点光束靶舰</t>
-        </is>
-      </c>
-      <c r="C2326" t="inlineStr">
+      <c r="B2326" s="2" t="inlineStr">
+        <is>
+          <t>重击哨卫</t>
+        </is>
+      </c>
+      <c r="C2326" s="2" t="inlineStr">
         <is>
           <t>{null,null,null,null,null,null,null,700002,null,null,null,null,null,null,null}</t>
         </is>
       </c>
-      <c r="D2326" t="inlineStr">
+      <c r="D2326" s="2" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
     </row>
     <row r="2327">
-      <c r="A2327" t="n">
+      <c r="A2327" s="2" t="n">
         <v>90703</v>
       </c>
-      <c r="B2327" t="inlineStr">
-        <is>
-          <t>第7关第3点光束靶舰</t>
-        </is>
-      </c>
-      <c r="C2327" t="inlineStr">
+      <c r="B2327" s="2" t="inlineStr">
+        <is>
+          <t>回充堡垒</t>
+        </is>
+      </c>
+      <c r="C2327" s="2" t="inlineStr">
         <is>
           <t>{null,null,null,null,null,null,null,700003,null,null,null,null,null,null,null}</t>
         </is>
       </c>
-      <c r="D2327" t="inlineStr">
+      <c r="D2327" s="2" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
     </row>
     <row r="2328">
-      <c r="A2328" t="n">
+      <c r="A2328" s="2" t="n">
         <v>90704</v>
       </c>
-      <c r="B2328" t="inlineStr">
-        <is>
-          <t>第7关第4点光束靶舰</t>
-        </is>
-      </c>
-      <c r="C2328" t="inlineStr">
-        <is>
-          <t>{null,null,null,null,null,null,null,700004,null,null,null,null,null,null,null}</t>
-        </is>
-      </c>
-      <c r="D2328" t="inlineStr">
+      <c r="B2328" s="2" t="inlineStr">
+        <is>
+          <t>双舰截击阵</t>
+        </is>
+      </c>
+      <c r="C2328" s="2" t="inlineStr">
+        <is>
+          <t>{null,null,null,null,null,970004,null,700004,null,null,null,null,null,null,null}</t>
+        </is>
+      </c>
+      <c r="D2328" s="2" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
     </row>
     <row r="2329">
-      <c r="A2329" t="n">
+      <c r="A2329" s="2" t="n">
         <v>90705</v>
       </c>
-      <c r="B2329" t="inlineStr">
-        <is>
-          <t>第7关第5点光束靶舰</t>
-        </is>
-      </c>
-      <c r="C2329" t="inlineStr">
+      <c r="B2329" s="2" t="inlineStr">
+        <is>
+          <t>长距炮艇</t>
+        </is>
+      </c>
+      <c r="C2329" s="2" t="inlineStr">
         <is>
           <t>{null,null,null,null,null,null,null,700005,null,null,null,null,null,null,null}</t>
         </is>
       </c>
-      <c r="D2329" t="inlineStr">
+      <c r="D2329" s="2" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
     </row>
     <row r="2330">
-      <c r="A2330" t="n">
+      <c r="A2330" s="2" t="n">
         <v>90706</v>
       </c>
-      <c r="B2330" t="inlineStr">
-        <is>
-          <t>第7关第6点光束靶舰</t>
-        </is>
-      </c>
-      <c r="C2330" t="inlineStr">
+      <c r="B2330" s="2" t="inlineStr">
+        <is>
+          <t>持续压制舰</t>
+        </is>
+      </c>
+      <c r="C2330" s="2" t="inlineStr">
         <is>
           <t>{null,null,null,null,null,null,null,700006,null,null,null,null,null,null,null}</t>
         </is>
       </c>
-      <c r="D2330" t="inlineStr">
+      <c r="D2330" s="2" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
     </row>
     <row r="2331">
-      <c r="A2331" t="n">
+      <c r="A2331" s="2" t="n">
         <v>90707</v>
       </c>
-      <c r="B2331" t="inlineStr">
-        <is>
-          <t>第7关第7点光束靶舰</t>
-        </is>
-      </c>
-      <c r="C2331" t="inlineStr">
-        <is>
-          <t>{null,null,null,null,null,null,null,700007,null,null,null,null,null,null,null}</t>
-        </is>
-      </c>
-      <c r="D2331" t="inlineStr">
+      <c r="B2331" s="2" t="inlineStr">
+        <is>
+          <t>双翼护航阵</t>
+        </is>
+      </c>
+      <c r="C2331" s="2" t="inlineStr">
+        <is>
+          <t>{null,null,null,null,null,null,null,700007,null,970007,null,null,null,null,null}</t>
+        </is>
+      </c>
+      <c r="D2331" s="2" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
     </row>
     <row r="2332">
-      <c r="A2332" t="n">
+      <c r="A2332" s="2" t="n">
         <v>90708</v>
       </c>
-      <c r="B2332" t="inlineStr">
-        <is>
-          <t>第7关第8点光束靶舰</t>
-        </is>
-      </c>
-      <c r="C2332" t="inlineStr">
+      <c r="B2332" s="2" t="inlineStr">
+        <is>
+          <t>高压突击舰</t>
+        </is>
+      </c>
+      <c r="C2332" s="2" t="inlineStr">
         <is>
           <t>{null,null,null,null,null,null,null,700008,null,null,null,null,null,null,null}</t>
         </is>
       </c>
-      <c r="D2332" t="inlineStr">
+      <c r="D2332" s="2" t="inlineStr">
         <is>
           <t>normal</t>
         </is>
       </c>
     </row>
     <row r="2333">
-      <c r="A2333" t="n">
+      <c r="A2333" s="2" t="n">
         <v>90709</v>
       </c>
-      <c r="B2333" t="inlineStr">
-        <is>
-          <t>第7关第9点光束靶舰</t>
-        </is>
-      </c>
-      <c r="C2333" t="inlineStr">
+      <c r="B2333" s="2" t="inlineStr">
+        <is>
+          <t>异空间门卫</t>
+        </is>
+      </c>
+      <c r="C2333" s="2" t="inlineStr">
         <is>
           <t>{null,null,null,null,null,null,null,700009,null,null,null,null,null,null,null}</t>
         </is>
       </c>
-      <c r="D2333" t="inlineStr">
+      <c r="D2333" s="2" t="inlineStr">
         <is>
           <t>boss</t>
         </is>

</xml_diff>

<commit_message>
Differentiate stages 3-7 encounter choices after three-way review
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/monGroup.xlsx
+++ b/space-battleship/config_excel/monGroup.xlsx
@@ -45672,7 +45672,7 @@
       </c>
       <c r="C2302" s="2" t="inlineStr">
         <is>
-          <t>{null,null,null,null,null,400004,400004,400004,null,null,null,null,null,null,null}</t>
+          <t>{null,null,null,400004,null,400004,null,400004,null,400004,null,400004,null,null,null}</t>
         </is>
       </c>
       <c r="D2302" s="2" t="inlineStr">
@@ -45712,7 +45712,7 @@
       </c>
       <c r="C2304" s="2" t="inlineStr">
         <is>
-          <t>{null,null,null,null,null,null,400006,400006,400006,null,null,null,null,null,null}</t>
+          <t>{null,null,null,null,null,400006,null,null,null,400006,null,null,null,null,null}</t>
         </is>
       </c>
       <c r="D2304" s="2" t="inlineStr">
@@ -45792,7 +45792,7 @@
       </c>
       <c r="C2308" s="2" t="inlineStr">
         <is>
-          <t>{null,null,null,null,null,null,500002,500002,500002,null,null,null,null,null,null}</t>
+          <t>{null,null,null,null,null,500002,null,null,null,500002,null,null,null,null,null}</t>
         </is>
       </c>
       <c r="D2308" s="2" t="inlineStr">
@@ -45832,7 +45832,7 @@
       </c>
       <c r="C2310" s="2" t="inlineStr">
         <is>
-          <t>{null,null,500004,500004,500004,500004,500004,500004,500004,500004,500004,500004,null,null,null}</t>
+          <t>{null,500004,null,500004,null,500004,500004,null,500004,500004,null,500004,null,500004,null}</t>
         </is>
       </c>
       <c r="D2310" s="2" t="inlineStr">
@@ -45872,7 +45872,7 @@
       </c>
       <c r="C2312" s="2" t="inlineStr">
         <is>
-          <t>{null,null,null,null,null,null,null,500006,null,null,null,null,null,null,null}</t>
+          <t>{null,null,null,null,null,500006,null,null,null,500006,null,null,null,null,null}</t>
         </is>
       </c>
       <c r="D2312" s="2" t="inlineStr">

</xml_diff>